<commit_message>
update c phi + checks
checks import, export, fout c-phi+ beschrijving analyse tools
</commit_message>
<xml_diff>
--- a/resultaten/c_phi_data_geforceerd.xlsx
+++ b/resultaten/c_phi_data_geforceerd.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="19">
   <si>
     <t>PV_NAAM</t>
   </si>
@@ -70,7 +70,7 @@
     <t>kappa_2_ondergrens_cor</t>
   </si>
   <si>
-    <t>TXT_SAFE_klei_licht_12_16</t>
+    <t>TXT_klei_14_16</t>
   </si>
 </sst>
 </file>
@@ -428,7 +428,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R29"/>
+  <dimension ref="A1:R74"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
@@ -492,55 +492,55 @@
         <v>18</v>
       </c>
       <c r="B2">
-        <v>156.55</v>
+        <v>143.8</v>
       </c>
       <c r="C2">
-        <v>98.11</v>
+        <v>85.09999999999999</v>
       </c>
       <c r="D2">
-        <v>3856.498741700467</v>
+        <v>1665.815084102405</v>
       </c>
       <c r="E2">
-        <v>6092.701099824045</v>
+        <v>3473.305269800001</v>
       </c>
       <c r="F2">
-        <v>1.270070326572332</v>
+        <v>22.00037539803776</v>
       </c>
       <c r="G2">
-        <v>14.609999656677</v>
+        <v>13.56</v>
       </c>
       <c r="H2">
-        <v>7.077704519453753</v>
+        <v>5.030972332908122</v>
       </c>
       <c r="I2">
-        <v>18.47677080057899</v>
+        <v>19.94635179074794</v>
       </c>
       <c r="J2">
-        <v>12013.25606262991</v>
+        <v>15348.73210000003</v>
       </c>
       <c r="K2">
-        <v>-775.7518050696976</v>
+        <v>-623.2871623239879</v>
       </c>
       <c r="L2">
-        <v>0.3943983516083208</v>
+        <v>0.1517378637092041</v>
       </c>
       <c r="M2">
-        <v>94.23</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="N2">
-        <v>1.269204331240707</v>
+        <v>21.72773083189701</v>
       </c>
       <c r="O2">
-        <v>7.07960274556101</v>
+        <v>5.995015971522179</v>
       </c>
       <c r="P2">
-        <v>18.47866927798847</v>
+        <v>20.94947294203445</v>
       </c>
       <c r="Q2">
-        <v>-775.9598601425095</v>
+        <v>-742.7225287118835</v>
       </c>
       <c r="R2">
-        <v>0.3920177395004212</v>
+        <v>0.3300596633529649</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -548,55 +548,55 @@
         <v>18</v>
       </c>
       <c r="B3">
-        <v>144.64</v>
+        <v>110.23</v>
       </c>
       <c r="C3">
-        <v>89.43000000000001</v>
+        <v>65.8</v>
       </c>
       <c r="D3">
-        <v>2519.107822254855</v>
+        <v>52.48130238240406</v>
       </c>
       <c r="E3">
-        <v>4488.555597943779</v>
+        <v>476.6813884000002</v>
       </c>
       <c r="F3">
-        <v>6.51398233522302</v>
+        <v>8.394908899002235</v>
       </c>
       <c r="G3">
-        <v>22.72888855828155</v>
+        <v>17.00138888888889</v>
       </c>
       <c r="H3">
-        <v>12.12353864733159</v>
+        <v>6.848966125776429</v>
       </c>
       <c r="I3">
-        <v>23.32183412029794</v>
+        <v>21.71776477294472</v>
       </c>
       <c r="J3">
-        <v>10299.43078071837</v>
+        <v>14507.86791859571</v>
       </c>
       <c r="K3">
-        <v>-1230.370792149929</v>
+        <v>-824.9484573968192</v>
       </c>
       <c r="L3">
-        <v>0.2396333019539502</v>
+        <v>0.127605456976626</v>
       </c>
       <c r="M3">
-        <v>85.55000000000001</v>
+        <v>59.3</v>
       </c>
       <c r="N3">
-        <v>6.512998501879683</v>
+        <v>6.876111340008016</v>
       </c>
       <c r="O3">
-        <v>12.12530631049206</v>
+        <v>7.787851511851661</v>
       </c>
       <c r="P3">
-        <v>23.32360203033446</v>
+        <v>22.6956056324091</v>
       </c>
       <c r="Q3">
-        <v>-1230.550185410121</v>
+        <v>-938.0358981421005</v>
       </c>
       <c r="R3">
-        <v>0.2379058011105912</v>
+        <v>0.3383357146466803</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -604,55 +604,55 @@
         <v>18</v>
       </c>
       <c r="B4">
-        <v>121.67</v>
+        <v>218.35</v>
       </c>
       <c r="C4">
-        <v>75.73999999999999</v>
+        <v>129.55</v>
       </c>
       <c r="D4">
-        <v>740.9672980176069</v>
+        <v>13308.9443259024</v>
       </c>
       <c r="E4">
-        <v>2061.696916406819</v>
+        <v>14945.4577609</v>
       </c>
       <c r="F4">
-        <v>5.06503311189327</v>
+        <v>105.3131061460526</v>
       </c>
       <c r="G4">
-        <v>30.84777745988611</v>
+        <v>20.44277777777778</v>
       </c>
       <c r="H4">
-        <v>17.16016353002255</v>
+        <v>8.66611497684951</v>
       </c>
       <c r="I4">
-        <v>28.17610668520377</v>
+        <v>23.49002269693672</v>
       </c>
       <c r="J4">
-        <v>8717.438212800031</v>
+        <v>13690.69005216052</v>
       </c>
       <c r="K4">
-        <v>-1602.196804186622</v>
+        <v>-1013.99804089956</v>
       </c>
       <c r="L4">
-        <v>0.1297763955962047</v>
+        <v>0.1061115094529364</v>
       </c>
       <c r="M4">
-        <v>71.86</v>
+        <v>123.05</v>
       </c>
       <c r="N4">
-        <v>5.065828266528083</v>
+        <v>116.1950809800736</v>
       </c>
       <c r="O4">
-        <v>17.16180063003321</v>
+        <v>9.579839896682689</v>
       </c>
       <c r="P4">
-        <v>28.17774402807036</v>
+        <v>24.44258547828221</v>
       </c>
       <c r="Q4">
-        <v>-1602.349655667356</v>
+        <v>-1120.910455644463</v>
       </c>
       <c r="R4">
-        <v>0.1285995617987638</v>
+        <v>0.3457173096004614</v>
       </c>
     </row>
     <row r="5" spans="1:18">
@@ -660,55 +660,55 @@
         <v>18</v>
       </c>
       <c r="B5">
-        <v>233.82</v>
+        <v>86.48</v>
       </c>
       <c r="C5">
-        <v>143.77</v>
+        <v>48.82</v>
       </c>
       <c r="D5">
-        <v>19424.19606089124</v>
+        <v>272.4348973824038</v>
       </c>
       <c r="E5">
-        <v>20037.32762400064</v>
+        <v>-805.8034896399998</v>
       </c>
       <c r="F5">
-        <v>6.422946155392101</v>
+        <v>2.879287678438584</v>
       </c>
       <c r="G5">
-        <v>38.96666636149067</v>
+        <v>23.88416666666667</v>
       </c>
       <c r="H5">
-        <v>22.18711494325641</v>
+        <v>10.48241118753726</v>
       </c>
       <c r="I5">
-        <v>33.0400527195667</v>
+        <v>25.26313326131406</v>
       </c>
       <c r="J5">
-        <v>7267.278358874882</v>
+        <v>12897.19850069448</v>
       </c>
       <c r="K5">
-        <v>-1891.414573350005</v>
+        <v>-1190.443761855326</v>
       </c>
       <c r="L5">
-        <v>0.05790748675202095</v>
+        <v>0.08710101599992996</v>
       </c>
       <c r="M5">
-        <v>139.89</v>
+        <v>42.32</v>
       </c>
       <c r="N5">
-        <v>6.414702485459595</v>
+        <v>4.605550424106501</v>
       </c>
       <c r="O5">
-        <v>22.18862147990399</v>
+        <v>11.37097340725525</v>
       </c>
       <c r="P5">
-        <v>33.04155949547662</v>
+        <v>26.19042019841378</v>
       </c>
       <c r="Q5">
-        <v>-1891.543003088517</v>
+        <v>-1291.354070806116</v>
       </c>
       <c r="R5">
-        <v>0.05718469121603996</v>
+        <v>0.3521632087374658</v>
       </c>
     </row>
     <row r="6" spans="1:18">
@@ -716,55 +716,55 @@
         <v>18</v>
       </c>
       <c r="B6">
-        <v>92.25</v>
+        <v>166.59</v>
       </c>
       <c r="C6">
-        <v>55.06</v>
+        <v>92.61</v>
       </c>
       <c r="D6">
-        <v>4.836856700241534</v>
+        <v>4045.519444942404</v>
       </c>
       <c r="E6">
-        <v>-121.0926595014593</v>
+        <v>5890.40329878</v>
       </c>
       <c r="F6">
-        <v>25.10004733263522</v>
+        <v>0.0994420970070284</v>
       </c>
       <c r="G6">
-        <v>47.08555526309522</v>
+        <v>27.32555555555555</v>
       </c>
       <c r="H6">
-        <v>27.20395118713778</v>
+        <v>12.29784726319209</v>
       </c>
       <c r="I6">
-        <v>37.91411392328213</v>
+        <v>27.03710396072432</v>
       </c>
       <c r="J6">
-        <v>5948.951218942929</v>
+        <v>12127.39326419756</v>
       </c>
       <c r="K6">
-        <v>-2098.225645043926</v>
+        <v>-1354.293597721662</v>
       </c>
       <c r="L6">
-        <v>0.01720025647144032</v>
+        <v>0.07042131330167158</v>
       </c>
       <c r="M6">
-        <v>51.18</v>
+        <v>86.11</v>
       </c>
       <c r="N6">
-        <v>25.10655846503516</v>
+        <v>0.2053905037184341</v>
       </c>
       <c r="O6">
-        <v>27.20532716019928</v>
+        <v>13.16124452928617</v>
       </c>
       <c r="P6">
-        <v>37.91549013245838</v>
+        <v>27.93911730708699</v>
       </c>
       <c r="Q6">
-        <v>-2098.331773081896</v>
+        <v>-1449.374741985125</v>
       </c>
       <c r="R6">
-        <v>0.01684123273201987</v>
+        <v>0.3576364388162609</v>
       </c>
     </row>
     <row r="7" spans="1:18">
@@ -772,55 +772,55 @@
         <v>18</v>
       </c>
       <c r="B7">
-        <v>182.31</v>
+        <v>35.79</v>
       </c>
       <c r="C7">
-        <v>110.99</v>
+        <v>22.39</v>
       </c>
       <c r="D7">
-        <v>7719.505152860743</v>
+        <v>4515.248928142405</v>
       </c>
       <c r="E7">
-        <v>9751.660702614112</v>
+        <v>-1504.50952878</v>
       </c>
       <c r="F7">
-        <v>15.50887427131842</v>
+        <v>2.861951488432676</v>
       </c>
       <c r="G7">
-        <v>55.20444416469978</v>
+        <v>30.76694444444444</v>
       </c>
       <c r="H7">
-        <v>32.21026306540776</v>
+        <v>14.11241592483642</v>
       </c>
       <c r="I7">
-        <v>42.79869949260893</v>
+        <v>28.81194207414506</v>
       </c>
       <c r="J7">
-        <v>4762.456793004173</v>
+        <v>11381.27434266978</v>
       </c>
       <c r="K7">
-        <v>-2222.848152215767</v>
+        <v>-1505.555652132433</v>
       </c>
       <c r="L7">
-        <v>0.001035817413159087</v>
+        <v>0.05592226511386782</v>
       </c>
       <c r="M7">
-        <v>107.11</v>
+        <v>15.89</v>
       </c>
       <c r="N7">
-        <v>15.50258538662682</v>
+        <v>6.31218529773553</v>
       </c>
       <c r="O7">
-        <v>32.21150847465118</v>
+        <v>14.95064596472734</v>
       </c>
       <c r="P7">
-        <v>42.79994513528354</v>
+        <v>29.68868410234995</v>
       </c>
       <c r="Q7">
-        <v>-2222.934098599684</v>
+        <v>-1594.980594046452</v>
       </c>
       <c r="R7">
-        <v>0.000957203662727089</v>
+        <v>0.3621044471629272</v>
       </c>
     </row>
     <row r="8" spans="1:18">
@@ -828,55 +828,55 @@
         <v>18</v>
       </c>
       <c r="B8">
-        <v>23.14</v>
+        <v>135.5</v>
       </c>
       <c r="C8">
-        <v>21.26</v>
+        <v>76.38</v>
       </c>
       <c r="D8">
-        <v>5085.014198187559</v>
+        <v>1057.186077302404</v>
       </c>
       <c r="E8">
-        <v>-1516.035409680367</v>
+        <v>2483.44971924</v>
       </c>
       <c r="F8">
-        <v>10.80367094282593</v>
+        <v>0.08937217839633568</v>
       </c>
       <c r="G8">
-        <v>63.32333306630434</v>
+        <v>34.20833333333333</v>
       </c>
       <c r="H8">
-        <v>37.20568413731235</v>
+        <v>15.9261101207881</v>
       </c>
       <c r="I8">
-        <v>47.69417586830113</v>
+        <v>30.58765465325848</v>
       </c>
       <c r="J8">
-        <v>3707.795081058612</v>
+        <v>10658.84173611114</v>
       </c>
       <c r="K8">
-        <v>-2265.516120142723</v>
+        <v>-1644.238152387033</v>
       </c>
       <c r="L8">
-        <v>0.003123771139530943</v>
+        <v>0.04345644732966312</v>
       </c>
       <c r="M8">
-        <v>17.38</v>
+        <v>69.88</v>
       </c>
       <c r="N8">
-        <v>10.79209645251792</v>
+        <v>0.04366978335534576</v>
       </c>
       <c r="O8">
-        <v>37.20679898249758</v>
+        <v>16.73917064342155</v>
       </c>
       <c r="P8">
-        <v>47.69529094471418</v>
+        <v>31.43912765435987</v>
       </c>
       <c r="Q8">
-        <v>-2265.584004924233</v>
+        <v>-1728.179875844582</v>
       </c>
       <c r="R8">
-        <v>0.003249632990725502</v>
+        <v>0.3655392520903757</v>
       </c>
     </row>
     <row r="9" spans="1:18">
@@ -884,55 +884,55 @@
         <v>18</v>
       </c>
       <c r="B9">
-        <v>39.85</v>
+        <v>29.36</v>
       </c>
       <c r="C9">
-        <v>25.77</v>
+        <v>20.81</v>
       </c>
       <c r="D9">
-        <v>2981.08197685558</v>
+        <v>5420.729269862404</v>
       </c>
       <c r="E9">
-        <v>-1407.023587274838</v>
+        <v>-1532.14877762</v>
       </c>
       <c r="F9">
-        <v>5.672246027534334</v>
+        <v>0.006650456254538931</v>
       </c>
       <c r="G9">
-        <v>71.44222196790889</v>
+        <v>37.64972222222222</v>
       </c>
       <c r="H9">
-        <v>42.18990073968807</v>
+        <v>17.73892303814511</v>
       </c>
       <c r="I9">
-        <v>52.60085671352221</v>
+        <v>32.36424851096655</v>
       </c>
       <c r="J9">
-        <v>2784.966083106246</v>
+        <v>9960.095444521634</v>
       </c>
       <c r="K9">
-        <v>-2226.478259689132</v>
+        <v>-1770.349446685506</v>
       </c>
       <c r="L9">
-        <v>0.01762549960078353</v>
+        <v>0.0328793322989577</v>
       </c>
       <c r="M9">
-        <v>21.89</v>
+        <v>14.31</v>
       </c>
       <c r="N9">
-        <v>5.679357239199657</v>
+        <v>0.6181829454218588</v>
       </c>
       <c r="O9">
-        <v>42.1908850205681</v>
+        <v>18.52681173461736</v>
       </c>
       <c r="P9">
-        <v>52.60184122392071</v>
+        <v>33.1904547938682</v>
       </c>
       <c r="Q9">
-        <v>-2226.530202925366</v>
+        <v>-1848.980957451408</v>
       </c>
       <c r="R9">
-        <v>0.01788781675964047</v>
+        <v>0.3679175888142764</v>
       </c>
     </row>
     <row r="10" spans="1:18">
@@ -940,55 +940,55 @@
         <v>18</v>
       </c>
       <c r="B10">
-        <v>145.4</v>
+        <v>42.79</v>
       </c>
       <c r="C10">
-        <v>87.65000000000001</v>
+        <v>36.42</v>
       </c>
       <c r="D10">
-        <v>2595.975308298406</v>
+        <v>3623.510500142404</v>
       </c>
       <c r="E10">
-        <v>4465.830126129625</v>
+        <v>-2192.32382484</v>
       </c>
       <c r="F10">
-        <v>22.99383085482459</v>
+        <v>75.47666753534391</v>
       </c>
       <c r="G10">
-        <v>79.56111086951344</v>
+        <v>41.0911111111111</v>
       </c>
       <c r="H10">
-        <v>47.16266120965867</v>
+        <v>19.55084811409046</v>
       </c>
       <c r="I10">
-        <v>57.51899369114837</v>
+        <v>34.14173021008629</v>
       </c>
       <c r="J10">
-        <v>1993.969799147075</v>
+        <v>9285.035467901262</v>
       </c>
       <c r="K10">
-        <v>-2105.996236658782</v>
+        <v>-1883.898001109188</v>
       </c>
       <c r="L10">
-        <v>0.03927344343877169</v>
+        <v>0.02404947182152869</v>
       </c>
       <c r="M10">
-        <v>83.77000000000001</v>
+        <v>29.92</v>
       </c>
       <c r="N10">
-        <v>22.99186517905022</v>
+        <v>62.70030607420173</v>
       </c>
       <c r="O10">
-        <v>47.16351492598094</v>
+        <v>20.31356265830353</v>
       </c>
       <c r="P10">
-        <v>57.51984763578491</v>
+        <v>34.94267210088616</v>
       </c>
       <c r="Q10">
-        <v>-2106.034358412639</v>
+        <v>-1957.392327128955</v>
       </c>
       <c r="R10">
-        <v>0.03961254322065077</v>
+        <v>0.3692210502723116</v>
       </c>
     </row>
     <row r="11" spans="1:18">
@@ -996,55 +996,55 @@
         <v>18</v>
       </c>
       <c r="B11">
-        <v>32.94</v>
+        <v>13.56</v>
       </c>
       <c r="C11">
-        <v>24.39</v>
+        <v>10.26</v>
       </c>
       <c r="D11">
-        <v>3783.392202433316</v>
+        <v>7996.938293062403</v>
       </c>
       <c r="E11">
-        <v>-1500.21147328806</v>
+        <v>-917.5066765199999</v>
       </c>
       <c r="F11">
-        <v>0.2001953698168769</v>
+        <v>4.96693458583156</v>
       </c>
       <c r="G11">
-        <v>87.67999977111799</v>
+        <v>44.53249999999999</v>
       </c>
       <c r="H11">
-        <v>52.12378372081377</v>
+        <v>21.36187904697708</v>
       </c>
       <c r="I11">
-        <v>62.44876862759006</v>
+        <v>35.92010605226475</v>
       </c>
       <c r="J11">
-        <v>1334.8062291811</v>
+        <v>8633.661806250024</v>
       </c>
       <c r="K11">
-        <v>-1904.342441222479</v>
+        <v>-1984.892396347495</v>
       </c>
       <c r="L11">
-        <v>0.0634795827320279</v>
+        <v>0.01682867822056685</v>
       </c>
       <c r="M11">
-        <v>20.51</v>
+        <v>3.76</v>
       </c>
       <c r="N11">
-        <v>0.198762959783889</v>
+        <v>10.318514450103</v>
       </c>
       <c r="O11">
-        <v>52.12450687232172</v>
+        <v>22.099417096323</v>
       </c>
       <c r="P11">
-        <v>62.44949200672117</v>
+        <v>36.69578589357082</v>
       </c>
       <c r="Q11">
-        <v>-1904.368861562863</v>
+        <v>-2053.422588047596</v>
       </c>
       <c r="R11">
-        <v>0.06384450396441585</v>
+        <v>0.3694362222551806</v>
       </c>
     </row>
     <row r="12" spans="1:18">
@@ -1052,55 +1052,55 @@
         <v>18</v>
       </c>
       <c r="B12">
-        <v>134.9</v>
+        <v>16.889999</v>
       </c>
       <c r="C12">
-        <v>71.16</v>
+        <v>11.69</v>
       </c>
       <c r="D12">
-        <v>1636.26030374938</v>
+        <v>7412.452855933609</v>
       </c>
       <c r="E12">
-        <v>2878.472843986127</v>
+        <v>-1006.45759907</v>
       </c>
       <c r="F12">
-        <v>221.6923363280198</v>
+        <v>6.427619349279396</v>
       </c>
       <c r="G12">
-        <v>95.79888867272254</v>
+        <v>47.97388888888888</v>
       </c>
       <c r="H12">
-        <v>57.07316218966984</v>
+        <v>23.17200980715261</v>
       </c>
       <c r="I12">
-        <v>67.39028760633077</v>
+        <v>37.69938206715431</v>
       </c>
       <c r="J12">
-        <v>807.4753732083196</v>
+        <v>8005.974459567927</v>
       </c>
       <c r="K12">
-        <v>-1621.797320784154</v>
+        <v>-2073.341324172547</v>
       </c>
       <c r="L12">
-        <v>0.08642645692537579</v>
+        <v>0.01108220289252352</v>
       </c>
       <c r="M12">
-        <v>67.28</v>
+        <v>5.19</v>
       </c>
       <c r="N12">
-        <v>221.6912610103579</v>
+        <v>12.21121167672809</v>
       </c>
       <c r="O12">
-        <v>57.07375477610455</v>
+        <v>23.88436900322604</v>
       </c>
       <c r="P12">
-        <v>67.39088042021538</v>
+        <v>38.44980221737192</v>
       </c>
       <c r="Q12">
-        <v>-1621.814159786152</v>
+        <v>-2137.080454751435</v>
       </c>
       <c r="R12">
-        <v>0.0867752296721124</v>
+        <v>0.368554812262245</v>
       </c>
     </row>
     <row r="13" spans="1:18">
@@ -1108,55 +1108,55 @@
         <v>18</v>
       </c>
       <c r="B13">
-        <v>48.49</v>
+        <v>85.550003</v>
       </c>
       <c r="C13">
-        <v>39.72</v>
+        <v>51.25</v>
       </c>
       <c r="D13">
-        <v>2112.255923455921</v>
+        <v>304.0001124888009</v>
       </c>
       <c r="E13">
-        <v>-1825.502819967271</v>
+        <v>-893.5744487499998</v>
       </c>
       <c r="F13">
-        <v>39.75907506237547</v>
+        <v>1.483894782548073</v>
       </c>
       <c r="G13">
-        <v>103.9177775743271</v>
+        <v>51.41527777777777</v>
       </c>
       <c r="H13">
-        <v>62.01076981738558</v>
+        <v>24.9812346474837</v>
       </c>
       <c r="I13">
-        <v>72.34357742621182</v>
+        <v>39.47956400188831</v>
       </c>
       <c r="J13">
-        <v>411.9772312287345</v>
+        <v>7401.973427854964</v>
       </c>
       <c r="K13">
-        <v>-1258.646377125815</v>
+        <v>-2149.253583664417</v>
       </c>
       <c r="L13">
-        <v>0.105134917392095</v>
+        <v>0.00667891172177141</v>
       </c>
       <c r="M13">
-        <v>35.84</v>
+        <v>44.75</v>
       </c>
       <c r="N13">
-        <v>39.74200789347633</v>
+        <v>0.5808402266173337</v>
       </c>
       <c r="O13">
-        <v>62.01123183848755</v>
+        <v>25.66841261682212</v>
       </c>
       <c r="P13">
-        <v>72.34403967510941</v>
+        <v>40.20472683447998</v>
       </c>
       <c r="Q13">
-        <v>-1258.655754870808</v>
+        <v>-2208.374749373679</v>
       </c>
       <c r="R13">
-        <v>0.105434747058748</v>
+        <v>0.3665737715038319</v>
       </c>
     </row>
     <row r="14" spans="1:18">
@@ -1164,55 +1164,55 @@
         <v>18</v>
       </c>
       <c r="B14">
-        <v>14.609999656677</v>
+        <v>61.560001</v>
       </c>
       <c r="C14">
-        <v>10.710000038147</v>
+        <v>39.459999</v>
       </c>
       <c r="D14">
-        <v>6374.311563599057</v>
+        <v>1716.080418211201</v>
       </c>
       <c r="E14">
-        <v>-855.0787544026153</v>
+        <v>-1634.654174034399</v>
       </c>
       <c r="F14">
-        <v>4.273471385272138</v>
+        <v>3.759993488654166</v>
       </c>
       <c r="G14">
-        <v>112.0366664759316</v>
+        <v>54.85666666666665</v>
       </c>
       <c r="H14">
-        <v>66.9366599956837</v>
+        <v>26.78954811353956</v>
       </c>
       <c r="I14">
-        <v>77.30858469551049</v>
+        <v>41.26065731089754</v>
       </c>
       <c r="J14">
-        <v>148.3118032423444</v>
+        <v>6821.658711111135</v>
       </c>
       <c r="K14">
-        <v>-815.1769589241504</v>
+        <v>-2212.638077190948</v>
       </c>
       <c r="L14">
-        <v>0.1175043540786763</v>
+        <v>0.003491456744817566</v>
       </c>
       <c r="M14">
-        <v>6.830000038146999</v>
+        <v>32.959999</v>
       </c>
       <c r="N14">
-        <v>4.28132367736041</v>
+        <v>1.708883418182524</v>
       </c>
       <c r="O14">
-        <v>66.9369914511946</v>
+        <v>27.45154246839012</v>
       </c>
       <c r="P14">
-        <v>77.30891637967939</v>
+        <v>41.9605652136161</v>
       </c>
       <c r="Q14">
-        <v>-815.1809954998537</v>
+        <v>-2267.314397605905</v>
       </c>
       <c r="R14">
-        <v>0.1177317026014065</v>
+        <v>0.3634954094845989</v>
       </c>
     </row>
     <row r="15" spans="1:18">
@@ -1220,55 +1220,55 @@
         <v>18</v>
       </c>
       <c r="B15">
-        <v>17.920000076294</v>
+        <v>180.910004</v>
       </c>
       <c r="C15">
-        <v>12.319999694824</v>
+        <v>118.910004</v>
       </c>
       <c r="D15">
-        <v>5856.731527105735</v>
+        <v>6072.212427057602</v>
       </c>
       <c r="E15">
-        <v>-942.8407730363949</v>
+        <v>9265.990953517607</v>
       </c>
       <c r="F15">
-        <v>6.117976739056285</v>
+        <v>366.6224259369736</v>
       </c>
       <c r="G15">
-        <v>120.1555553775362</v>
+        <v>58.29805555555554</v>
       </c>
       <c r="H15">
-        <v>71.85096450644581</v>
+        <v>28.59694505339505</v>
       </c>
       <c r="I15">
-        <v>82.28517763234517</v>
+        <v>43.04266714610714</v>
       </c>
       <c r="J15">
-        <v>16.47908924914938</v>
+        <v>6265.030309336441</v>
       </c>
       <c r="K15">
-        <v>-291.6749991504826</v>
+        <v>-2263.503806147159</v>
       </c>
       <c r="L15">
-        <v>0.1223232049114333</v>
+        <v>0.001396443448674873</v>
       </c>
       <c r="M15">
-        <v>8.439999694823999</v>
+        <v>112.410004</v>
       </c>
       <c r="N15">
-        <v>6.127107791257605</v>
+        <v>375.9791973319084</v>
       </c>
       <c r="O15">
-        <v>71.85116539611023</v>
+        <v>29.23375339250713</v>
       </c>
       <c r="P15">
-        <v>82.28537875204078</v>
+        <v>43.71732252020324</v>
       </c>
       <c r="Q15">
-        <v>-291.6758146509161</v>
+        <v>-2313.908424426318</v>
       </c>
       <c r="R15">
-        <v>0.1224637665213901</v>
+        <v>0.3593275006194322</v>
       </c>
     </row>
     <row r="16" spans="1:18">
@@ -1276,55 +1276,55 @@
         <v>18</v>
       </c>
       <c r="B16">
-        <v>96.98999786377</v>
+        <v>64.199997</v>
       </c>
       <c r="C16">
-        <v>59.290000915527</v>
+        <v>39.200001</v>
       </c>
       <c r="D16">
-        <v>6.455219327276619</v>
+        <v>1504.323155216025</v>
       </c>
       <c r="E16">
-        <v>150.63883851243</v>
+        <v>-1520.395754785605</v>
       </c>
       <c r="F16">
-        <v>13.44881678345931</v>
+        <v>0.09138511563656197</v>
       </c>
       <c r="G16">
-        <v>128.2744442791407</v>
+        <v>61.73944444444443</v>
       </c>
       <c r="H16">
-        <v>76.75388915467806</v>
+        <v>30.40342062701389</v>
       </c>
       <c r="I16">
-        <v>87.27315043170969</v>
+        <v>44.82559834755338</v>
       </c>
       <c r="J16">
-        <v>16.47908924914938</v>
+        <v>5732.088222530886</v>
       </c>
       <c r="K16">
-        <v>311.5781494064507</v>
+        <v>-2301.859866460463</v>
       </c>
       <c r="L16">
-        <v>0.1192498703135998</v>
+        <v>0.0002745930917143237</v>
       </c>
       <c r="M16">
-        <v>55.410000915527</v>
+        <v>32.700001</v>
       </c>
       <c r="N16">
-        <v>13.45302379408194</v>
+        <v>0.09621249470389934</v>
       </c>
       <c r="O16">
-        <v>76.75395947824515</v>
+        <v>31.01504053645622</v>
       </c>
       <c r="P16">
-        <v>87.27322098718292</v>
+        <v>45.47500360695827</v>
       </c>
       <c r="Q16">
-        <v>311.5784348810649</v>
+        <v>-2348.165949593181</v>
       </c>
       <c r="R16">
-        <v>0.1192984443354259</v>
+        <v>0.3540833823534913</v>
       </c>
     </row>
     <row r="17" spans="1:18">
@@ -1332,55 +1332,55 @@
         <v>18</v>
       </c>
       <c r="B17">
-        <v>50.369998931885</v>
+        <v>95.69000200000001</v>
       </c>
       <c r="C17">
-        <v>34.569999694824</v>
+        <v>63.389999</v>
       </c>
       <c r="D17">
-        <v>1942.983504148192</v>
+        <v>53.2257793599999</v>
       </c>
       <c r="E17">
-        <v>-1523.820923127089</v>
+        <v>-462.4680767043996</v>
       </c>
       <c r="F17">
-        <v>0.0001064620019475684</v>
+        <v>65.12627992607956</v>
       </c>
       <c r="G17">
-        <v>136.3933331807453</v>
+        <v>65.18083333333333</v>
       </c>
       <c r="H17">
-        <v>81.64570716561455</v>
+        <v>32.20897031517408</v>
       </c>
       <c r="I17">
-        <v>92.27222986836999</v>
+        <v>46.60945543445828</v>
       </c>
       <c r="J17">
-        <v>148.3118032423444</v>
+        <v>5222.832450694465</v>
       </c>
       <c r="K17">
-        <v>994.3086386558446</v>
+        <v>-2327.71544386904</v>
       </c>
       <c r="L17">
-        <v>0.1087663967806528</v>
+        <v>1.089944297256455E-05</v>
       </c>
       <c r="M17">
-        <v>30.689999694824</v>
+        <v>56.889999</v>
       </c>
       <c r="N17">
-        <v>8.090590014752722E-05</v>
+        <v>59.11103691555994</v>
       </c>
       <c r="O17">
-        <v>81.64564692283942</v>
+        <v>32.79539936917528</v>
       </c>
       <c r="P17">
-        <v>92.27216985986568</v>
+        <v>47.23361300494336</v>
       </c>
       <c r="Q17">
-        <v>994.3079049992468</v>
+        <v>-2370.096182910828</v>
       </c>
       <c r="R17">
-        <v>0.1087266645755251</v>
+        <v>0.3477820442832472</v>
       </c>
     </row>
     <row r="18" spans="1:18">
@@ -1388,55 +1388,55 @@
         <v>18</v>
       </c>
       <c r="B18">
-        <v>16.26</v>
+        <v>121.790001</v>
       </c>
       <c r="C18">
-        <v>15.46</v>
+        <v>74.69000200000001</v>
       </c>
       <c r="D18">
-        <v>6113.564366635434</v>
+        <v>353.6054217512012</v>
       </c>
       <c r="E18">
-        <v>-1208.806353793908</v>
+        <v>1404.500598918798</v>
       </c>
       <c r="F18">
-        <v>2.814676209413497</v>
+        <v>33.16371176447267</v>
       </c>
       <c r="G18">
-        <v>144.5122220823498</v>
+        <v>68.62222222222222</v>
       </c>
       <c r="H18">
-        <v>86.5267508237969</v>
+        <v>34.01358992789823</v>
       </c>
       <c r="I18">
-        <v>97.28208365778443</v>
+        <v>48.39424259679922</v>
       </c>
       <c r="J18">
-        <v>411.9772312287345</v>
+        <v>4737.262993827178</v>
       </c>
       <c r="K18">
-        <v>1756.252692388067</v>
+        <v>-2341.079808981845</v>
       </c>
       <c r="L18">
-        <v>0.09210916618180391</v>
+        <v>0.0004947793475855651</v>
       </c>
       <c r="M18">
-        <v>11.58</v>
+        <v>68.19000200000001</v>
       </c>
       <c r="N18">
-        <v>2.808399019475039</v>
+        <v>31.00647388786647</v>
       </c>
       <c r="O18">
-        <v>86.52656001444201</v>
+        <v>34.57482568970939</v>
       </c>
       <c r="P18">
-        <v>97.28189308554012</v>
+        <v>48.99315491511339</v>
       </c>
       <c r="Q18">
-        <v>1756.248819488183</v>
+        <v>-2379.708419276724</v>
       </c>
       <c r="R18">
-        <v>0.09199338325039684</v>
+        <v>0.3404482078034555</v>
       </c>
     </row>
     <row r="19" spans="1:18">
@@ -1444,55 +1444,55 @@
         <v>18</v>
       </c>
       <c r="B19">
-        <v>67.889999389648</v>
+        <v>34.225982</v>
       </c>
       <c r="C19">
-        <v>44.590000152588</v>
+        <v>22.625982</v>
       </c>
       <c r="D19">
-        <v>705.3956785675285</v>
+        <v>4727.885342544399</v>
       </c>
       <c r="E19">
-        <v>-1184.278571609126</v>
+        <v>-1555.75392444684</v>
       </c>
       <c r="F19">
-        <v>0.4116731985843231</v>
+        <v>0.4097334694939737</v>
       </c>
       <c r="G19">
-        <v>152.6311109839544</v>
+        <v>72.06361111111111</v>
       </c>
       <c r="H19">
-        <v>91.39740191914416</v>
+        <v>35.81727561235326</v>
       </c>
       <c r="I19">
-        <v>102.302330010034</v>
+        <v>50.1799636874093</v>
       </c>
       <c r="J19">
-        <v>807.4753732083196</v>
+        <v>4275.379851929029</v>
       </c>
       <c r="K19">
-        <v>2597.158732268904</v>
+        <v>-2341.96231212985</v>
       </c>
       <c r="L19">
-        <v>0.07118211592453576</v>
+        <v>0.001620216541707712</v>
       </c>
       <c r="M19">
-        <v>40.71000015258799</v>
+        <v>16.125982</v>
       </c>
       <c r="N19">
-        <v>0.4130108001714324</v>
+        <v>2.167495602654039</v>
       </c>
       <c r="O19">
-        <v>91.39708054298045</v>
+        <v>36.35331563513122</v>
       </c>
       <c r="P19">
-        <v>102.3020088742787</v>
+        <v>50.75363320039568</v>
       </c>
       <c r="Q19">
-        <v>2597.149600008114</v>
+        <v>-2377.01203351922</v>
       </c>
       <c r="R19">
-        <v>0.07101073303567421</v>
+        <v>0.3321123958375676</v>
       </c>
     </row>
     <row r="20" spans="1:18">
@@ -1500,55 +1500,55 @@
         <v>18</v>
       </c>
       <c r="B20">
-        <v>65.620002746582</v>
+        <v>100.94474</v>
       </c>
       <c r="C20">
-        <v>42.419998168945</v>
+        <v>56.676224</v>
       </c>
       <c r="D20">
-        <v>831.1275439419171</v>
+        <v>4.165117703044017</v>
       </c>
       <c r="E20">
-        <v>-1222.938121512957</v>
+        <v>-115.6683518650882</v>
       </c>
       <c r="F20">
-        <v>2.04175345761865</v>
+        <v>1.915634559248155</v>
       </c>
       <c r="G20">
-        <v>160.7499998855589</v>
+        <v>75.50500000000001</v>
       </c>
       <c r="H20">
-        <v>96.25808158770762</v>
+        <v>37.62002386018566</v>
       </c>
       <c r="I20">
-        <v>107.3325477890673</v>
+        <v>51.96662221464198</v>
       </c>
       <c r="J20">
-        <v>1334.8062291811</v>
+        <v>3837.183025000015</v>
       </c>
       <c r="K20">
-        <v>3516.789016314831</v>
+        <v>-2330.372378019205</v>
       </c>
       <c r="L20">
-        <v>0.04845862073791947</v>
+        <v>0.003285898159995985</v>
       </c>
       <c r="M20">
-        <v>38.539998168945</v>
+        <v>50.176224</v>
       </c>
       <c r="N20">
-        <v>2.044835402719979</v>
+        <v>2.983468089640847</v>
       </c>
       <c r="O20">
-        <v>96.25762964451521</v>
+        <v>38.13086568789562</v>
       </c>
       <c r="P20">
-        <v>107.332096090021</v>
+        <v>52.51505137833543</v>
       </c>
       <c r="Q20">
-        <v>3516.77250457027</v>
+        <v>-2362.016475036699</v>
       </c>
       <c r="R20">
-        <v>0.04825984959851298</v>
+        <v>0.3228109922451789</v>
       </c>
     </row>
     <row r="21" spans="1:18">
@@ -1556,55 +1556,55 @@
         <v>18</v>
       </c>
       <c r="B21">
-        <v>37.849998474121</v>
+        <v>201.277569</v>
       </c>
       <c r="C21">
-        <v>29.14999961853</v>
+        <v>81.830321</v>
       </c>
       <c r="D21">
-        <v>3203.479291573566</v>
+        <v>9661.310776729089</v>
       </c>
       <c r="E21">
-        <v>-1649.86919514539</v>
+        <v>8043.263211331407</v>
       </c>
       <c r="F21">
-        <v>4.913361274994942</v>
+        <v>815.3362933349026</v>
       </c>
       <c r="G21">
-        <v>168.8688887871635</v>
+        <v>78.9463888888889</v>
       </c>
       <c r="H21">
-        <v>101.1092400991161</v>
+        <v>39.42183151426043</v>
       </c>
       <c r="I21">
-        <v>112.3722867252556</v>
+        <v>53.75422133563232</v>
       </c>
       <c r="J21">
-        <v>1993.969799147075</v>
+        <v>3422.672513040137</v>
       </c>
       <c r="K21">
-        <v>4514.92078009711</v>
+        <v>-2306.319500198041</v>
       </c>
       <c r="L21">
-        <v>0.02687811144042358</v>
+        <v>0.005395343402445789</v>
       </c>
       <c r="M21">
-        <v>25.26999961853</v>
+        <v>75.330321</v>
       </c>
       <c r="N21">
-        <v>4.90660464857203</v>
+        <v>793.1004951923939</v>
       </c>
       <c r="O21">
-        <v>101.1086575886851</v>
+        <v>39.90747268259602</v>
       </c>
       <c r="P21">
-        <v>112.3717044631281</v>
+        <v>54.27741261433918</v>
       </c>
       <c r="Q21">
-        <v>4514.894768741006</v>
+        <v>-2334.731262249892</v>
       </c>
       <c r="R21">
-        <v>0.0266874508862774</v>
+        <v>0.3125862905392953</v>
       </c>
     </row>
     <row r="22" spans="1:18">
@@ -1612,55 +1612,55 @@
         <v>18</v>
       </c>
       <c r="B22">
-        <v>81.25</v>
+        <v>70.31999999999999</v>
       </c>
       <c r="C22">
-        <v>63.849998474121</v>
+        <v>42.54</v>
       </c>
       <c r="D22">
-        <v>174.2211376488813</v>
+        <v>1067.041554022404</v>
       </c>
       <c r="E22">
-        <v>-842.774358885426</v>
+        <v>-1389.59470908</v>
       </c>
       <c r="F22">
-        <v>109.8392051164199</v>
+        <v>0.20311535813847</v>
       </c>
       <c r="G22">
-        <v>176.987777688768</v>
+        <v>82.3877777777778</v>
       </c>
       <c r="H22">
-        <v>105.9513470625915</v>
+        <v>41.22269577477378</v>
       </c>
       <c r="I22">
-        <v>117.4210772093769</v>
+        <v>55.54276385018404</v>
       </c>
       <c r="J22">
-        <v>2784.966083106246</v>
+        <v>3031.848316049395</v>
       </c>
       <c r="K22">
-        <v>5591.346902547419</v>
+        <v>-2269.813235349659</v>
       </c>
       <c r="L22">
-        <v>0.009742907740996461</v>
+        <v>0.007857023854873791</v>
       </c>
       <c r="M22">
-        <v>59.969998474121</v>
+        <v>36.04</v>
       </c>
       <c r="N22">
-        <v>109.8218780947433</v>
+        <v>0.01367709897068594</v>
       </c>
       <c r="O22">
-        <v>105.9506339847224</v>
+        <v>41.6831338120933</v>
       </c>
       <c r="P22">
-        <v>117.4203643843679</v>
+        <v>56.04071971554603</v>
       </c>
       <c r="Q22">
-        <v>5591.309271447435</v>
+        <v>-2295.165976880111</v>
       </c>
       <c r="R22">
-        <v>0.009602645852143796</v>
+        <v>0.3014865315890716</v>
       </c>
     </row>
     <row r="23" spans="1:18">
@@ -1668,55 +1668,55 @@
         <v>18</v>
       </c>
       <c r="B23">
-        <v>196.190002441406</v>
+        <v>29.952212</v>
       </c>
       <c r="C23">
-        <v>137.490005493164</v>
+        <v>20.252212</v>
       </c>
       <c r="D23">
-        <v>10351.17348422634</v>
+        <v>5333.8760548921</v>
       </c>
       <c r="E23">
-        <v>13988.33173147333</v>
+        <v>-1479.08769735868</v>
       </c>
       <c r="F23">
-        <v>199.0121330359492</v>
+        <v>0.6163498403909494</v>
       </c>
       <c r="G23">
-        <v>185.1066665903726</v>
+        <v>85.82916666666669</v>
       </c>
       <c r="H23">
-        <v>110.7848824165389</v>
+        <v>43.02261420471277</v>
       </c>
       <c r="I23">
-        <v>122.4784393030264</v>
+        <v>57.33225219531015</v>
       </c>
       <c r="J23">
-        <v>3707.795081058611</v>
+        <v>2664.710434027788</v>
       </c>
       <c r="K23">
-        <v>6745.876142379017</v>
+        <v>-2220.863197425782</v>
       </c>
       <c r="L23">
-        <v>0.0006197747298017207</v>
+        <v>0.01058447498864428</v>
       </c>
       <c r="M23">
-        <v>133.610005493164</v>
+        <v>13.752212</v>
       </c>
       <c r="N23">
-        <v>199.0409622138604</v>
+        <v>2.71767123634853</v>
       </c>
       <c r="O23">
-        <v>110.7840387710427</v>
+        <v>43.45784663298967</v>
       </c>
       <c r="P23">
-        <v>122.4775959153247</v>
+        <v>57.80497512535381</v>
       </c>
       <c r="Q23">
-        <v>6745.824771398597</v>
+        <v>-2243.330258067126</v>
       </c>
       <c r="R23">
-        <v>0.0005784808938411909</v>
+        <v>0.2895659300292264</v>
       </c>
     </row>
     <row r="24" spans="1:18">
@@ -1724,55 +1724,55 @@
         <v>18</v>
       </c>
       <c r="B24">
-        <v>193.559997558594</v>
+        <v>64.300003</v>
       </c>
       <c r="C24">
-        <v>130.360000610352</v>
+        <v>28.68</v>
       </c>
       <c r="D24">
-        <v>9822.933245224291</v>
+        <v>1496.575569988801</v>
       </c>
       <c r="E24">
-        <v>12920.07248475507</v>
+        <v>-1109.50297932</v>
       </c>
       <c r="F24">
-        <v>73.60220499994074</v>
+        <v>105.4699211441236</v>
       </c>
       <c r="G24">
-        <v>193.2255554919771</v>
+        <v>89.27055555555559</v>
       </c>
       <c r="H24">
-        <v>115.6103284506142</v>
+        <v>44.82158473463686</v>
       </c>
       <c r="I24">
-        <v>127.5438907165478</v>
+        <v>59.12268844045116</v>
       </c>
       <c r="J24">
-        <v>4762.456793004171</v>
+        <v>2321.258866975318</v>
       </c>
       <c r="K24">
-        <v>7978.333006832663</v>
+        <v>-2159.4790516344</v>
       </c>
       <c r="L24">
-        <v>0.003249562965363522</v>
+        <v>0.01349639839996538</v>
       </c>
       <c r="M24">
-        <v>126.480000610352</v>
+        <v>22.18</v>
       </c>
       <c r="N24">
-        <v>73.61901187476565</v>
+        <v>118.4092883556502</v>
       </c>
       <c r="O24">
-        <v>115.6093542373126</v>
+        <v>45.23160907042277</v>
       </c>
       <c r="P24">
-        <v>127.5429167663318</v>
+        <v>59.57018091862485</v>
       </c>
       <c r="Q24">
-        <v>7978.265775831383</v>
+        <v>-2179.233796341268</v>
       </c>
       <c r="R24">
-        <v>0.003361581994790644</v>
+        <v>0.2768846891453528</v>
       </c>
     </row>
     <row r="25" spans="1:18">
@@ -1780,55 +1780,55 @@
         <v>18</v>
       </c>
       <c r="B25">
-        <v>92.029998779297</v>
+        <v>62.765547</v>
       </c>
       <c r="C25">
-        <v>56.529998779297</v>
+        <v>35.197163</v>
       </c>
       <c r="D25">
-        <v>5.852948225673935</v>
+        <v>1617.652824203025</v>
       </c>
       <c r="E25">
-        <v>-136.7622752361374</v>
+        <v>-1415.631831703965</v>
       </c>
       <c r="F25">
-        <v>11.6007467211298</v>
+        <v>8.717047566117088</v>
       </c>
       <c r="G25">
-        <v>201.3444443935817</v>
+        <v>92.71194444444448</v>
       </c>
       <c r="H25">
-        <v>120.4281629983217</v>
+        <v>46.61960566676003</v>
       </c>
       <c r="I25">
-        <v>132.6169536164371</v>
+        <v>60.91407428339308</v>
       </c>
       <c r="J25">
-        <v>5948.951218942927</v>
+        <v>2001.493614891983</v>
       </c>
       <c r="K25">
-        <v>9288.557322073124</v>
+        <v>-2085.670508297607</v>
       </c>
       <c r="L25">
-        <v>0.02146712514519689</v>
+        <v>0.0165167543872387</v>
       </c>
       <c r="M25">
-        <v>52.649998779297</v>
+        <v>28.697163</v>
       </c>
       <c r="N25">
-        <v>11.60519747950523</v>
+        <v>12.78389800465068</v>
       </c>
       <c r="O25">
-        <v>120.4270582170468</v>
+        <v>47.00441942215846</v>
       </c>
       <c r="P25">
-        <v>132.6158491038746</v>
+        <v>61.33633879759329</v>
       </c>
       <c r="Q25">
-        <v>9288.472110907027</v>
+        <v>-2102.886327465164</v>
       </c>
       <c r="R25">
-        <v>0.02179208336260765</v>
+        <v>0.2635090040550479</v>
       </c>
     </row>
     <row r="26" spans="1:18">
@@ -1836,55 +1836,55 @@
         <v>18</v>
       </c>
       <c r="B26">
-        <v>57.340000152588</v>
+        <v>120.717151</v>
       </c>
       <c r="C26">
-        <v>42.139999389648</v>
+        <v>57.828844</v>
       </c>
       <c r="D26">
-        <v>1377.09905882238</v>
+        <v>314.407829939401</v>
       </c>
       <c r="E26">
-        <v>-1563.785261791837</v>
+        <v>1025.394980999356</v>
       </c>
       <c r="F26">
-        <v>11.12015433652707</v>
+        <v>111.1520335814055</v>
       </c>
       <c r="G26">
-        <v>209.4633332951862</v>
+        <v>96.15333333333338</v>
       </c>
       <c r="H26">
-        <v>125.2388538425501</v>
+        <v>48.41667567831461</v>
       </c>
       <c r="I26">
-        <v>137.6971602198055</v>
+        <v>62.7064110469036</v>
       </c>
       <c r="J26">
-        <v>7267.278358874877</v>
+        <v>1705.414677777785</v>
       </c>
       <c r="K26">
-        <v>10676.40357537552</v>
+        <v>-1999.44731659547</v>
       </c>
       <c r="L26">
-        <v>0.05913264150090131</v>
+        <v>0.01957484450594661</v>
       </c>
       <c r="M26">
-        <v>38.25999938964799</v>
+        <v>51.328844</v>
       </c>
       <c r="N26">
-        <v>11.11207796701194</v>
+        <v>115.3728867321592</v>
       </c>
       <c r="O26">
-        <v>125.2376184931445</v>
+        <v>48.7762763619635</v>
       </c>
       <c r="P26">
-        <v>137.6959251450539</v>
+        <v>63.10345008849239</v>
       </c>
       <c r="Q26">
-        <v>10676.29826389744</v>
+        <v>-2014.297626161223</v>
       </c>
       <c r="R26">
-        <v>0.05973497246155524</v>
+        <v>0.2495110530568852</v>
       </c>
     </row>
     <row r="27" spans="1:18">
@@ -1892,55 +1892,55 @@
         <v>18</v>
       </c>
       <c r="B27">
-        <v>70.56999969482401</v>
+        <v>29.673616</v>
       </c>
       <c r="C27">
-        <v>45.270000457764</v>
+        <v>23.973616</v>
       </c>
       <c r="D27">
-        <v>570.2202904537846</v>
+        <v>5374.647291264197</v>
       </c>
       <c r="E27">
-        <v>-1081.015279225709</v>
+        <v>-1757.553400561376</v>
       </c>
       <c r="F27">
-        <v>2.541099328526418</v>
+        <v>9.496343899721124</v>
       </c>
       <c r="G27">
-        <v>217.5822221967908</v>
+        <v>99.59472222222227</v>
       </c>
       <c r="H27">
-        <v>130.0428543012904</v>
+        <v>50.21279382418135</v>
       </c>
       <c r="I27">
-        <v>142.784057208662</v>
+        <v>64.49969967610194</v>
       </c>
       <c r="J27">
-        <v>8717.438212800023</v>
+        <v>1433.022055632722</v>
       </c>
       <c r="K27">
-        <v>12141.74009497682</v>
+        <v>-1900.819258212674</v>
       </c>
       <c r="L27">
-        <v>0.1200746062422986</v>
+        <v>0.0226053837844949</v>
       </c>
       <c r="M27">
-        <v>41.390000457764</v>
+        <v>17.473616</v>
       </c>
       <c r="N27">
-        <v>2.544283460970352</v>
+        <v>4.911168599484327</v>
       </c>
       <c r="O27">
-        <v>130.0414883836065</v>
+        <v>50.54717894224247</v>
       </c>
       <c r="P27">
-        <v>142.782691571869</v>
+        <v>64.87151573891755</v>
       </c>
       <c r="Q27">
-        <v>12141.6125630367</v>
+        <v>-1913.477499741633</v>
       </c>
       <c r="R27">
-        <v>0.1210231016358975</v>
+        <v>0.2349689770729362</v>
       </c>
     </row>
     <row r="28" spans="1:18">
@@ -1948,55 +1948,55 @@
         <v>18</v>
       </c>
       <c r="B28">
-        <v>101.110000610352</v>
+        <v>79.769435</v>
       </c>
       <c r="C28">
-        <v>70.80999755859401</v>
+        <v>40.669435</v>
       </c>
       <c r="D28">
-        <v>44.36512581237114</v>
+        <v>538.9904101718889</v>
       </c>
       <c r="E28">
-        <v>471.6452208678255</v>
+        <v>-944.1883947556449</v>
       </c>
       <c r="F28">
-        <v>28.54894881009995</v>
+        <v>40.294749377817</v>
       </c>
       <c r="G28">
-        <v>225.7011110983953</v>
+        <v>103.0361111111112</v>
       </c>
       <c r="H28">
-        <v>134.8405999073384</v>
+        <v>52.00795953877365</v>
       </c>
       <c r="I28">
-        <v>147.8772090502108</v>
+        <v>66.29394073657475</v>
       </c>
       <c r="J28">
-        <v>10299.43078071836</v>
+        <v>1184.315748456795</v>
       </c>
       <c r="K28">
-        <v>13684.44812591736</v>
+        <v>-1789.796140905189</v>
       </c>
       <c r="L28">
-        <v>0.2080440595631325</v>
+        <v>0.02554856233057633</v>
       </c>
       <c r="M28">
-        <v>66.92999755859401</v>
+        <v>34.169435</v>
       </c>
       <c r="N28">
-        <v>28.54352805702124</v>
+        <v>46.87044474534498</v>
       </c>
       <c r="O28">
-        <v>134.8391034212385</v>
+        <v>52.31712659592696</v>
       </c>
       <c r="P28">
-        <v>147.8757128515141</v>
+        <v>66.64053631593721</v>
       </c>
       <c r="Q28">
-        <v>13684.29625336251</v>
+        <v>-1800.435781658168</v>
       </c>
       <c r="R28">
-        <v>0.2094114489372536</v>
+        <v>0.2199668471657003</v>
       </c>
     </row>
     <row r="29" spans="1:18">
@@ -2004,55 +2004,2575 @@
         <v>18</v>
       </c>
       <c r="B29">
-        <v>129.059997558594</v>
+        <v>22.760776</v>
       </c>
       <c r="C29">
-        <v>81.459999084473</v>
+        <v>16.560776</v>
       </c>
       <c r="D29">
-        <v>1197.901389364506</v>
+        <v>6436.022706730278</v>
       </c>
       <c r="E29">
-        <v>2819.388572796199</v>
+        <v>-1328.585373024976</v>
       </c>
       <c r="F29">
-        <v>1.065073130421706</v>
+        <v>0.5272818595790737</v>
       </c>
       <c r="G29">
-        <v>233.8199999999999</v>
+        <v>106.4775000000001</v>
       </c>
       <c r="H29">
-        <v>139.6325060625153</v>
+        <v>53.80217263716703</v>
       </c>
       <c r="I29">
-        <v>152.9762003426307</v>
+        <v>68.08913441324646</v>
       </c>
       <c r="J29">
-        <v>12013.2560626299</v>
+        <v>959.2957562500042</v>
       </c>
       <c r="K29">
-        <v>15304.4208509515</v>
+        <v>-1666.38779200466</v>
       </c>
       <c r="L29">
-        <v>0.3266791911686779</v>
+        <v>0.02835009610583865</v>
       </c>
       <c r="M29">
-        <v>77.579999084473</v>
+        <v>10.060776</v>
       </c>
       <c r="N29">
-        <v>1.065192449181499</v>
+        <v>2.697145350897132</v>
       </c>
       <c r="O29">
-        <v>139.6308790078705</v>
+        <v>54.08611913760802</v>
       </c>
       <c r="P29">
-        <v>152.9745735821591</v>
+        <v>68.4105120049603</v>
       </c>
       <c r="Q29">
-        <v>15304.24251762688</v>
+        <v>-1675.182324989568</v>
       </c>
       <c r="R29">
-        <v>0.3285417525055422</v>
+        <v>0.2045946201651749</v>
+      </c>
+    </row>
+    <row r="30" spans="1:18">
+      <c r="A30" t="s">
+        <v>18</v>
+      </c>
+      <c r="B30">
+        <v>25.03273</v>
+      </c>
+      <c r="C30">
+        <v>13.33273</v>
+      </c>
+      <c r="D30">
+        <v>6076.650253048384</v>
+      </c>
+      <c r="E30">
+        <v>-1039.32459510056</v>
+      </c>
+      <c r="F30">
+        <v>26.40957148951076</v>
+      </c>
+      <c r="G30">
+        <v>109.918888888889</v>
+      </c>
+      <c r="H30">
+        <v>55.59543331546889</v>
+      </c>
+      <c r="I30">
+        <v>69.88528051000971</v>
+      </c>
+      <c r="J30">
+        <v>757.962079012349</v>
+      </c>
+      <c r="K30">
+        <v>-1530.604051878546</v>
+      </c>
+      <c r="L30">
+        <v>0.03096126669658746</v>
+      </c>
+      <c r="M30">
+        <v>6.83273</v>
+      </c>
+      <c r="N30">
+        <v>36.46386894706053</v>
+      </c>
+      <c r="O30">
+        <v>55.8541567639068</v>
+      </c>
+      <c r="P30">
+        <v>70.18144260936566</v>
+      </c>
+      <c r="Q30">
+        <v>-1537.72699588454</v>
+      </c>
+      <c r="R30">
+        <v>0.1889480824976725</v>
+      </c>
+    </row>
+    <row r="31" spans="1:18">
+      <c r="A31" t="s">
+        <v>18</v>
+      </c>
+      <c r="B31">
+        <v>41.68</v>
+      </c>
+      <c r="C31">
+        <v>26.89</v>
+      </c>
+      <c r="D31">
+        <v>3758.376836582404</v>
+      </c>
+      <c r="E31">
+        <v>-1648.50763778</v>
+      </c>
+      <c r="F31">
+        <v>0.06937849741848641</v>
+      </c>
+      <c r="G31">
+        <v>113.3602777777779</v>
+      </c>
+      <c r="H31">
+        <v>57.38774215042637</v>
+      </c>
+      <c r="I31">
+        <v>71.68237845011731</v>
+      </c>
+      <c r="J31">
+        <v>580.3147167438299</v>
+      </c>
+      <c r="K31">
+        <v>-1382.454767364288</v>
+      </c>
+      <c r="L31">
+        <v>0.03333894995913642</v>
+      </c>
+      <c r="M31">
+        <v>20.39</v>
+      </c>
+      <c r="N31">
+        <v>1.083495064881758</v>
+      </c>
+      <c r="O31">
+        <v>57.62124005308154</v>
+      </c>
+      <c r="P31">
+        <v>71.95332755089508</v>
+      </c>
+      <c r="Q31">
+        <v>-1388.079666978723</v>
+      </c>
+      <c r="R31">
+        <v>0.1731287823627732</v>
+      </c>
+    </row>
+    <row r="32" spans="1:18">
+      <c r="A32" t="s">
+        <v>18</v>
+      </c>
+      <c r="B32">
+        <v>22.12932</v>
+      </c>
+      <c r="C32">
+        <v>17.42932</v>
+      </c>
+      <c r="D32">
+        <v>6537.738338863523</v>
+      </c>
+      <c r="E32">
+        <v>-1409.27001298824</v>
+      </c>
+      <c r="F32">
+        <v>0.2225103642881569</v>
+      </c>
+      <c r="G32">
+        <v>116.8016666666667</v>
+      </c>
+      <c r="H32">
+        <v>59.17910009827472</v>
+      </c>
+      <c r="I32">
+        <v>73.48042727733406</v>
+      </c>
+      <c r="J32">
+        <v>426.3536694444465</v>
+      </c>
+      <c r="K32">
+        <v>-1221.949785195879</v>
+      </c>
+      <c r="L32">
+        <v>0.03544563347050846</v>
+      </c>
+      <c r="M32">
+        <v>10.92932</v>
+      </c>
+      <c r="N32">
+        <v>0.2016678590115071</v>
+      </c>
+      <c r="O32">
+        <v>59.38736996387271</v>
+      </c>
+      <c r="P32">
+        <v>73.72616587080802</v>
+      </c>
+      <c r="Q32">
+        <v>-1226.250210804035</v>
+      </c>
+      <c r="R32">
+        <v>0.1572439504592698</v>
+      </c>
+    </row>
+    <row r="33" spans="1:18">
+      <c r="A33" t="s">
+        <v>18</v>
+      </c>
+      <c r="B33">
+        <v>36.570606</v>
+      </c>
+      <c r="C33">
+        <v>24.270606</v>
+      </c>
+      <c r="D33">
+        <v>4410.951693680016</v>
+      </c>
+      <c r="E33">
+        <v>-1611.932200407576</v>
+      </c>
+      <c r="F33">
+        <v>0.04761764706150799</v>
+      </c>
+      <c r="G33">
+        <v>120.2430555555556</v>
+      </c>
+      <c r="H33">
+        <v>60.96950849283093</v>
+      </c>
+      <c r="I33">
+        <v>75.27942565784292</v>
+      </c>
+      <c r="J33">
+        <v>296.0789371141991</v>
+      </c>
+      <c r="K33">
+        <v>-1049.098945441228</v>
+      </c>
+      <c r="L33">
+        <v>0.03724942276711969</v>
+      </c>
+      <c r="M33">
+        <v>17.770606</v>
+      </c>
+      <c r="N33">
+        <v>1.06744061531326</v>
+      </c>
+      <c r="O33">
+        <v>61.15254783359189</v>
+      </c>
+      <c r="P33">
+        <v>75.49995623179298</v>
+      </c>
+      <c r="Q33">
+        <v>-1052.24849320885</v>
+      </c>
+      <c r="R33">
+        <v>0.1414064095141856</v>
+      </c>
+    </row>
+    <row r="34" spans="1:18">
+      <c r="A34" t="s">
+        <v>18</v>
+      </c>
+      <c r="B34">
+        <v>28.13</v>
+      </c>
+      <c r="C34">
+        <v>20.22</v>
+      </c>
+      <c r="D34">
+        <v>5603.361150782404</v>
+      </c>
+      <c r="E34">
+        <v>-1513.58027244</v>
+      </c>
+      <c r="F34">
+        <v>0.01768957183603532</v>
+      </c>
+      <c r="G34">
+        <v>123.6844444444445</v>
+      </c>
+      <c r="H34">
+        <v>62.75896904284201</v>
+      </c>
+      <c r="I34">
+        <v>77.07937188289694</v>
+      </c>
+      <c r="J34">
+        <v>189.4905197530875</v>
+      </c>
+      <c r="K34">
+        <v>-863.9120749686354</v>
+      </c>
+      <c r="L34">
+        <v>0.03872403640645273</v>
+      </c>
+      <c r="M34">
+        <v>13.72</v>
+      </c>
+      <c r="N34">
+        <v>0.5532503506469325</v>
+      </c>
+      <c r="O34">
+        <v>62.9167753754629</v>
+      </c>
+      <c r="P34">
+        <v>77.27469692062611</v>
+      </c>
+      <c r="Q34">
+        <v>-866.0843668073468</v>
+      </c>
+      <c r="R34">
+        <v>0.1257344729195889</v>
+      </c>
+    </row>
+    <row r="35" spans="1:18">
+      <c r="A35" t="s">
+        <v>18</v>
+      </c>
+      <c r="B35">
+        <v>32.84</v>
+      </c>
+      <c r="C35">
+        <v>23.24</v>
+      </c>
+      <c r="D35">
+        <v>4920.405479942404</v>
+      </c>
+      <c r="E35">
+        <v>-1630.18379048</v>
+      </c>
+      <c r="F35">
+        <v>0.4854062642143876</v>
+      </c>
+      <c r="G35">
+        <v>127.1258333333334</v>
+      </c>
+      <c r="H35">
+        <v>64.54748382859982</v>
+      </c>
+      <c r="I35">
+        <v>78.88026387220422</v>
+      </c>
+      <c r="J35">
+        <v>106.5884173611118</v>
+      </c>
+      <c r="K35">
+        <v>-666.3989809604381</v>
+      </c>
+      <c r="L35">
+        <v>0.03984878993813478</v>
+      </c>
+      <c r="M35">
+        <v>16.74</v>
+      </c>
+      <c r="N35">
+        <v>0.02119446315351226</v>
+      </c>
+      <c r="O35">
+        <v>64.68005467522784</v>
+      </c>
+      <c r="P35">
+        <v>79.05038585156532</v>
+      </c>
+      <c r="Q35">
+        <v>-667.7676644761668</v>
+      </c>
+      <c r="R35">
+        <v>0.1103518328320733</v>
+      </c>
+    </row>
+    <row r="36" spans="1:18">
+      <c r="A36" t="s">
+        <v>18</v>
+      </c>
+      <c r="B36">
+        <v>83.56925200000001</v>
+      </c>
+      <c r="C36">
+        <v>52.269249</v>
+      </c>
+      <c r="D36">
+        <v>376.9946473224998</v>
+      </c>
+      <c r="E36">
+        <v>-1014.87803282115</v>
+      </c>
+      <c r="F36">
+        <v>10.69534498492492</v>
+      </c>
+      <c r="G36">
+        <v>130.5672222222223</v>
+      </c>
+      <c r="H36">
+        <v>66.33505529783811</v>
+      </c>
+      <c r="I36">
+        <v>80.68209917803101</v>
+      </c>
+      <c r="J36">
+        <v>47.37262993827216</v>
+      </c>
+      <c r="K36">
+        <v>-456.5694444916228</v>
+      </c>
+      <c r="L36">
+        <v>0.04060856892151829</v>
+      </c>
+      <c r="M36">
+        <v>45.769249</v>
+      </c>
+      <c r="N36">
+        <v>7.839075955325459</v>
+      </c>
+      <c r="O36">
+        <v>66.4423881870334</v>
+      </c>
+      <c r="P36">
+        <v>80.82702057046387</v>
+      </c>
+      <c r="Q36">
+        <v>-457.3081929162009</v>
+      </c>
+      <c r="R36">
+        <v>0.09538743813557457</v>
+      </c>
+    </row>
+    <row r="37" spans="1:18">
+      <c r="A37" t="s">
+        <v>18</v>
+      </c>
+      <c r="B37">
+        <v>93.11</v>
+      </c>
+      <c r="C37">
+        <v>58.51</v>
+      </c>
+      <c r="D37">
+        <v>97.52751486240402</v>
+      </c>
+      <c r="E37">
+        <v>-577.82147302</v>
+      </c>
+      <c r="F37">
+        <v>20.57141196608997</v>
+      </c>
+      <c r="G37">
+        <v>134.0086111111112</v>
+      </c>
+      <c r="H37">
+        <v>68.12168626093077</v>
+      </c>
+      <c r="I37">
+        <v>82.48487499000345</v>
+      </c>
+      <c r="J37">
+        <v>11.84315748456814</v>
+      </c>
+      <c r="K37">
+        <v>-234.4332141907444</v>
+      </c>
+      <c r="L37">
+        <v>0.04099379117632389</v>
+      </c>
+      <c r="M37">
+        <v>52.01</v>
+      </c>
+      <c r="N37">
+        <v>17.09780944683915</v>
+      </c>
+      <c r="O37">
+        <v>68.20377872861653</v>
+      </c>
+      <c r="P37">
+        <v>82.60459825958489</v>
+      </c>
+      <c r="Q37">
+        <v>-234.7157262968996</v>
+      </c>
+      <c r="R37">
+        <v>0.08097536271248905</v>
+      </c>
+    </row>
+    <row r="38" spans="1:18">
+      <c r="A38" t="s">
+        <v>18</v>
+      </c>
+      <c r="B38">
+        <v>132</v>
+      </c>
+      <c r="C38">
+        <v>61</v>
+      </c>
+      <c r="D38">
+        <v>841.835291302404</v>
+      </c>
+      <c r="E38">
+        <v>1769.878278</v>
+      </c>
+      <c r="F38">
+        <v>175.7156714243275</v>
+      </c>
+      <c r="G38">
+        <v>137.4500000000001</v>
+      </c>
+      <c r="H38">
+        <v>69.90737988541267</v>
+      </c>
+      <c r="I38">
+        <v>84.28858814058663</v>
+      </c>
+      <c r="J38">
+        <v>8.077935669463161E-28</v>
+      </c>
+      <c r="K38">
+        <v>-1.986887238144069E-12</v>
+      </c>
+      <c r="L38">
+        <v>0.04100035850007877</v>
+      </c>
+      <c r="M38">
+        <v>54.5</v>
+      </c>
+      <c r="N38">
+        <v>178.7945042046773</v>
+      </c>
+      <c r="O38">
+        <v>69.96422947581082</v>
+      </c>
+      <c r="P38">
+        <v>84.38311574309473</v>
+      </c>
+      <c r="Q38">
+        <v>-1.988503000683603E-12</v>
+      </c>
+      <c r="R38">
+        <v>0.06725466450822415</v>
+      </c>
+    </row>
+    <row r="39" spans="1:18">
+      <c r="A39" t="s">
+        <v>18</v>
+      </c>
+      <c r="B39">
+        <v>143</v>
+      </c>
+      <c r="C39">
+        <v>89</v>
+      </c>
+      <c r="D39">
+        <v>1601.152047302404</v>
+      </c>
+      <c r="E39">
+        <v>3561.281422</v>
+      </c>
+      <c r="F39">
+        <v>81.13794251459477</v>
+      </c>
+      <c r="G39">
+        <v>140.891388888889</v>
+      </c>
+      <c r="H39">
+        <v>71.6921396898481</v>
+      </c>
+      <c r="I39">
+        <v>86.09323511121629</v>
+      </c>
+      <c r="J39">
+        <v>11.84315748456775</v>
+      </c>
+      <c r="K39">
+        <v>246.7205329493118</v>
+      </c>
+      <c r="L39">
+        <v>0.04062959813196867</v>
+      </c>
+      <c r="M39">
+        <v>82.5</v>
+      </c>
+      <c r="N39">
+        <v>80.50832717061252</v>
+      </c>
+      <c r="O39">
+        <v>71.72374395639908</v>
+      </c>
+      <c r="P39">
+        <v>86.16256949321063</v>
+      </c>
+      <c r="Q39">
+        <v>246.8292955210618</v>
+      </c>
+      <c r="R39">
+        <v>0.05436923591181075</v>
+      </c>
+    </row>
+    <row r="40" spans="1:18">
+      <c r="A40" t="s">
+        <v>18</v>
+      </c>
+      <c r="B40">
+        <v>183</v>
+      </c>
+      <c r="C40">
+        <v>82.7</v>
+      </c>
+      <c r="D40">
+        <v>6402.303887302404</v>
+      </c>
+      <c r="E40">
+        <v>6617.1907146</v>
+      </c>
+      <c r="F40">
+        <v>329.5154919450508</v>
+      </c>
+      <c r="G40">
+        <v>144.3327777777779</v>
+      </c>
+      <c r="H40">
+        <v>73.47596953707401</v>
+      </c>
+      <c r="I40">
+        <v>87.89881203905549</v>
+      </c>
+      <c r="J40">
+        <v>47.37262993827138</v>
+      </c>
+      <c r="K40">
+        <v>505.7187703304487</v>
+      </c>
+      <c r="L40">
+        <v>0.03988819428520194</v>
+      </c>
+      <c r="M40">
+        <v>76.2</v>
+      </c>
+      <c r="N40">
+        <v>320.2113238857289</v>
+      </c>
+      <c r="O40">
+        <v>73.48232604333863</v>
+      </c>
+      <c r="P40">
+        <v>87.94295563697521</v>
+      </c>
+      <c r="Q40">
+        <v>505.7625207505112</v>
+      </c>
+      <c r="R40">
+        <v>0.04246764600772128</v>
+      </c>
+    </row>
+    <row r="41" spans="1:18">
+      <c r="A41" t="s">
+        <v>18</v>
+      </c>
+      <c r="B41">
+        <v>74.78</v>
+      </c>
+      <c r="C41">
+        <v>47.28</v>
+      </c>
+      <c r="D41">
+        <v>795.5559841824039</v>
+      </c>
+      <c r="E41">
+        <v>-1333.56086256</v>
+      </c>
+      <c r="F41">
+        <v>8.206898458902371</v>
+      </c>
+      <c r="G41">
+        <v>147.7741666666668</v>
+      </c>
+      <c r="H41">
+        <v>75.2588736268476</v>
+      </c>
+      <c r="I41">
+        <v>89.70531472434699</v>
+      </c>
+      <c r="J41">
+        <v>106.5884173611109</v>
+      </c>
+      <c r="K41">
+        <v>776.9851544691783</v>
+      </c>
+      <c r="L41">
+        <v>0.03878811011056933</v>
+      </c>
+      <c r="M41">
+        <v>40.78</v>
+      </c>
+      <c r="N41">
+        <v>5.428061343089738</v>
+      </c>
+      <c r="O41">
+        <v>75.23997994738986</v>
+      </c>
+      <c r="P41">
+        <v>89.72426996362813</v>
+      </c>
+      <c r="Q41">
+        <v>776.79009297351</v>
+      </c>
+      <c r="R41">
+        <v>0.03170297528402215</v>
+      </c>
+    </row>
+    <row r="42" spans="1:18">
+      <c r="A42" t="s">
+        <v>18</v>
+      </c>
+      <c r="B42">
+        <v>260.6</v>
+      </c>
+      <c r="C42">
+        <v>146.5</v>
+      </c>
+      <c r="D42">
+        <v>24842.29845690241</v>
+      </c>
+      <c r="E42">
+        <v>23090.509307</v>
+      </c>
+      <c r="F42">
+        <v>26.81798225748312</v>
+      </c>
+      <c r="G42">
+        <v>151.2155555555557</v>
+      </c>
+      <c r="H42">
+        <v>77.04085648793065</v>
+      </c>
+      <c r="I42">
+        <v>91.51273863832901</v>
+      </c>
+      <c r="J42">
+        <v>189.4905197530863</v>
+      </c>
+      <c r="K42">
+        <v>1060.510190032192</v>
+      </c>
+      <c r="L42">
+        <v>0.03734650049081102</v>
+      </c>
+      <c r="M42">
+        <v>140</v>
+      </c>
+      <c r="N42">
+        <v>36.06471451148824</v>
+      </c>
+      <c r="O42">
+        <v>76.99671020917964</v>
+      </c>
+      <c r="P42">
+        <v>91.50650793254249</v>
+      </c>
+      <c r="Q42">
+        <v>1059.902491979474</v>
+      </c>
+      <c r="R42">
+        <v>0.02223264340662332</v>
+      </c>
+    </row>
+    <row r="43" spans="1:18">
+      <c r="A43" t="s">
+        <v>18</v>
+      </c>
+      <c r="B43">
+        <v>220.2</v>
+      </c>
+      <c r="C43">
+        <v>131.2</v>
+      </c>
+      <c r="D43">
+        <v>13739.2150985024</v>
+      </c>
+      <c r="E43">
+        <v>15378.5290176</v>
+      </c>
+      <c r="F43">
+        <v>119.8462706976806</v>
+      </c>
+      <c r="G43">
+        <v>154.6569444444446</v>
+      </c>
+      <c r="H43">
+        <v>78.82192296964406</v>
+      </c>
+      <c r="I43">
+        <v>93.3210789316807</v>
+      </c>
+      <c r="J43">
+        <v>296.0789371141976</v>
+      </c>
+      <c r="K43">
+        <v>1356.284449542945</v>
+      </c>
+      <c r="L43">
+        <v>0.03558561609923037</v>
+      </c>
+      <c r="M43">
+        <v>124.7</v>
+      </c>
+      <c r="N43">
+        <v>131.7480232725451</v>
+      </c>
+      <c r="O43">
+        <v>78.75252169073386</v>
+      </c>
+      <c r="P43">
+        <v>93.28966468169241</v>
+      </c>
+      <c r="Q43">
+        <v>1355.090265592364</v>
+      </c>
+      <c r="R43">
+        <v>0.01421823069025201</v>
+      </c>
+    </row>
+    <row r="44" spans="1:18">
+      <c r="A44" t="s">
+        <v>18</v>
+      </c>
+      <c r="B44">
+        <v>224</v>
+      </c>
+      <c r="C44">
+        <v>127</v>
+      </c>
+      <c r="D44">
+        <v>14644.4845233024</v>
+      </c>
+      <c r="E44">
+        <v>15368.828546</v>
+      </c>
+      <c r="F44">
+        <v>22.71200210221842</v>
+      </c>
+      <c r="G44">
+        <v>158.0983333333335</v>
+      </c>
+      <c r="H44">
+        <v>80.60207823292855</v>
+      </c>
+      <c r="I44">
+        <v>95.13033044346132</v>
+      </c>
+      <c r="J44">
+        <v>426.3536694444447</v>
+      </c>
+      <c r="K44">
+        <v>1664.29857871292</v>
+      </c>
+      <c r="L44">
+        <v>0.03353269918664008</v>
+      </c>
+      <c r="M44">
+        <v>120.5</v>
+      </c>
+      <c r="N44">
+        <v>28.34796135192731</v>
+      </c>
+      <c r="O44">
+        <v>80.5074195665146</v>
+      </c>
+      <c r="P44">
+        <v>95.07373503661582</v>
+      </c>
+      <c r="Q44">
+        <v>1662.344035015916</v>
+      </c>
+      <c r="R44">
+        <v>0.007825293913520466</v>
+      </c>
+    </row>
+    <row r="45" spans="1:18">
+      <c r="A45" t="s">
+        <v>18</v>
+      </c>
+      <c r="B45">
+        <v>200.9</v>
+      </c>
+      <c r="C45">
+        <v>98.86</v>
+      </c>
+      <c r="D45">
+        <v>9587.229335702405</v>
+      </c>
+      <c r="E45">
+        <v>9679.817386280001</v>
+      </c>
+      <c r="F45">
+        <v>128.3125016848963</v>
+      </c>
+      <c r="G45">
+        <v>161.5397222222224</v>
+      </c>
+      <c r="H45">
+        <v>82.38132774094845</v>
+      </c>
+      <c r="I45">
+        <v>96.94048771050652</v>
+      </c>
+      <c r="J45">
+        <v>580.3147167438278</v>
+      </c>
+      <c r="K45">
+        <v>1984.543301577299</v>
+      </c>
+      <c r="L45">
+        <v>0.0312198715871578</v>
+      </c>
+      <c r="M45">
+        <v>92.36</v>
+      </c>
+      <c r="N45">
+        <v>119.644734476178</v>
+      </c>
+      <c r="O45">
+        <v>82.26140931399942</v>
+      </c>
+      <c r="P45">
+        <v>96.85871351983513</v>
+      </c>
+      <c r="Q45">
+        <v>1981.654499982771</v>
+      </c>
+      <c r="R45">
+        <v>0.003223177137289242</v>
+      </c>
+    </row>
+    <row r="46" spans="1:18">
+      <c r="A46" t="s">
+        <v>18</v>
+      </c>
+      <c r="B46">
+        <v>174.9</v>
+      </c>
+      <c r="C46">
+        <v>110.1</v>
+      </c>
+      <c r="D46">
+        <v>5171.680639702405</v>
+      </c>
+      <c r="E46">
+        <v>7917.7752198</v>
+      </c>
+      <c r="F46">
+        <v>181.4849046441677</v>
+      </c>
+      <c r="G46">
+        <v>164.9811111111113</v>
+      </c>
+      <c r="H46">
+        <v>84.159677249277</v>
+      </c>
+      <c r="I46">
+        <v>98.75154497724307</v>
+      </c>
+      <c r="J46">
+        <v>757.9620790123467</v>
+      </c>
+      <c r="K46">
+        <v>2317.009425425097</v>
+      </c>
+      <c r="L46">
+        <v>0.02868401545673308</v>
+      </c>
+      <c r="M46">
+        <v>103.6</v>
+      </c>
+      <c r="N46">
+        <v>186.8794742564436</v>
+      </c>
+      <c r="O46">
+        <v>84.01449670384085</v>
+      </c>
+      <c r="P46">
+        <v>98.64459436069785</v>
+      </c>
+      <c r="Q46">
+        <v>2313.012443697522</v>
+      </c>
+      <c r="R46">
+        <v>0.0005848181935182172</v>
+      </c>
+    </row>
+    <row r="47" spans="1:18">
+      <c r="A47" t="s">
+        <v>18</v>
+      </c>
+      <c r="B47">
+        <v>173.5</v>
+      </c>
+      <c r="C47">
+        <v>94.16</v>
+      </c>
+      <c r="D47">
+        <v>4972.280325302404</v>
+      </c>
+      <c r="E47">
+        <v>6639.63571568</v>
+      </c>
+      <c r="F47">
+        <v>3.021544019964498</v>
+      </c>
+      <c r="G47">
+        <v>168.4225000000002</v>
+      </c>
+      <c r="H47">
+        <v>85.93713279570214</v>
+      </c>
+      <c r="I47">
+        <v>100.563496205883</v>
+      </c>
+      <c r="J47">
+        <v>959.2957562500015</v>
+      </c>
+      <c r="K47">
+        <v>2661.687845514887</v>
+      </c>
+      <c r="L47">
+        <v>0.02596664727728694</v>
+      </c>
+      <c r="M47">
+        <v>87.66</v>
+      </c>
+      <c r="N47">
+        <v>2.401771521175263</v>
+      </c>
+      <c r="O47">
+        <v>85.76668778964554</v>
+      </c>
+      <c r="P47">
+        <v>100.4313715055973</v>
+      </c>
+      <c r="Q47">
+        <v>2656.408737564799</v>
+      </c>
+      <c r="R47">
+        <v>8.655151522198734E-05</v>
+      </c>
+    </row>
+    <row r="48" spans="1:18">
+      <c r="A48" t="s">
+        <v>18</v>
+      </c>
+      <c r="B48">
+        <v>237.1</v>
+      </c>
+      <c r="C48">
+        <v>148.6</v>
+      </c>
+      <c r="D48">
+        <v>17986.6717509024</v>
+      </c>
+      <c r="E48">
+        <v>19929.3995428</v>
+      </c>
+      <c r="F48">
+        <v>381.5767044887225</v>
+      </c>
+      <c r="G48">
+        <v>171.8638888888891</v>
+      </c>
+      <c r="H48">
+        <v>87.71370068969291</v>
+      </c>
+      <c r="I48">
+        <v>102.3763350869573</v>
+      </c>
+      <c r="J48">
+        <v>1184.315748456792</v>
+      </c>
+      <c r="K48">
+        <v>3018.569549568351</v>
+      </c>
+      <c r="L48">
+        <v>0.02311378567480634</v>
+      </c>
+      <c r="M48">
+        <v>142.1</v>
+      </c>
+      <c r="N48">
+        <v>407.5778527333748</v>
+      </c>
+      <c r="O48">
+        <v>87.51798889741299</v>
+      </c>
+      <c r="P48">
+        <v>102.219038628534</v>
+      </c>
+      <c r="Q48">
+        <v>3011.834345694585</v>
+      </c>
+      <c r="R48">
+        <v>0.00190790797751309</v>
+      </c>
+    </row>
+    <row r="49" spans="1:18">
+      <c r="A49" t="s">
+        <v>18</v>
+      </c>
+      <c r="B49">
+        <v>134.8</v>
+      </c>
+      <c r="C49">
+        <v>79.67</v>
+      </c>
+      <c r="D49">
+        <v>1012.155920102405</v>
+      </c>
+      <c r="E49">
+        <v>2534.653088660001</v>
+      </c>
+      <c r="F49">
+        <v>15.63416092416712</v>
+      </c>
+      <c r="G49">
+        <v>175.3052777777779</v>
+      </c>
+      <c r="H49">
+        <v>89.48938750156638</v>
+      </c>
+      <c r="I49">
+        <v>104.190055050149</v>
+      </c>
+      <c r="J49">
+        <v>1433.022055632719</v>
+      </c>
+      <c r="K49">
+        <v>3387.645622034994</v>
+      </c>
+      <c r="L49">
+        <v>0.02017581361137463</v>
+      </c>
+      <c r="M49">
+        <v>73.17</v>
+      </c>
+      <c r="N49">
+        <v>14.89108827990491</v>
+      </c>
+      <c r="O49">
+        <v>89.26840661467412</v>
+      </c>
+      <c r="P49">
+        <v>104.007589141977</v>
+      </c>
+      <c r="Q49">
+        <v>3379.280329178107</v>
+      </c>
+      <c r="R49">
+        <v>0.006231412415090595</v>
+      </c>
+    </row>
+    <row r="50" spans="1:18">
+      <c r="A50" t="s">
+        <v>18</v>
+      </c>
+      <c r="B50">
+        <v>123.91</v>
+      </c>
+      <c r="C50">
+        <v>87.45</v>
+      </c>
+      <c r="D50">
+        <v>437.8304316624038</v>
+      </c>
+      <c r="E50">
+        <v>1829.8386051</v>
+      </c>
+      <c r="F50">
+        <v>303.2195713035505</v>
+      </c>
+      <c r="G50">
+        <v>178.7466666666668</v>
+      </c>
+      <c r="H50">
+        <v>91.26420005139568</v>
+      </c>
+      <c r="I50">
+        <v>106.0046492753848</v>
+      </c>
+      <c r="J50">
+        <v>1705.414677777781</v>
+      </c>
+      <c r="K50">
+        <v>3768.907248122474</v>
+      </c>
+      <c r="L50">
+        <v>0.01720733551884646</v>
+      </c>
+      <c r="M50">
+        <v>80.95</v>
+      </c>
+      <c r="N50">
+        <v>297.158583545951</v>
+      </c>
+      <c r="O50">
+        <v>91.01794777937036</v>
+      </c>
+      <c r="P50">
+        <v>105.7970162079849</v>
+      </c>
+      <c r="Q50">
+        <v>3758.737850128735</v>
+      </c>
+      <c r="R50">
+        <v>0.01324237947292302</v>
+      </c>
+    </row>
+    <row r="51" spans="1:18">
+      <c r="A51" t="s">
+        <v>18</v>
+      </c>
+      <c r="B51">
+        <v>126.69</v>
+      </c>
+      <c r="C51">
+        <v>75.53</v>
+      </c>
+      <c r="D51">
+        <v>561.8984845424039</v>
+      </c>
+      <c r="E51">
+        <v>1790.39318094</v>
+      </c>
+      <c r="F51">
+        <v>16.34921011511307</v>
+      </c>
+      <c r="G51">
+        <v>182.1880555555557</v>
+      </c>
+      <c r="H51">
+        <v>93.03814539769937</v>
+      </c>
+      <c r="I51">
+        <v>107.8201107041461</v>
+      </c>
+      <c r="J51">
+        <v>2001.49361489198</v>
+      </c>
+      <c r="K51">
+        <v>4162.345717588134</v>
+      </c>
+      <c r="L51">
+        <v>0.014267029945998</v>
+      </c>
+      <c r="M51">
+        <v>69.03</v>
+      </c>
+      <c r="N51">
+        <v>15.12335150203694</v>
+      </c>
+      <c r="O51">
+        <v>92.76661946851321</v>
+      </c>
+      <c r="P51">
+        <v>107.5873127495462</v>
+      </c>
+      <c r="Q51">
+        <v>4150.198175483431</v>
+      </c>
+      <c r="R51">
+        <v>0.02312870843487621</v>
+      </c>
+    </row>
+    <row r="52" spans="1:18">
+      <c r="A52" t="s">
+        <v>18</v>
+      </c>
+      <c r="B52">
+        <v>96.26000000000001</v>
+      </c>
+      <c r="C52">
+        <v>59.43</v>
+      </c>
+      <c r="D52">
+        <v>45.23372226240393</v>
+      </c>
+      <c r="E52">
+        <v>-399.7025268599997</v>
+      </c>
+      <c r="F52">
+        <v>14.53766787545371</v>
+      </c>
+      <c r="G52">
+        <v>185.6294444444446</v>
+      </c>
+      <c r="H52">
+        <v>94.81123082595202</v>
+      </c>
+      <c r="I52">
+        <v>109.6364320509586</v>
+      </c>
+      <c r="J52">
+        <v>2321.258866975314</v>
+      </c>
+      <c r="K52">
+        <v>4567.952428288359</v>
+      </c>
+      <c r="L52">
+        <v>0.01141749829159993</v>
+      </c>
+      <c r="M52">
+        <v>52.93</v>
+      </c>
+      <c r="N52">
+        <v>11.80122558751293</v>
+      </c>
+      <c r="O52">
+        <v>94.51442898666477</v>
+      </c>
+      <c r="P52">
+        <v>109.3784714620988</v>
+      </c>
+      <c r="Q52">
+        <v>4553.65268056141</v>
+      </c>
+      <c r="R52">
+        <v>0.03608067765929159</v>
+      </c>
+    </row>
+    <row r="53" spans="1:18">
+      <c r="A53" t="s">
+        <v>18</v>
+      </c>
+      <c r="B53">
+        <v>37.22</v>
+      </c>
+      <c r="C53">
+        <v>26.37</v>
+      </c>
+      <c r="D53">
+        <v>4325.114406422404</v>
+      </c>
+      <c r="E53">
+        <v>-1734.23892474</v>
+      </c>
+      <c r="F53">
+        <v>2.379357915013926</v>
+      </c>
+      <c r="G53">
+        <v>189.0708333333335</v>
+      </c>
+      <c r="H53">
+        <v>96.5834638369552</v>
+      </c>
+      <c r="I53">
+        <v>111.4536058150205</v>
+      </c>
+      <c r="J53">
+        <v>2664.710434027784</v>
+      </c>
+      <c r="K53">
+        <v>4985.718889483498</v>
+      </c>
+      <c r="L53">
+        <v>0.008725110192818677</v>
+      </c>
+      <c r="M53">
+        <v>19.87</v>
+      </c>
+      <c r="N53">
+        <v>0.5362928112458372</v>
+      </c>
+      <c r="O53">
+        <v>96.26138385427832</v>
+      </c>
+      <c r="P53">
+        <v>111.1704848251893</v>
+      </c>
+      <c r="Q53">
+        <v>4969.092852377731</v>
+      </c>
+      <c r="R53">
+        <v>0.05229073923204709</v>
+      </c>
+    </row>
+    <row r="54" spans="1:18">
+      <c r="A54" t="s">
+        <v>18</v>
+      </c>
+      <c r="B54">
+        <v>129.92</v>
+      </c>
+      <c r="C54">
+        <v>70.22</v>
+      </c>
+      <c r="D54">
+        <v>725.4617956224033</v>
+      </c>
+      <c r="E54">
+        <v>1891.333427559999</v>
+      </c>
+      <c r="F54">
+        <v>8.708679932506529</v>
+      </c>
+      <c r="G54">
+        <v>192.5122222222224</v>
+      </c>
+      <c r="H54">
+        <v>98.35485213510761</v>
+      </c>
+      <c r="I54">
+        <v>113.2716242919332</v>
+      </c>
+      <c r="J54">
+        <v>3031.84831604939</v>
+      </c>
+      <c r="K54">
+        <v>5415.636724897109</v>
+      </c>
+      <c r="L54">
+        <v>0.006259846132464981</v>
+      </c>
+      <c r="M54">
+        <v>63.72</v>
+      </c>
+      <c r="N54">
+        <v>9.498214806165647</v>
+      </c>
+      <c r="O54">
+        <v>98.00749179593768</v>
+      </c>
+      <c r="P54">
+        <v>112.9633451142341</v>
+      </c>
+      <c r="Q54">
+        <v>5396.510292710548</v>
+      </c>
+      <c r="R54">
+        <v>0.07195331442598557</v>
+      </c>
+    </row>
+    <row r="55" spans="1:18">
+      <c r="A55" t="s">
+        <v>18</v>
+      </c>
+      <c r="B55">
+        <v>75.87</v>
+      </c>
+      <c r="C55">
+        <v>41.98</v>
+      </c>
+      <c r="D55">
+        <v>735.2558718224037</v>
+      </c>
+      <c r="E55">
+        <v>-1138.31297196</v>
+      </c>
+      <c r="F55">
+        <v>9.022048855405597</v>
+      </c>
+      <c r="G55">
+        <v>195.9536111111113</v>
+      </c>
+      <c r="H55">
+        <v>100.1254036166118</v>
+      </c>
+      <c r="I55">
+        <v>115.0904795854941</v>
+      </c>
+      <c r="J55">
+        <v>3422.672513040132</v>
+      </c>
+      <c r="K55">
+        <v>5857.697675529301</v>
+      </c>
+      <c r="L55">
+        <v>0.004095137819228067</v>
+      </c>
+      <c r="M55">
+        <v>35.48</v>
+      </c>
+      <c r="N55">
+        <v>12.46537118025513</v>
+      </c>
+      <c r="O55">
+        <v>99.75276072853308</v>
+      </c>
+      <c r="P55">
+        <v>114.7570444123429</v>
+      </c>
+      <c r="Q55">
+        <v>5835.896720921823</v>
+      </c>
+      <c r="R55">
+        <v>0.09526459053144277</v>
+      </c>
+    </row>
+    <row r="56" spans="1:18">
+      <c r="A56" t="s">
+        <v>18</v>
+      </c>
+      <c r="B56">
+        <v>49.65</v>
+      </c>
+      <c r="C56">
+        <v>25.38</v>
+      </c>
+      <c r="D56">
+        <v>2844.686440702404</v>
+      </c>
+      <c r="E56">
+        <v>-1353.65757876</v>
+      </c>
+      <c r="F56">
+        <v>35.16249454112818</v>
+      </c>
+      <c r="G56">
+        <v>199.3950000000002</v>
+      </c>
+      <c r="H56">
+        <v>101.895126357654</v>
+      </c>
+      <c r="I56">
+        <v>116.910163619517</v>
+      </c>
+      <c r="J56">
+        <v>3837.18302500001</v>
+      </c>
+      <c r="K56">
+        <v>6311.893602224884</v>
+      </c>
+      <c r="L56">
+        <v>0.002307706883123237</v>
+      </c>
+      <c r="M56">
+        <v>18.88</v>
+      </c>
+      <c r="N56">
+        <v>44.20792345883999</v>
+      </c>
+      <c r="O56">
+        <v>101.4971987494099</v>
+      </c>
+      <c r="P56">
+        <v>116.5515746221702</v>
+      </c>
+      <c r="Q56">
+        <v>6287.243976532202</v>
+      </c>
+      <c r="R56">
+        <v>0.1224223195965372</v>
+      </c>
+    </row>
+    <row r="57" spans="1:18">
+      <c r="A57" t="s">
+        <v>18</v>
+      </c>
+      <c r="B57">
+        <v>118.68</v>
+      </c>
+      <c r="C57">
+        <v>63.92</v>
+      </c>
+      <c r="D57">
+        <v>246.3141285824042</v>
+      </c>
+      <c r="E57">
+        <v>1003.18592016</v>
+      </c>
+      <c r="F57">
+        <v>11.48752352321349</v>
+      </c>
+      <c r="G57">
+        <v>202.8363888888891</v>
+      </c>
+      <c r="H57">
+        <v>103.664028602592</v>
+      </c>
+      <c r="I57">
+        <v>118.7306681496441</v>
+      </c>
+      <c r="J57">
+        <v>4275.379851929023</v>
+      </c>
+      <c r="K57">
+        <v>6778.216487997989</v>
+      </c>
+      <c r="L57">
+        <v>0.0009774024137662752</v>
+      </c>
+      <c r="M57">
+        <v>57.42</v>
+      </c>
+      <c r="N57">
+        <v>12.97846965383376</v>
+      </c>
+      <c r="O57">
+        <v>103.2408141245257</v>
+      </c>
+      <c r="P57">
+        <v>118.3469274777586</v>
+      </c>
+      <c r="Q57">
+        <v>6750.544021551738</v>
+      </c>
+      <c r="R57">
+        <v>0.1536256195869764</v>
+      </c>
+    </row>
+    <row r="58" spans="1:18">
+      <c r="A58" t="s">
+        <v>18</v>
+      </c>
+      <c r="B58">
+        <v>118.24</v>
+      </c>
+      <c r="C58">
+        <v>70.08</v>
+      </c>
+      <c r="D58">
+        <v>232.6966583424039</v>
+      </c>
+      <c r="E58">
+        <v>1069.02821184</v>
+      </c>
+      <c r="F58">
+        <v>9.000825040046241</v>
+      </c>
+      <c r="G58">
+        <v>206.277777777778</v>
+      </c>
+      <c r="H58">
+        <v>105.4321187521848</v>
+      </c>
+      <c r="I58">
+        <v>120.5519847751164</v>
+      </c>
+      <c r="J58">
+        <v>4737.262993827173</v>
+      </c>
+      <c r="K58">
+        <v>7256.658440115664</v>
+      </c>
+      <c r="L58">
+        <v>0.0001870378521160602</v>
+      </c>
+      <c r="M58">
+        <v>63.58</v>
+      </c>
+      <c r="N58">
+        <v>7.748839292103415</v>
+      </c>
+      <c r="O58">
+        <v>104.9836152766491</v>
+      </c>
+      <c r="P58">
+        <v>120.1430945563393</v>
+      </c>
+      <c r="Q58">
+        <v>7225.788942568929</v>
+      </c>
+      <c r="R58">
+        <v>0.1890747784460575</v>
+      </c>
+    </row>
+    <row r="59" spans="1:18">
+      <c r="A59" t="s">
+        <v>18</v>
+      </c>
+      <c r="B59">
+        <v>246.48</v>
+      </c>
+      <c r="C59">
+        <v>128.96</v>
+      </c>
+      <c r="D59">
+        <v>20590.6422573824</v>
+      </c>
+      <c r="E59">
+        <v>18505.03756608</v>
+      </c>
+      <c r="F59">
+        <v>24.97734081407044</v>
+      </c>
+      <c r="G59">
+        <v>209.7191666666669</v>
+      </c>
+      <c r="H59">
+        <v>107.1994053518964</v>
+      </c>
+      <c r="I59">
+        <v>122.3741049504699</v>
+      </c>
+      <c r="J59">
+        <v>5222.832450694458</v>
+      </c>
+      <c r="K59">
+        <v>7747.211691943769</v>
+      </c>
+      <c r="L59">
+        <v>2.222772726870638E-05</v>
+      </c>
+      <c r="M59">
+        <v>122.46</v>
+      </c>
+      <c r="N59">
+        <v>18.27071583063505</v>
+      </c>
+      <c r="O59">
+        <v>106.7256107736326</v>
+      </c>
+      <c r="P59">
+        <v>121.9400672900599</v>
+      </c>
+      <c r="Q59">
+        <v>7712.970952601461</v>
+      </c>
+      <c r="R59">
+        <v>0.2289710615033038</v>
+      </c>
+    </row>
+    <row r="60" spans="1:18">
+      <c r="A60" t="s">
+        <v>18</v>
+      </c>
+      <c r="B60">
+        <v>83.66</v>
+      </c>
+      <c r="C60">
+        <v>54.86</v>
+      </c>
+      <c r="D60">
+        <v>373.4788926624041</v>
+      </c>
+      <c r="E60">
+        <v>-1060.20252572</v>
+      </c>
+      <c r="F60">
+        <v>33.80026165364934</v>
+      </c>
+      <c r="G60">
+        <v>213.1605555555558</v>
+      </c>
+      <c r="H60">
+        <v>108.9658970803031</v>
+      </c>
+      <c r="I60">
+        <v>124.1970199971283</v>
+      </c>
+      <c r="J60">
+        <v>5732.08822253088</v>
+      </c>
+      <c r="K60">
+        <v>8249.868604559246</v>
+      </c>
+      <c r="L60">
+        <v>0.0005712247089502928</v>
+      </c>
+      <c r="M60">
+        <v>48.36</v>
+      </c>
+      <c r="N60">
+        <v>28.55753893450419</v>
+      </c>
+      <c r="O60">
+        <v>108.4668093167901</v>
+      </c>
+      <c r="P60">
+        <v>123.7378369776066</v>
+      </c>
+      <c r="Q60">
+        <v>8212.082392712698</v>
+      </c>
+      <c r="R60">
+        <v>0.2735165226484922</v>
+      </c>
+    </row>
+    <row r="61" spans="1:18">
+      <c r="A61" t="s">
+        <v>18</v>
+      </c>
+      <c r="B61">
+        <v>84.03</v>
+      </c>
+      <c r="C61">
+        <v>46.12</v>
+      </c>
+      <c r="D61">
+        <v>359.314847182404</v>
+      </c>
+      <c r="E61">
+        <v>-874.2323642399999</v>
+      </c>
+      <c r="F61">
+        <v>9.729145426464875</v>
+      </c>
+      <c r="G61">
+        <v>216.6019444444447</v>
+      </c>
+      <c r="H61">
+        <v>110.7316027376345</v>
+      </c>
+      <c r="I61">
+        <v>126.020721114862</v>
+      </c>
+      <c r="J61">
+        <v>6265.030309336437</v>
+      </c>
+      <c r="K61">
+        <v>8764.62166813355</v>
+      </c>
+      <c r="L61">
+        <v>0.001924757423883817</v>
+      </c>
+      <c r="M61">
+        <v>39.62</v>
+      </c>
+      <c r="N61">
+        <v>12.86169246641947</v>
+      </c>
+      <c r="O61">
+        <v>110.2072197294073</v>
+      </c>
+      <c r="P61">
+        <v>125.5363947956935</v>
+      </c>
+      <c r="Q61">
+        <v>8723.115733398739</v>
+      </c>
+      <c r="R61">
+        <v>0.322913819654708</v>
+      </c>
+    </row>
+    <row r="62" spans="1:18">
+      <c r="A62" t="s">
+        <v>18</v>
+      </c>
+      <c r="B62">
+        <v>247.59</v>
+      </c>
+      <c r="C62">
+        <v>106.61</v>
+      </c>
+      <c r="D62">
+        <v>20910.43192094241</v>
+      </c>
+      <c r="E62">
+        <v>15416.27487078</v>
+      </c>
+      <c r="F62">
+        <v>779.8952513276754</v>
+      </c>
+      <c r="G62">
+        <v>220.0433333333336</v>
+      </c>
+      <c r="H62">
+        <v>112.4965312344737</v>
+      </c>
+      <c r="I62">
+        <v>127.8451993930878</v>
+      </c>
+      <c r="J62">
+        <v>6821.65871111113</v>
+      </c>
+      <c r="K62">
+        <v>9291.463503092647</v>
+      </c>
+      <c r="L62">
+        <v>0.004175869460340174</v>
+      </c>
+      <c r="M62">
+        <v>100.11</v>
+      </c>
+      <c r="N62">
+        <v>739.5768696336004</v>
+      </c>
+      <c r="O62">
+        <v>111.9468509454125</v>
+      </c>
+      <c r="P62">
+        <v>127.3357318103924</v>
+      </c>
+      <c r="Q62">
+        <v>9246.063575751448</v>
+      </c>
+      <c r="R62">
+        <v>0.3773660340000337</v>
+      </c>
+    </row>
+    <row r="63" spans="1:18">
+      <c r="A63" t="s">
+        <v>18</v>
+      </c>
+      <c r="B63">
+        <v>261.34</v>
+      </c>
+      <c r="C63">
+        <v>139.19</v>
+      </c>
+      <c r="D63">
+        <v>25076.11536594239</v>
+      </c>
+      <c r="E63">
+        <v>22041.34865762</v>
+      </c>
+      <c r="F63">
+        <v>6.336829317251824</v>
+      </c>
+      <c r="G63">
+        <v>223.4847222222225</v>
+      </c>
+      <c r="H63">
+        <v>114.260691580642</v>
+      </c>
+      <c r="I63">
+        <v>129.6704458219847</v>
+      </c>
+      <c r="J63">
+        <v>7401.973427854959</v>
+      </c>
+      <c r="K63">
+        <v>9830.386861059555</v>
+      </c>
+      <c r="L63">
+        <v>0.007419759960310863</v>
+      </c>
+      <c r="M63">
+        <v>132.69</v>
+      </c>
+      <c r="N63">
+        <v>2.839564578521499</v>
+      </c>
+      <c r="O63">
+        <v>113.6857119982322</v>
+      </c>
+      <c r="P63">
+        <v>129.1358389882768</v>
+      </c>
+      <c r="Q63">
+        <v>9780.918652403479</v>
+      </c>
+      <c r="R63">
+        <v>0.4370764955045162</v>
+      </c>
+    </row>
+    <row r="64" spans="1:18">
+      <c r="A64" t="s">
+        <v>18</v>
+      </c>
+      <c r="B64">
+        <v>118.8</v>
+      </c>
+      <c r="C64">
+        <v>77.29000000000001</v>
+      </c>
+      <c r="D64">
+        <v>250.0951841024039</v>
+      </c>
+      <c r="E64">
+        <v>1222.29482142</v>
+      </c>
+      <c r="F64">
+        <v>98.36859649574232</v>
+      </c>
+      <c r="G64">
+        <v>226.9261111111114</v>
+      </c>
+      <c r="H64">
+        <v>116.024092874291</v>
+      </c>
+      <c r="I64">
+        <v>131.4964513034008</v>
+      </c>
+      <c r="J64">
+        <v>8005.974459567924</v>
+      </c>
+      <c r="K64">
+        <v>10381.38462558595</v>
+      </c>
+      <c r="L64">
+        <v>0.01175362617295372</v>
+      </c>
+      <c r="M64">
+        <v>70.79000000000001</v>
+      </c>
+      <c r="N64">
+        <v>94.20128034460446</v>
+      </c>
+      <c r="O64">
+        <v>115.4238120098549</v>
+      </c>
+      <c r="P64">
+        <v>130.9367072073584</v>
+      </c>
+      <c r="Q64">
+        <v>10327.67382826179</v>
+      </c>
+      <c r="R64">
+        <v>0.5022486120648427</v>
+      </c>
+    </row>
+    <row r="65" spans="1:18">
+      <c r="A65" t="s">
+        <v>18</v>
+      </c>
+      <c r="B65">
+        <v>17.52</v>
+      </c>
+      <c r="C65">
+        <v>12.62</v>
+      </c>
+      <c r="D65">
+        <v>7304.369125222404</v>
+      </c>
+      <c r="E65">
+        <v>-1078.57589724</v>
+      </c>
+      <c r="F65">
+        <v>3.739675338103519</v>
+      </c>
+      <c r="G65">
+        <v>230.3675000000003</v>
+      </c>
+      <c r="H65">
+        <v>117.7867442912234</v>
+      </c>
+      <c r="I65">
+        <v>133.3232066615334</v>
+      </c>
+      <c r="J65">
+        <v>8633.661806250024</v>
+      </c>
+      <c r="K65">
+        <v>10944.44981267977</v>
+      </c>
+      <c r="L65">
+        <v>0.01727650831659461</v>
+      </c>
+      <c r="M65">
+        <v>6.119999999999999</v>
+      </c>
+      <c r="N65">
+        <v>8.342777401026858</v>
+      </c>
+      <c r="O65">
+        <v>117.1611601801233</v>
+      </c>
+      <c r="P65">
+        <v>132.7383272677941</v>
+      </c>
+      <c r="Q65">
+        <v>10886.32210103662</v>
+      </c>
+      <c r="R65">
+        <v>0.5730857047359137</v>
+      </c>
+    </row>
+    <row r="66" spans="1:18">
+      <c r="A66" t="s">
+        <v>18</v>
+      </c>
+      <c r="B66">
+        <v>124.2</v>
+      </c>
+      <c r="C66">
+        <v>61.58</v>
+      </c>
+      <c r="D66">
+        <v>450.0506825024041</v>
+      </c>
+      <c r="E66">
+        <v>1306.38262884</v>
+      </c>
+      <c r="F66">
+        <v>74.09827592278457</v>
+      </c>
+      <c r="G66">
+        <v>233.8088888888892</v>
+      </c>
+      <c r="H66">
+        <v>119.5486550744617</v>
+      </c>
+      <c r="I66">
+        <v>135.1507026533602</v>
+      </c>
+      <c r="J66">
+        <v>9285.035467901262</v>
+      </c>
+      <c r="K66">
+        <v>11519.57557113618</v>
+      </c>
+      <c r="L66">
+        <v>0.02408913706999165</v>
+      </c>
+      <c r="M66">
+        <v>55.08</v>
+      </c>
+      <c r="N66">
+        <v>77.10285469667225</v>
+      </c>
+      <c r="O66">
+        <v>118.897765776276</v>
+      </c>
+      <c r="P66">
+        <v>134.5406899023455</v>
+      </c>
+      <c r="Q66">
+        <v>11456.85660157333</v>
+      </c>
+      <c r="R66">
+        <v>0.6497908483761072</v>
+      </c>
+    </row>
+    <row r="67" spans="1:18">
+      <c r="A67" t="s">
+        <v>18</v>
+      </c>
+      <c r="B67">
+        <v>30.49</v>
+      </c>
+      <c r="C67">
+        <v>20.29</v>
+      </c>
+      <c r="D67">
+        <v>5255.612309342405</v>
+      </c>
+      <c r="E67">
+        <v>-1470.93576458</v>
+      </c>
+      <c r="F67">
+        <v>1.056271986650776</v>
+      </c>
+      <c r="G67">
+        <v>237.2502777777781</v>
+      </c>
+      <c r="H67">
+        <v>121.3098345240806</v>
+      </c>
+      <c r="I67">
+        <v>136.9789299788065</v>
+      </c>
+      <c r="J67">
+        <v>9960.095444521634</v>
+      </c>
+      <c r="K67">
+        <v>12106.75518267951</v>
+      </c>
+      <c r="L67">
+        <v>0.03229378398647876</v>
+      </c>
+      <c r="M67">
+        <v>13.79</v>
+      </c>
+      <c r="N67">
+        <v>3.561774771645233</v>
+      </c>
+      <c r="O67">
+        <v>120.6336381227536</v>
+      </c>
+      <c r="P67">
+        <v>136.3437857865721</v>
+      </c>
+      <c r="Q67">
+        <v>12039.27059399475</v>
+      </c>
+      <c r="R67">
+        <v>0.7325667180399115</v>
+      </c>
+    </row>
+    <row r="68" spans="1:18">
+      <c r="A68" t="s">
+        <v>18</v>
+      </c>
+      <c r="B68">
+        <v>37.1</v>
+      </c>
+      <c r="C68">
+        <v>24.7</v>
+      </c>
+      <c r="D68">
+        <v>4340.912550902405</v>
+      </c>
+      <c r="E68">
+        <v>-1627.3743694</v>
+      </c>
+      <c r="F68">
+        <v>0.004212345869516114</v>
+      </c>
+      <c r="G68">
+        <v>240.6916666666669</v>
+      </c>
+      <c r="H68">
+        <v>123.0702919873202</v>
+      </c>
+      <c r="I68">
+        <v>138.8078792906319</v>
+      </c>
+      <c r="J68">
+        <v>10658.84173611114</v>
+      </c>
+      <c r="K68">
+        <v>12705.98206192427</v>
+      </c>
+      <c r="L68">
+        <v>0.04199411509794655</v>
+      </c>
+      <c r="M68">
+        <v>18.2</v>
+      </c>
+      <c r="N68">
+        <v>0.7673384469952047</v>
+      </c>
+      <c r="O68">
+        <v>122.3687865912855</v>
+      </c>
+      <c r="P68">
+        <v>138.1476055487443</v>
+      </c>
+      <c r="Q68">
+        <v>12633.55747566199</v>
+      </c>
+      <c r="R68">
+        <v>0.82161544127181</v>
+      </c>
+    </row>
+    <row r="69" spans="1:18">
+      <c r="A69" t="s">
+        <v>18</v>
+      </c>
+      <c r="B69">
+        <v>87.19</v>
+      </c>
+      <c r="C69">
+        <v>60.69</v>
+      </c>
+      <c r="D69">
+        <v>249.5010425424041</v>
+      </c>
+      <c r="E69">
+        <v>-958.6350853800001</v>
+      </c>
+      <c r="F69">
+        <v>96.09654787374522</v>
+      </c>
+      <c r="G69">
+        <v>244.1330555555558</v>
+      </c>
+      <c r="H69">
+        <v>124.8300368489928</v>
+      </c>
+      <c r="I69">
+        <v>140.6375412040244</v>
+      </c>
+      <c r="J69">
+        <v>11381.27434266979</v>
+      </c>
+      <c r="K69">
+        <v>13317.24975616317</v>
+      </c>
+      <c r="L69">
+        <v>0.05329504794891016</v>
+      </c>
+      <c r="M69">
+        <v>54.19</v>
+      </c>
+      <c r="N69">
+        <v>87.58862521047325</v>
+      </c>
+      <c r="O69">
+        <v>124.1032205912715</v>
+      </c>
+      <c r="P69">
+        <v>139.9521397794624</v>
+      </c>
+      <c r="Q69">
+        <v>13239.710776962</v>
+      </c>
+      <c r="R69">
+        <v>0.9171384564237802</v>
+      </c>
+    </row>
+    <row r="70" spans="1:18">
+      <c r="A70" t="s">
+        <v>18</v>
+      </c>
+      <c r="B70">
+        <v>100.7</v>
+      </c>
+      <c r="C70">
+        <v>49.9</v>
+      </c>
+      <c r="D70">
+        <v>5.223976502403987</v>
+      </c>
+      <c r="E70">
+        <v>-114.0515397999999</v>
+      </c>
+      <c r="F70">
+        <v>64.52355020228318</v>
+      </c>
+      <c r="G70">
+        <v>247.5744444444447</v>
+      </c>
+      <c r="H70">
+        <v>126.5890785221932</v>
+      </c>
+      <c r="I70">
+        <v>142.4679063058892</v>
+      </c>
+      <c r="J70">
+        <v>12127.39326419757</v>
+      </c>
+      <c r="K70">
+        <v>13940.5519449907</v>
+      </c>
+      <c r="L70">
+        <v>0.0663026122747362</v>
+      </c>
+      <c r="M70">
+        <v>43.4</v>
+      </c>
+      <c r="N70">
+        <v>70.18512183066606</v>
+      </c>
+      <c r="O70">
+        <v>125.8369495604684</v>
+      </c>
+      <c r="P70">
+        <v>141.7573790409697</v>
+      </c>
+      <c r="Q70">
+        <v>13857.72416093018</v>
+      </c>
+      <c r="R70">
+        <v>1.01933637709012</v>
+      </c>
+    </row>
+    <row r="71" spans="1:18">
+      <c r="A71" t="s">
+        <v>18</v>
+      </c>
+      <c r="B71">
+        <v>25.76</v>
+      </c>
+      <c r="C71">
+        <v>17.56</v>
+      </c>
+      <c r="D71">
+        <v>5963.793604262403</v>
+      </c>
+      <c r="E71">
+        <v>-1356.08157112</v>
+      </c>
+      <c r="F71">
+        <v>1.666757709440546</v>
+      </c>
+      <c r="G71">
+        <v>251.0158333333336</v>
+      </c>
+      <c r="H71">
+        <v>128.3474264393248</v>
+      </c>
+      <c r="I71">
+        <v>144.2989651638226</v>
+      </c>
+      <c r="J71">
+        <v>12897.19850069448</v>
+      </c>
+      <c r="K71">
+        <v>14575.88243977065</v>
+      </c>
+      <c r="L71">
+        <v>0.08112381451229411</v>
+      </c>
+      <c r="M71">
+        <v>11.06</v>
+      </c>
+      <c r="N71">
+        <v>4.775132948243496</v>
+      </c>
+      <c r="O71">
+        <v>127.569982955992</v>
+      </c>
+      <c r="P71">
+        <v>143.5633138761502</v>
+      </c>
+      <c r="Q71">
+        <v>14487.59142271638</v>
+      </c>
+      <c r="R71">
+        <v>1.128408862726576</v>
+      </c>
+    </row>
+    <row r="72" spans="1:18">
+      <c r="A72" t="s">
+        <v>18</v>
+      </c>
+      <c r="B72">
+        <v>83.72</v>
+      </c>
+      <c r="C72">
+        <v>48.02</v>
+      </c>
+      <c r="D72">
+        <v>371.163420422404</v>
+      </c>
+      <c r="E72">
+        <v>-925.1342080400001</v>
+      </c>
+      <c r="F72">
+        <v>1.118287401912193</v>
+      </c>
+      <c r="G72">
+        <v>254.4572222222225</v>
+      </c>
+      <c r="H72">
+        <v>130.1050900434481</v>
+      </c>
+      <c r="I72">
+        <v>146.1307083347644</v>
+      </c>
+      <c r="J72">
+        <v>13690.69005216053</v>
+      </c>
+      <c r="K72">
+        <v>15223.23518295599</v>
+      </c>
+      <c r="L72">
+        <v>0.09786650630660242</v>
+      </c>
+      <c r="M72">
+        <v>41.52</v>
+      </c>
+      <c r="N72">
+        <v>2.331500613572123</v>
+      </c>
+      <c r="O72">
+        <v>129.302330245643</v>
+      </c>
+      <c r="P72">
+        <v>145.3699348172033</v>
+      </c>
+      <c r="Q72">
+        <v>15129.30648890314</v>
+      </c>
+      <c r="R72">
+        <v>1.24455449549283</v>
+      </c>
+    </row>
+    <row r="73" spans="1:18">
+      <c r="A73" t="s">
+        <v>18</v>
+      </c>
+      <c r="B73">
+        <v>28.34</v>
+      </c>
+      <c r="C73">
+        <v>18.74</v>
+      </c>
+      <c r="D73">
+        <v>5571.965897942404</v>
+      </c>
+      <c r="E73">
+        <v>-1398.85858148</v>
+      </c>
+      <c r="F73">
+        <v>2.121433074947147</v>
+      </c>
+      <c r="G73">
+        <v>257.8986111111114</v>
+      </c>
+      <c r="H73">
+        <v>131.8620787799574</v>
+      </c>
+      <c r="I73">
+        <v>147.9631263733202</v>
+      </c>
+      <c r="J73">
+        <v>14507.86791859572</v>
+      </c>
+      <c r="K73">
+        <v>15882.6042472698</v>
+      </c>
+      <c r="L73">
+        <v>0.1166392571522363</v>
+      </c>
+      <c r="M73">
+        <v>12.24</v>
+      </c>
+      <c r="N73">
+        <v>5.437222422917766</v>
+      </c>
+      <c r="O73">
+        <v>131.0340008995622</v>
+      </c>
+      <c r="P73">
+        <v>147.1772323939882</v>
+      </c>
+      <c r="Q73">
+        <v>15782.86341668437</v>
+      </c>
+      <c r="R73">
+        <v>1.367970663333548</v>
+      </c>
+    </row>
+    <row r="74" spans="1:18">
+      <c r="A74" t="s">
+        <v>18</v>
+      </c>
+      <c r="B74">
+        <v>117</v>
+      </c>
+      <c r="C74">
+        <v>62.81</v>
+      </c>
+      <c r="D74">
+        <v>196.403351302404</v>
+      </c>
+      <c r="E74">
+        <v>880.24433838</v>
+      </c>
+      <c r="F74">
+        <v>13.12754650706101</v>
+      </c>
+      <c r="G74">
+        <v>261.3400000000003</v>
+      </c>
+      <c r="H74">
+        <v>133.6184020885921</v>
+      </c>
+      <c r="I74">
+        <v>149.7962098397506</v>
+      </c>
+      <c r="J74">
+        <v>15348.73210000003</v>
+      </c>
+      <c r="K74">
+        <v>16553.98383475569</v>
+      </c>
+      <c r="L74">
+        <v>0.1375512312857222</v>
+      </c>
+      <c r="M74">
+        <v>56.31</v>
+      </c>
+      <c r="N74">
+        <v>14.81284899857283</v>
+      </c>
+      <c r="O74">
+        <v>132.7650043822207</v>
+      </c>
+      <c r="P74">
+        <v>148.9851971420339</v>
+      </c>
+      <c r="Q74">
+        <v>16448.25639291334</v>
+      </c>
+      <c r="R74">
+        <v>1.498853449289734</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
nieuwe versie notebook Leo
</commit_message>
<xml_diff>
--- a/resultaten/c_phi_data_geforceerd.xlsx
+++ b/resultaten/c_phi_data_geforceerd.xlsx
@@ -492,55 +492,55 @@
         <v>18</v>
       </c>
       <c r="B2">
-        <v>156.55</v>
+        <v>143.8</v>
       </c>
       <c r="C2">
-        <v>98.11</v>
+        <v>85.09999999999999</v>
       </c>
       <c r="D2">
-        <v>2673.103981375613</v>
+        <v>1665.815084102405</v>
       </c>
       <c r="E2">
-        <v>5072.490029909179</v>
+        <v>3473.305269800001</v>
       </c>
       <c r="F2">
-        <v>96.30305245544122</v>
+        <v>22.00037539803776</v>
       </c>
       <c r="G2">
-        <v>14.61</v>
+        <v>13.56</v>
       </c>
       <c r="H2">
-        <v>5.058239350155489</v>
+        <v>5.030972332908122</v>
       </c>
       <c r="I2">
-        <v>21.08444946785428</v>
+        <v>19.94635179074794</v>
       </c>
       <c r="J2">
-        <v>15218.92322499998</v>
+        <v>15348.73210000003</v>
       </c>
       <c r="K2">
-        <v>-624.0096974319316</v>
+        <v>-623.2871623239879</v>
       </c>
       <c r="L2">
-        <v>0.1657600316758227</v>
+        <v>0.1517378637092041</v>
       </c>
       <c r="M2">
-        <v>90.61</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="N2">
-        <v>98.24419925566107</v>
+        <v>21.60242432161142</v>
       </c>
       <c r="O2">
-        <v>6.94593002379909</v>
+        <v>6.426991131740807</v>
       </c>
       <c r="P2">
-        <v>23.11635541150777</v>
+        <v>21.42573874909166</v>
       </c>
       <c r="Q2">
-        <v>-856.8846573859743</v>
+        <v>-796.2399313113693</v>
       </c>
       <c r="R2">
-        <v>2.192041017312654</v>
+        <v>1.013008739480786</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -548,55 +548,55 @@
         <v>18</v>
       </c>
       <c r="B3">
-        <v>121.67</v>
+        <v>110.23</v>
       </c>
       <c r="C3">
-        <v>75.73999999999999</v>
+        <v>65.8</v>
       </c>
       <c r="D3">
-        <v>282.9820192671192</v>
+        <v>52.48130238240406</v>
       </c>
       <c r="E3">
-        <v>1274.103537186027</v>
+        <v>476.6813884000002</v>
       </c>
       <c r="F3">
-        <v>35.15405365810402</v>
+        <v>8.394908899002235</v>
       </c>
       <c r="G3">
-        <v>18.03680555555555</v>
+        <v>17.00138888888889</v>
       </c>
       <c r="H3">
-        <v>6.899017112451866</v>
+        <v>6.848966125776429</v>
       </c>
       <c r="I3">
-        <v>22.87594284990325</v>
+        <v>21.71776477294472</v>
       </c>
       <c r="J3">
-        <v>14385.17048659335</v>
+        <v>14507.86791859571</v>
       </c>
       <c r="K3">
-        <v>-827.4556559088011</v>
+        <v>-824.9484573968192</v>
       </c>
       <c r="L3">
-        <v>0.1394155075261186</v>
+        <v>0.127605456976626</v>
       </c>
       <c r="M3">
-        <v>68.23999999999999</v>
+        <v>58.8</v>
       </c>
       <c r="N3">
-        <v>30.48934364130204</v>
+        <v>6.225979104654242</v>
       </c>
       <c r="O3">
-        <v>8.737238979348684</v>
+        <v>8.208252081457152</v>
       </c>
       <c r="P3">
-        <v>24.85793649080233</v>
+        <v>23.16015852892369</v>
       </c>
       <c r="Q3">
-        <v>-1047.928667612701</v>
+        <v>-988.6725628614018</v>
       </c>
       <c r="R3">
-        <v>2.145750384026431</v>
+        <v>1.004138063000265</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -604,55 +604,55 @@
         <v>18</v>
       </c>
       <c r="B4">
-        <v>233.82</v>
+        <v>218.35</v>
       </c>
       <c r="C4">
-        <v>143.77</v>
+        <v>129.55</v>
       </c>
       <c r="D4">
-        <v>16633.7946881452</v>
+        <v>13308.9443259024</v>
       </c>
       <c r="E4">
-        <v>18542.31441921356</v>
+        <v>14945.4577609</v>
       </c>
       <c r="F4">
-        <v>210.88619585934</v>
+        <v>105.3131061460526</v>
       </c>
       <c r="G4">
-        <v>21.46361111111111</v>
+        <v>20.44277777777778</v>
       </c>
       <c r="H4">
-        <v>8.738912840612334</v>
+        <v>8.66611497684951</v>
       </c>
       <c r="I4">
-        <v>24.66831826608813</v>
+        <v>23.49002269693672</v>
       </c>
       <c r="J4">
-        <v>13574.90374081789</v>
+        <v>13690.69005216052</v>
       </c>
       <c r="K4">
-        <v>-1018.182872438688</v>
+        <v>-1013.99804089956</v>
       </c>
       <c r="L4">
-        <v>0.115949359295722</v>
+        <v>0.1061115094529364</v>
       </c>
       <c r="M4">
-        <v>136.27</v>
+        <v>122.55</v>
       </c>
       <c r="N4">
-        <v>247.7724005652218</v>
+        <v>121.3997939799514</v>
       </c>
       <c r="O4">
-        <v>10.52765796359007</v>
+        <v>9.988663366652812</v>
       </c>
       <c r="P4">
-        <v>26.6004075414051</v>
+        <v>24.8954279732764</v>
       </c>
       <c r="Q4">
-        <v>-1226.59205108505</v>
+        <v>-1168.745754244917</v>
       </c>
       <c r="R4">
-        <v>2.09737519269557</v>
+        <v>0.9936117822777024</v>
       </c>
     </row>
     <row r="5" spans="1:18">
@@ -660,55 +660,55 @@
         <v>18</v>
       </c>
       <c r="B5">
-        <v>92.25</v>
+        <v>86.48</v>
       </c>
       <c r="C5">
-        <v>55.06</v>
+        <v>48.82</v>
       </c>
       <c r="D5">
-        <v>158.7078551262974</v>
+        <v>272.4348973824038</v>
       </c>
       <c r="E5">
-        <v>-693.6420582326029</v>
+        <v>-805.8034896399998</v>
       </c>
       <c r="F5">
-        <v>0.7074032008101983</v>
+        <v>2.879287678438584</v>
       </c>
       <c r="G5">
-        <v>24.89041666666666</v>
+        <v>23.88416666666667</v>
       </c>
       <c r="H5">
-        <v>10.57791861809657</v>
+        <v>10.48241118753726</v>
       </c>
       <c r="I5">
-        <v>26.46158363294924</v>
+        <v>25.26313326131406</v>
       </c>
       <c r="J5">
-        <v>12788.1229876736</v>
+        <v>12897.19850069448</v>
       </c>
       <c r="K5">
-        <v>-1196.199519461359</v>
+        <v>-1190.443761855326</v>
       </c>
       <c r="L5">
-        <v>0.09519251460971738</v>
+        <v>0.08710101599992996</v>
       </c>
       <c r="M5">
-        <v>47.56</v>
+        <v>41.82</v>
       </c>
       <c r="N5">
-        <v>5.03646173296279E-05</v>
+        <v>5.538747051658929</v>
       </c>
       <c r="O5">
-        <v>12.31717898874424</v>
+        <v>11.7682172457071</v>
       </c>
       <c r="P5">
-        <v>28.34377655109508</v>
+        <v>26.63155482377049</v>
       </c>
       <c r="Q5">
-        <v>-1392.88305378423</v>
+        <v>-1336.467398356434</v>
       </c>
       <c r="R5">
-        <v>2.04698126115088</v>
+        <v>0.9814414049796752</v>
       </c>
     </row>
     <row r="6" spans="1:18">
@@ -716,55 +716,55 @@
         <v>18</v>
       </c>
       <c r="B6">
-        <v>182.31</v>
+        <v>166.59</v>
       </c>
       <c r="C6">
-        <v>110.99</v>
+        <v>92.61</v>
       </c>
       <c r="D6">
-        <v>6000.372197428215</v>
+        <v>4045.519444942404</v>
       </c>
       <c r="E6">
-        <v>8597.515083922328</v>
+        <v>5890.40329878</v>
       </c>
       <c r="F6">
-        <v>81.74236414109349</v>
+        <v>0.0994420970070284</v>
       </c>
       <c r="G6">
-        <v>28.31722222222221</v>
+        <v>27.32555555555555</v>
       </c>
       <c r="H6">
-        <v>12.41602673516045</v>
+        <v>12.29784726319209</v>
       </c>
       <c r="I6">
-        <v>28.25574666023071</v>
+        <v>27.03710396072432</v>
       </c>
       <c r="J6">
-        <v>12024.82822716048</v>
+        <v>12127.39326419756</v>
       </c>
       <c r="K6">
-        <v>-1361.513900607172</v>
+        <v>-1354.293597721662</v>
       </c>
       <c r="L6">
-        <v>0.07697848495770271</v>
+        <v>0.07042131330167158</v>
       </c>
       <c r="M6">
-        <v>103.49</v>
+        <v>85.61</v>
       </c>
       <c r="N6">
-        <v>90.49891552568995</v>
+        <v>0.2671322893220296</v>
       </c>
       <c r="O6">
-        <v>14.1057942756893</v>
+        <v>13.54690618208179</v>
       </c>
       <c r="P6">
-        <v>30.08805129899417</v>
+        <v>28.36854661694417</v>
       </c>
       <c r="Q6">
-        <v>-1546.810054062586</v>
+        <v>-1491.845517242769</v>
       </c>
       <c r="R6">
-        <v>1.994640924581889</v>
+        <v>0.9676436059363372</v>
       </c>
     </row>
     <row r="7" spans="1:18">
@@ -772,55 +772,55 @@
         <v>18</v>
       </c>
       <c r="B7">
-        <v>39.85</v>
+        <v>35.79</v>
       </c>
       <c r="C7">
-        <v>25.77</v>
+        <v>22.39</v>
       </c>
       <c r="D7">
-        <v>4224.730980857804</v>
+        <v>4515.248928142405</v>
       </c>
       <c r="E7">
-        <v>-1674.996671279589</v>
+        <v>-1504.50952878</v>
       </c>
       <c r="F7">
-        <v>0.4597093838247798</v>
+        <v>2.861951488432676</v>
       </c>
       <c r="G7">
-        <v>31.74402777777777</v>
+        <v>30.76694444444444</v>
       </c>
       <c r="H7">
-        <v>14.25322970057299</v>
+        <v>14.11241592483642</v>
       </c>
       <c r="I7">
-        <v>30.05081483916351</v>
+        <v>28.81194207414506</v>
       </c>
       <c r="J7">
-        <v>11285.01945927854</v>
+        <v>11381.27434266978</v>
       </c>
       <c r="K7">
-        <v>-1514.134448398521</v>
+        <v>-1505.555652132433</v>
       </c>
       <c r="L7">
-        <v>0.06114356383807958</v>
+        <v>0.05592226511386782</v>
       </c>
       <c r="M7">
-        <v>18.27</v>
+        <v>15.39</v>
       </c>
       <c r="N7">
-        <v>5.161180759814882</v>
+        <v>8.35968955797278</v>
       </c>
       <c r="O7">
-        <v>15.89349626578282</v>
+        <v>15.32472285611412</v>
       </c>
       <c r="P7">
-        <v>31.8332393437448</v>
+        <v>30.10641067246021</v>
       </c>
       <c r="Q7">
-        <v>-1688.381560324366</v>
+        <v>-1634.888259832317</v>
       </c>
       <c r="R7">
-        <v>1.940433172245608</v>
+        <v>0.9522403673890971</v>
       </c>
     </row>
     <row r="8" spans="1:18">
@@ -828,55 +828,55 @@
         <v>18</v>
       </c>
       <c r="B8">
-        <v>145.4</v>
+        <v>135.5</v>
       </c>
       <c r="C8">
-        <v>87.65000000000001</v>
+        <v>76.38</v>
       </c>
       <c r="D8">
-        <v>1644.470333511229</v>
+        <v>1057.186077302404</v>
       </c>
       <c r="E8">
-        <v>3554.388883870548</v>
+        <v>2483.44971924</v>
       </c>
       <c r="F8">
-        <v>27.69579697226567</v>
+        <v>0.08937217839633568</v>
       </c>
       <c r="G8">
-        <v>35.17083333333332</v>
+        <v>34.20833333333333</v>
       </c>
       <c r="H8">
-        <v>16.08952025323313</v>
+        <v>15.9261101207881</v>
       </c>
       <c r="I8">
-        <v>31.84679543084872</v>
+        <v>30.58765465325848</v>
       </c>
       <c r="J8">
-        <v>10568.69668402777</v>
+        <v>10658.84173611114</v>
       </c>
       <c r="K8">
-        <v>-1654.069721700086</v>
+        <v>-1644.238152387033</v>
       </c>
       <c r="L8">
-        <v>0.04752702464956905</v>
+        <v>0.04345644732966312</v>
       </c>
       <c r="M8">
-        <v>80.15000000000001</v>
+        <v>69.38</v>
       </c>
       <c r="N8">
-        <v>27.03384210786232</v>
+        <v>0.02803279930913141</v>
       </c>
       <c r="O8">
-        <v>17.68027763258318</v>
+        <v>17.10166017670717</v>
       </c>
       <c r="P8">
-        <v>33.57934801178859</v>
+        <v>31.84515408141554</v>
       </c>
       <c r="Q8">
-        <v>-1817.606208453019</v>
+        <v>-1765.603899410212</v>
       </c>
       <c r="R8">
-        <v>1.884443776534967</v>
+        <v>0.9352591135872037</v>
       </c>
     </row>
     <row r="9" spans="1:18">
@@ -884,55 +884,55 @@
         <v>18</v>
       </c>
       <c r="B9">
-        <v>32.94</v>
+        <v>29.36</v>
       </c>
       <c r="C9">
-        <v>24.39</v>
+        <v>20.81</v>
       </c>
       <c r="D9">
-        <v>5170.750481598353</v>
+        <v>5420.729269862404</v>
       </c>
       <c r="E9">
-        <v>-1753.834427066713</v>
+        <v>-1532.14877762</v>
       </c>
       <c r="F9">
-        <v>2.573256674985664</v>
+        <v>0.006650456254538931</v>
       </c>
       <c r="G9">
-        <v>38.59763888888887</v>
+        <v>37.64972222222222</v>
       </c>
       <c r="H9">
-        <v>17.92489137364905</v>
+        <v>17.73892303814511</v>
       </c>
       <c r="I9">
-        <v>33.64369545477815</v>
+        <v>32.36424851096655</v>
       </c>
       <c r="J9">
-        <v>9875.859901408172</v>
+        <v>9960.095444521634</v>
       </c>
       <c r="K9">
-        <v>-1781.328402916561</v>
+        <v>-1770.349446685506</v>
       </c>
       <c r="L9">
-        <v>0.03597131774331105</v>
+        <v>0.0328793322989577</v>
       </c>
       <c r="M9">
-        <v>16.89</v>
+        <v>13.81</v>
       </c>
       <c r="N9">
-        <v>0.008075883925641441</v>
+        <v>1.408750980453257</v>
       </c>
       <c r="O9">
-        <v>19.46613129343216</v>
+        <v>18.87771129287886</v>
       </c>
       <c r="P9">
-        <v>35.32638438578376</v>
+        <v>33.58478369479222</v>
       </c>
       <c r="Q9">
-        <v>-1934.492758983707</v>
+        <v>-1884.000830838005</v>
       </c>
       <c r="R9">
-        <v>1.826765413763743</v>
+        <v>0.9167328391288382</v>
       </c>
     </row>
     <row r="10" spans="1:18">
@@ -940,55 +940,55 @@
         <v>18</v>
       </c>
       <c r="B10">
-        <v>48.49</v>
+        <v>42.79</v>
       </c>
       <c r="C10">
-        <v>39.72</v>
+        <v>36.42</v>
       </c>
       <c r="D10">
-        <v>3176.216340279174</v>
+        <v>3623.510500142404</v>
       </c>
       <c r="E10">
-        <v>-2238.537002996712</v>
+        <v>-2192.32382484</v>
       </c>
       <c r="F10">
-        <v>75.56757497117069</v>
+        <v>75.47666753534391</v>
       </c>
       <c r="G10">
-        <v>42.02444444444443</v>
+        <v>41.0911111111111</v>
       </c>
       <c r="H10">
-        <v>19.7593362952418</v>
+        <v>19.55084811409046</v>
       </c>
       <c r="I10">
-        <v>35.44152167753074</v>
+        <v>34.14173021008629</v>
       </c>
       <c r="J10">
-        <v>9206.509111419744</v>
+        <v>9285.035467901262</v>
       </c>
       <c r="K10">
-        <v>-1895.919294937503</v>
+        <v>-1883.898001109188</v>
       </c>
       <c r="L10">
-        <v>0.02632226603197113</v>
+        <v>0.02404947182152869</v>
       </c>
       <c r="M10">
-        <v>32.22</v>
+        <v>29.42</v>
       </c>
       <c r="N10">
-        <v>52.19255430056087</v>
+        <v>57.20093695815025</v>
       </c>
       <c r="O10">
-        <v>21.25105042086031</v>
+        <v>20.65286960512991</v>
       </c>
       <c r="P10">
-        <v>37.07435529319976</v>
+        <v>35.32530611208955</v>
       </c>
       <c r="Q10">
-        <v>-2039.050094020668</v>
+        <v>-1990.087567517427</v>
       </c>
       <c r="R10">
-        <v>1.767497776035174</v>
+        <v>0.8967002304460866</v>
       </c>
     </row>
     <row r="11" spans="1:18">
@@ -996,55 +996,55 @@
         <v>18</v>
       </c>
       <c r="B11">
-        <v>14.61</v>
+        <v>13.56</v>
       </c>
       <c r="C11">
-        <v>10.71</v>
+        <v>10.26</v>
       </c>
       <c r="D11">
-        <v>8142.884116992599</v>
+        <v>7996.938293062403</v>
       </c>
       <c r="E11">
-        <v>-966.4482366086303</v>
+        <v>-917.5066765199999</v>
       </c>
       <c r="F11">
-        <v>5.575947417938633</v>
+        <v>4.96693458583156</v>
       </c>
       <c r="G11">
-        <v>45.45124999999998</v>
+        <v>44.53249999999999</v>
       </c>
       <c r="H11">
-        <v>21.59284851543454</v>
+        <v>21.36187904697708</v>
       </c>
       <c r="I11">
-        <v>37.24028060168335</v>
+        <v>35.92010605226475</v>
       </c>
       <c r="J11">
-        <v>8560.644314062491</v>
+        <v>8633.661806250024</v>
       </c>
       <c r="K11">
-        <v>-1997.851317829935</v>
+        <v>-1984.892396347495</v>
       </c>
       <c r="L11">
-        <v>0.01842925853825314</v>
+        <v>0.01682867822056685</v>
       </c>
       <c r="M11">
-        <v>3.210000000000001</v>
+        <v>3.26</v>
       </c>
       <c r="N11">
-        <v>18.67227438632926</v>
+        <v>13.44223187631334</v>
       </c>
       <c r="O11">
-        <v>23.03502845377596</v>
+        <v>22.42712877659077</v>
       </c>
       <c r="P11">
-        <v>38.82326729512826</v>
+        <v>37.06672767017706</v>
       </c>
       <c r="Q11">
-        <v>-2131.287213900052</v>
+        <v>-2083.872738098876</v>
       </c>
       <c r="R11">
-        <v>1.706747673576038</v>
+        <v>0.8752057798419322</v>
       </c>
     </row>
     <row r="12" spans="1:18">
@@ -1052,55 +1052,55 @@
         <v>18</v>
       </c>
       <c r="B12">
-        <v>17.92</v>
+        <v>16.889999</v>
       </c>
       <c r="C12">
-        <v>12.32</v>
+        <v>11.69</v>
       </c>
       <c r="D12">
-        <v>7556.465116493147</v>
+        <v>7412.452855933609</v>
       </c>
       <c r="E12">
-        <v>-1070.952104856986</v>
+        <v>-1006.45759907</v>
       </c>
       <c r="F12">
-        <v>6.277908433446108</v>
+        <v>6.427619349279396</v>
       </c>
       <c r="G12">
-        <v>48.87805555555553</v>
+        <v>47.97388888888888</v>
       </c>
       <c r="H12">
-        <v>23.42542180648832</v>
+        <v>23.17200980715261</v>
       </c>
       <c r="I12">
-        <v>39.03997845497491</v>
+        <v>37.69938206715431</v>
       </c>
       <c r="J12">
-        <v>7938.265509336413</v>
+        <v>8005.974459567927</v>
       </c>
       <c r="K12">
-        <v>-2087.133505280366</v>
+        <v>-2073.341324172547</v>
       </c>
       <c r="L12">
-        <v>0.01214544125432737</v>
+        <v>0.01108220289252352</v>
       </c>
       <c r="M12">
-        <v>4.82</v>
+        <v>4.69</v>
       </c>
       <c r="N12">
-        <v>19.51321927612854</v>
+        <v>15.50239454079438</v>
       </c>
       <c r="O12">
-        <v>24.81805910839854</v>
+        <v>24.20048274390688</v>
       </c>
       <c r="P12">
-        <v>40.57312667534983</v>
+        <v>38.80905443240932</v>
       </c>
       <c r="Q12">
-        <v>-2211.213233599922</v>
+        <v>-2165.365082936343</v>
       </c>
       <c r="R12">
-        <v>1.644629126937563</v>
+        <v>0.8522998914991469</v>
       </c>
     </row>
     <row r="13" spans="1:18">
@@ -1108,55 +1108,55 @@
         <v>18</v>
       </c>
       <c r="B13">
-        <v>96.989998</v>
+        <v>85.550003</v>
       </c>
       <c r="C13">
-        <v>59.290001</v>
+        <v>51.25</v>
       </c>
       <c r="D13">
-        <v>61.74710457391414</v>
+        <v>304.0001124888009</v>
       </c>
       <c r="E13">
-        <v>-465.8968310621793</v>
+        <v>-893.5744487499998</v>
       </c>
       <c r="F13">
-        <v>6.548345025272724</v>
+        <v>1.483894782548073</v>
       </c>
       <c r="G13">
-        <v>52.30486111111109</v>
+        <v>51.41527777777777</v>
       </c>
       <c r="H13">
-        <v>25.25705022604533</v>
+        <v>24.9812346474837</v>
       </c>
       <c r="I13">
-        <v>40.84062117976323</v>
+        <v>39.47956400188831</v>
       </c>
       <c r="J13">
-        <v>7339.372697241507</v>
+        <v>7401.973427854964</v>
       </c>
       <c r="K13">
-        <v>-2163.775000788945</v>
+        <v>-2149.253583664417</v>
       </c>
       <c r="L13">
-        <v>0.007327904676167626</v>
+        <v>0.00667891172177141</v>
       </c>
       <c r="M13">
-        <v>51.790001</v>
+        <v>44.25</v>
       </c>
       <c r="N13">
-        <v>3.217467849933493</v>
+        <v>0.3042432435915888</v>
       </c>
       <c r="O13">
-        <v>26.60013638889664</v>
+        <v>25.97292572782181</v>
       </c>
       <c r="P13">
-        <v>42.32393942969587</v>
+        <v>40.55229217804275</v>
       </c>
       <c r="Q13">
-        <v>-2278.837378900162</v>
+        <v>-2234.573450291562</v>
       </c>
       <c r="R13">
-        <v>1.5812634484874</v>
+        <v>0.8280389788975425</v>
       </c>
     </row>
     <row r="14" spans="1:18">
@@ -1164,55 +1164,55 @@
         <v>18</v>
       </c>
       <c r="B14">
-        <v>67.889999</v>
+        <v>61.560001</v>
       </c>
       <c r="C14">
-        <v>44.59</v>
+        <v>39.459999</v>
       </c>
       <c r="D14">
-        <v>1365.888707340242</v>
+        <v>1716.080418211201</v>
       </c>
       <c r="E14">
-        <v>-1647.954169555343</v>
+        <v>-1634.654174034399</v>
       </c>
       <c r="F14">
-        <v>10.76736162906301</v>
+        <v>3.759993488654166</v>
       </c>
       <c r="G14">
-        <v>55.73166666666664</v>
+        <v>54.85666666666665</v>
       </c>
       <c r="H14">
-        <v>27.08772812734043</v>
+        <v>26.78954811353956</v>
       </c>
       <c r="I14">
-        <v>42.6422144228135</v>
+        <v>41.26065731089754</v>
       </c>
       <c r="J14">
-        <v>6763.965877777771</v>
+        <v>6821.658711111135</v>
       </c>
       <c r="K14">
-        <v>-2227.785053619567</v>
+        <v>-2212.638077190948</v>
       </c>
       <c r="L14">
-        <v>0.003837867372846165</v>
+        <v>0.003491456744817566</v>
       </c>
       <c r="M14">
-        <v>37.09</v>
+        <v>32.459999</v>
       </c>
       <c r="N14">
-        <v>4.385492009707529</v>
+        <v>1.031296235306548</v>
       </c>
       <c r="O14">
-        <v>28.38125459769151</v>
+        <v>27.74445224341776</v>
       </c>
       <c r="P14">
-        <v>44.07571125574516</v>
+        <v>42.29644639199519</v>
       </c>
       <c r="Q14">
-        <v>-2334.168982296141</v>
+        <v>-2291.506792291354</v>
       </c>
       <c r="R14">
-        <v>1.516779312645018</v>
+        <v>0.8024855530961895</v>
       </c>
     </row>
     <row r="15" spans="1:18">
@@ -1220,55 +1220,55 @@
         <v>18</v>
       </c>
       <c r="B15">
-        <v>193.559998</v>
+        <v>180.910004</v>
       </c>
       <c r="C15">
-        <v>130.360001</v>
+        <v>118.910004</v>
       </c>
       <c r="D15">
-        <v>7869.830904326518</v>
+        <v>6072.212427057602</v>
       </c>
       <c r="E15">
-        <v>11564.50519640467</v>
+        <v>9265.990953517607</v>
       </c>
       <c r="F15">
-        <v>503.9524268373502</v>
+        <v>366.6224259369736</v>
       </c>
       <c r="G15">
-        <v>59.15847222222219</v>
+        <v>58.29805555555554</v>
       </c>
       <c r="H15">
-        <v>28.91745016904228</v>
+        <v>28.59694505339505</v>
       </c>
       <c r="I15">
-        <v>44.444763525457</v>
+        <v>43.04266714610714</v>
       </c>
       <c r="J15">
-        <v>6212.045050945209</v>
+        <v>6265.030309336441</v>
       </c>
       <c r="K15">
-        <v>-2279.173014510824</v>
+        <v>-2263.503806147159</v>
       </c>
       <c r="L15">
-        <v>0.001540854950634075</v>
+        <v>0.001396443448674873</v>
       </c>
       <c r="M15">
-        <v>122.860001</v>
+        <v>111.910004</v>
       </c>
       <c r="N15">
-        <v>532.8691765541626</v>
+        <v>380.3390067853571</v>
       </c>
       <c r="O15">
-        <v>30.16140834538672</v>
+        <v>29.51505710997332</v>
       </c>
       <c r="P15">
-        <v>45.82844754289411</v>
+        <v>44.041522254988</v>
       </c>
       <c r="Q15">
-        <v>-2377.217478671069</v>
+        <v>-2336.174160643217</v>
       </c>
       <c r="R15">
-        <v>1.451312814344609</v>
+        <v>0.7757083013618696</v>
       </c>
     </row>
     <row r="16" spans="1:18">
@@ -1276,55 +1276,55 @@
         <v>18</v>
       </c>
       <c r="B16">
-        <v>70.56999999999999</v>
+        <v>64.199997</v>
       </c>
       <c r="C16">
-        <v>45.27</v>
+        <v>39.200001</v>
       </c>
       <c r="D16">
-        <v>1174.97652546712</v>
+        <v>1504.323155216025</v>
       </c>
       <c r="E16">
-        <v>-1551.761917765891</v>
+        <v>-1520.395754785605</v>
       </c>
       <c r="F16">
-        <v>6.456788259705566</v>
+        <v>0.09138511563656197</v>
       </c>
       <c r="G16">
-        <v>62.58527777777775</v>
+        <v>61.73944444444443</v>
       </c>
       <c r="H16">
-        <v>30.74621132468617</v>
+        <v>30.40342062701389</v>
       </c>
       <c r="I16">
-        <v>46.24827351415844</v>
+        <v>44.82559834755338</v>
       </c>
       <c r="J16">
-        <v>5683.610216743822</v>
+        <v>5732.088222530886</v>
       </c>
       <c r="K16">
-        <v>-2317.948331153832</v>
+        <v>-2301.859866460463</v>
       </c>
       <c r="L16">
-        <v>0.0003068737753793297</v>
+        <v>0.0002745930917143237</v>
       </c>
       <c r="M16">
-        <v>37.77</v>
+        <v>32.200001</v>
       </c>
       <c r="N16">
-        <v>1.939539206921728</v>
+        <v>0.3516065672870776</v>
       </c>
       <c r="O16">
-        <v>31.94059256028581</v>
+        <v>31.28473546039928</v>
       </c>
       <c r="P16">
-        <v>47.58215336283916</v>
+        <v>45.7875246341104</v>
       </c>
       <c r="Q16">
-        <v>-2407.992400733124</v>
+        <v>-2368.584702115423</v>
       </c>
       <c r="R16">
-        <v>1.385007515246289</v>
+        <v>0.7477821556536064</v>
       </c>
     </row>
     <row r="17" spans="1:18">
@@ -1332,55 +1332,55 @@
         <v>18</v>
       </c>
       <c r="B17">
-        <v>101.110001</v>
+        <v>95.69000200000001</v>
       </c>
       <c r="C17">
-        <v>70.80999799999999</v>
+        <v>63.389999</v>
       </c>
       <c r="D17">
-        <v>13.97211761262898</v>
+        <v>53.2257793599999</v>
       </c>
       <c r="E17">
-        <v>-264.6827867241412</v>
+        <v>-462.4680767043996</v>
       </c>
       <c r="F17">
-        <v>141.501841374422</v>
+        <v>65.12627992607956</v>
       </c>
       <c r="G17">
-        <v>66.01208333333331</v>
+        <v>65.18083333333333</v>
       </c>
       <c r="H17">
-        <v>32.574006891661</v>
+        <v>32.20897031517408</v>
       </c>
       <c r="I17">
-        <v>48.05274909152895</v>
+        <v>46.60945543445828</v>
       </c>
       <c r="J17">
-        <v>5178.661375173606</v>
+        <v>5222.832450694465</v>
       </c>
       <c r="K17">
-        <v>-2344.120543444025</v>
+        <v>-2327.71544386904</v>
       </c>
       <c r="L17">
-        <v>1.057882432056571E-05</v>
+        <v>1.089944297256455E-05</v>
       </c>
       <c r="M17">
-        <v>63.30999799999999</v>
+        <v>56.389999</v>
       </c>
       <c r="N17">
-        <v>125.215063057427</v>
+        <v>56.43212886827529</v>
       </c>
       <c r="O17">
-        <v>33.71880249746027</v>
+        <v>33.0534827502139</v>
       </c>
       <c r="P17">
-        <v>49.33683346050886</v>
+        <v>47.53445807384417</v>
       </c>
       <c r="Q17">
-        <v>-2426.503374224524</v>
+        <v>-2388.747653789004</v>
       </c>
       <c r="R17">
-        <v>1.31801447725639</v>
+        <v>0.7187883505055718</v>
       </c>
     </row>
     <row r="18" spans="1:18">
@@ -1388,55 +1388,55 @@
         <v>18</v>
       </c>
       <c r="B18">
-        <v>129.059998</v>
+        <v>121.790001</v>
       </c>
       <c r="C18">
-        <v>81.459999</v>
+        <v>74.69000200000001</v>
       </c>
       <c r="D18">
-        <v>586.2242083128184</v>
+        <v>353.6054217512012</v>
       </c>
       <c r="E18">
-        <v>1972.314987084645</v>
+        <v>1404.500598918798</v>
       </c>
       <c r="F18">
-        <v>59.79216517553878</v>
+        <v>33.16371176447267</v>
       </c>
       <c r="G18">
-        <v>69.43888888888887</v>
+        <v>68.62222222222222</v>
       </c>
       <c r="H18">
-        <v>34.4008324997145</v>
+        <v>34.01358992789823</v>
       </c>
       <c r="I18">
-        <v>49.85819462782082</v>
+        <v>48.39424259679922</v>
       </c>
       <c r="J18">
-        <v>4697.198526234562</v>
+        <v>4737.262993827178</v>
       </c>
       <c r="K18">
-        <v>-2357.699278515153</v>
+        <v>-2341.079808981845</v>
       </c>
       <c r="L18">
-        <v>0.0005314350501514392</v>
+        <v>0.0004947793475855651</v>
       </c>
       <c r="M18">
-        <v>73.959999</v>
+        <v>67.69000200000001</v>
       </c>
       <c r="N18">
-        <v>55.23950889243303</v>
+        <v>30.03495398825103</v>
       </c>
       <c r="O18">
-        <v>35.49603374733114</v>
+        <v>34.82129476602024</v>
       </c>
       <c r="P18">
-        <v>51.09249224548215</v>
+        <v>49.28232678758622</v>
       </c>
       <c r="Q18">
-        <v>-2432.760112910835</v>
+        <v>-2396.672338090142</v>
       </c>
       <c r="R18">
-        <v>1.250492282961866</v>
+        <v>0.6888144698871799</v>
       </c>
     </row>
     <row r="19" spans="1:18">
@@ -1450,49 +1450,49 @@
         <v>22.625982</v>
       </c>
       <c r="D19">
-        <v>4987.459622513164</v>
+        <v>4727.885342544399</v>
       </c>
       <c r="E19">
-        <v>-1597.890937580569</v>
+        <v>-1555.75392444684</v>
       </c>
       <c r="F19">
-        <v>0.707994876859297</v>
+        <v>0.4097334694939737</v>
       </c>
       <c r="G19">
-        <v>72.86569444444443</v>
+        <v>72.06361111111111</v>
       </c>
       <c r="H19">
-        <v>36.22668411894173</v>
+        <v>35.81727561235326</v>
       </c>
       <c r="I19">
-        <v>51.66461415293896</v>
+        <v>50.1799636874093</v>
       </c>
       <c r="J19">
-        <v>4239.221669926691</v>
+        <v>4275.379851929029</v>
       </c>
       <c r="K19">
-        <v>-2358.694245564767</v>
+        <v>-2341.96231212985</v>
       </c>
       <c r="L19">
-        <v>0.001753871655916221</v>
+        <v>0.001620216541707712</v>
       </c>
       <c r="M19">
-        <v>15.125982</v>
+        <v>15.625982</v>
       </c>
       <c r="N19">
-        <v>6.33418235180159</v>
+        <v>3.446369324678761</v>
       </c>
       <c r="O19">
-        <v>37.27228224372953</v>
+        <v>36.58816763345017</v>
       </c>
       <c r="P19">
-        <v>52.84913378392791</v>
+        <v>51.03113464970467</v>
       </c>
       <c r="Q19">
-        <v>-2426.772413359892</v>
+        <v>-2392.368157612635</v>
       </c>
       <c r="R19">
-        <v>1.182607042632092</v>
+        <v>0.6579544826594816</v>
       </c>
     </row>
     <row r="20" spans="1:18">
@@ -1506,49 +1506,49 @@
         <v>56.676224</v>
       </c>
       <c r="D20">
-        <v>15.23489677437903</v>
+        <v>4.165117703044017</v>
       </c>
       <c r="E20">
-        <v>-221.2181041391855</v>
+        <v>-115.6683518650882</v>
       </c>
       <c r="F20">
-        <v>4.625658718025387</v>
+        <v>1.915634559248155</v>
       </c>
       <c r="G20">
-        <v>76.29249999999999</v>
+        <v>75.50500000000001</v>
       </c>
       <c r="H20">
-        <v>38.05155806722384</v>
+        <v>37.62002386018566</v>
       </c>
       <c r="I20">
-        <v>53.47201134900218</v>
+        <v>51.96662221464198</v>
       </c>
       <c r="J20">
-        <v>3804.730806249994</v>
+        <v>3837.183025000015</v>
       </c>
       <c r="K20">
-        <v>-2347.115230481533</v>
+        <v>-2330.372378019205</v>
       </c>
       <c r="L20">
-        <v>0.003567428699157712</v>
+        <v>0.003285898159995985</v>
       </c>
       <c r="M20">
-        <v>49.176224</v>
+        <v>49.676224</v>
       </c>
       <c r="N20">
-        <v>8.171775884750147</v>
+        <v>3.555980919141899</v>
       </c>
       <c r="O20">
-        <v>39.04754427140231</v>
+        <v>38.35409782454058</v>
       </c>
       <c r="P20">
-        <v>54.6067617910993</v>
+        <v>52.78088518816264</v>
       </c>
       <c r="Q20">
-        <v>-2408.550149520771</v>
+        <v>-2375.844589741171</v>
       </c>
       <c r="R20">
-        <v>1.11453238749262</v>
+        <v>0.6263087662902891</v>
       </c>
     </row>
     <row r="21" spans="1:18">
@@ -1562,49 +1562,49 @@
         <v>81.830321</v>
       </c>
       <c r="D21">
-        <v>9298.67516406828</v>
+        <v>9661.310776729089</v>
       </c>
       <c r="E21">
-        <v>7890.868265082697</v>
+        <v>8043.263211331407</v>
       </c>
       <c r="F21">
-        <v>910.2860509696048</v>
+        <v>815.3362933349026</v>
       </c>
       <c r="G21">
-        <v>79.71930555555555</v>
+        <v>78.9463888888889</v>
       </c>
       <c r="H21">
-        <v>39.87545101708577</v>
+        <v>39.42183151426043</v>
       </c>
       <c r="I21">
-        <v>55.28038954348563</v>
+        <v>53.75422133563232</v>
       </c>
       <c r="J21">
-        <v>3393.725935204468</v>
+        <v>3422.672513040137</v>
       </c>
       <c r="K21">
-        <v>-2322.972090285758</v>
+        <v>-2306.319500198041</v>
       </c>
       <c r="L21">
-        <v>0.005866895467595122</v>
+        <v>0.005395343402445789</v>
       </c>
       <c r="M21">
-        <v>74.330321</v>
+        <v>74.830321</v>
       </c>
       <c r="N21">
-        <v>865.7696339153384</v>
+        <v>782.937947638273</v>
       </c>
       <c r="O21">
-        <v>40.82181647293136</v>
+        <v>40.11908216450992</v>
       </c>
       <c r="P21">
-        <v>56.36537962441442</v>
+        <v>54.53158157774168</v>
       </c>
       <c r="Q21">
-        <v>-2378.103267114276</v>
+        <v>-2347.111181087207</v>
       </c>
       <c r="R21">
-        <v>1.046449449029601</v>
+        <v>0.5939841185376188</v>
       </c>
     </row>
     <row r="22" spans="1:18">
@@ -1618,49 +1618,49 @@
         <v>42.54</v>
       </c>
       <c r="D22">
-        <v>1192.177990761641</v>
+        <v>1067.041554022404</v>
       </c>
       <c r="E22">
-        <v>-1468.818167257809</v>
+        <v>-1389.59470908</v>
       </c>
       <c r="F22">
-        <v>0.00319045368743497</v>
+        <v>0.20311535813847</v>
       </c>
       <c r="G22">
-        <v>83.14611111111111</v>
+        <v>82.3877777777778</v>
       </c>
       <c r="H22">
-        <v>41.69836000194321</v>
+        <v>41.22269577477378</v>
       </c>
       <c r="I22">
-        <v>57.08975170297352</v>
+        <v>55.54276385018404</v>
       </c>
       <c r="J22">
-        <v>3006.207056790116</v>
+        <v>3031.848316049395</v>
       </c>
       <c r="K22">
-        <v>-2286.27474739543</v>
+        <v>-2269.813235349659</v>
       </c>
       <c r="L22">
-        <v>0.008552440096323199</v>
+        <v>0.007857023854873791</v>
       </c>
       <c r="M22">
-        <v>35.04</v>
+        <v>35.54</v>
       </c>
       <c r="N22">
-        <v>1.460368177817526</v>
+        <v>0.1436601524402014</v>
       </c>
       <c r="O22">
-        <v>42.59509585503698</v>
+        <v>41.88311783790518</v>
       </c>
       <c r="P22">
-        <v>58.12499027715295</v>
+        <v>56.28322663389479</v>
       </c>
       <c r="Q22">
-        <v>-2335.441777847392</v>
+        <v>-2306.177541750259</v>
       </c>
       <c r="R22">
-        <v>0.9785468241410855</v>
+        <v>0.5610937568604923</v>
       </c>
     </row>
     <row r="23" spans="1:18">
@@ -1674,49 +1674,49 @@
         <v>20.252212</v>
       </c>
       <c r="D23">
-        <v>5609.368662968835</v>
+        <v>5333.8760548921</v>
       </c>
       <c r="E23">
-        <v>-1516.803970757601</v>
+        <v>-1479.08769735868</v>
       </c>
       <c r="F23">
-        <v>0.9028519654943314</v>
+        <v>0.6163498403909494</v>
       </c>
       <c r="G23">
-        <v>86.57291666666667</v>
+        <v>85.82916666666669</v>
       </c>
       <c r="H23">
-        <v>43.52028242171257</v>
+        <v>43.02261420471277</v>
       </c>
       <c r="I23">
-        <v>58.90010042754952</v>
+        <v>57.33225219531015</v>
       </c>
       <c r="J23">
-        <v>2642.174171006938</v>
+        <v>2664.710434027788</v>
       </c>
       <c r="K23">
-        <v>-2237.033183731069</v>
+        <v>-2220.863197425782</v>
       </c>
       <c r="L23">
-        <v>0.01152972992813695</v>
+        <v>0.01058447498864428</v>
       </c>
       <c r="M23">
-        <v>12.752212</v>
+        <v>13.252212</v>
       </c>
       <c r="N23">
-        <v>7.222726504625855</v>
+        <v>4.191005002190891</v>
       </c>
       <c r="O23">
-        <v>44.36737979423813</v>
+        <v>43.64620239409194</v>
       </c>
       <c r="P23">
-        <v>59.88559637279597</v>
+        <v>58.03582280725642</v>
       </c>
       <c r="Q23">
-        <v>-2280.575753465075</v>
+        <v>-2253.053339418359</v>
       </c>
       <c r="R23">
-        <v>0.9110205260110008</v>
+        <v>0.5277573053686522</v>
       </c>
     </row>
     <row r="24" spans="1:18">
@@ -1730,49 +1730,49 @@
         <v>28.68</v>
       </c>
       <c r="D24">
-        <v>1644.13443176612</v>
+        <v>1496.575569988801</v>
       </c>
       <c r="E24">
-        <v>-1162.914563253699</v>
+        <v>-1109.50297932</v>
       </c>
       <c r="F24">
-        <v>115.0473135492912</v>
+        <v>105.4699211441236</v>
       </c>
       <c r="G24">
-        <v>89.99972222222223</v>
+        <v>89.27055555555559</v>
       </c>
       <c r="H24">
-        <v>45.34121604775874</v>
+        <v>44.82158473463686</v>
       </c>
       <c r="I24">
-        <v>60.71143794584869</v>
+        <v>59.12268844045116</v>
       </c>
       <c r="J24">
-        <v>2301.627277854931</v>
+        <v>2321.258866975318</v>
       </c>
       <c r="K24">
-        <v>-2175.257434673458</v>
+        <v>-2159.4790516344</v>
       </c>
       <c r="L24">
-        <v>0.01471004215365229</v>
+        <v>0.01349639839996538</v>
       </c>
       <c r="M24">
-        <v>21.18</v>
+        <v>21.68</v>
       </c>
       <c r="N24">
-        <v>143.1678575663022</v>
+        <v>124.6359604482749</v>
       </c>
       <c r="O24">
-        <v>46.13866604184487</v>
+        <v>45.40833375206271</v>
       </c>
       <c r="P24">
-        <v>61.64720016003338</v>
+        <v>59.78937217883402</v>
       </c>
       <c r="Q24">
-        <v>-2213.515319653627</v>
+        <v>-2187.748293322301</v>
       </c>
       <c r="R24">
-        <v>0.8440739206428882</v>
+        <v>0.4941007691771303</v>
       </c>
     </row>
     <row r="25" spans="1:18">
@@ -1786,49 +1786,49 @@
         <v>35.197163</v>
       </c>
       <c r="D25">
-        <v>1770.927008535196</v>
+        <v>1617.652824203025</v>
       </c>
       <c r="E25">
-        <v>-1481.180514612005</v>
+        <v>-1415.631831703965</v>
       </c>
       <c r="F25">
-        <v>11.53022399663394</v>
+        <v>8.717047566117088</v>
       </c>
       <c r="G25">
-        <v>93.42652777777779</v>
+        <v>92.71194444444448</v>
       </c>
       <c r="H25">
-        <v>47.16115902715947</v>
+        <v>46.61960566676003</v>
       </c>
       <c r="I25">
-        <v>62.52376611079333</v>
+        <v>60.91407428339308</v>
       </c>
       <c r="J25">
-        <v>1984.566377334098</v>
+        <v>2001.493614891983</v>
       </c>
       <c r="K25">
-        <v>-2100.957582889215</v>
+        <v>-2085.670508297607</v>
       </c>
       <c r="L25">
-        <v>0.01801036430647598</v>
+        <v>0.0165167543872387</v>
       </c>
       <c r="M25">
-        <v>27.697163</v>
+        <v>28.197163</v>
       </c>
       <c r="N25">
-        <v>21.68890540640488</v>
+        <v>14.92349484649733</v>
       </c>
       <c r="O25">
-        <v>47.90895272826102</v>
+        <v>47.16951020454186</v>
       </c>
       <c r="P25">
-        <v>63.40980350846139</v>
+        <v>61.54387645590325</v>
       </c>
       <c r="Q25">
-        <v>-2134.27064981069</v>
+        <v>-2110.272168059143</v>
       </c>
       <c r="R25">
-        <v>0.7779176490533302</v>
+        <v>0.4602564960879656</v>
       </c>
     </row>
     <row r="26" spans="1:18">
@@ -1842,49 +1842,49 @@
         <v>57.828844</v>
       </c>
       <c r="D26">
-        <v>251.8321564515946</v>
+        <v>314.407829939401</v>
       </c>
       <c r="E26">
-        <v>917.6986715469583</v>
+        <v>1025.394980999356</v>
       </c>
       <c r="F26">
-        <v>131.7233762866402</v>
+        <v>111.1520335814055</v>
       </c>
       <c r="G26">
-        <v>96.85333333333335</v>
+        <v>96.15333333333338</v>
       </c>
       <c r="H26">
-        <v>48.98010988626702</v>
+        <v>48.41667567831461</v>
       </c>
       <c r="I26">
-        <v>64.33708639603113</v>
+        <v>62.7064110469036</v>
       </c>
       <c r="J26">
-        <v>1690.991469444438</v>
+        <v>1705.414677777785</v>
       </c>
       <c r="K26">
-        <v>-2014.143752039773</v>
+        <v>-1999.44731659547</v>
       </c>
       <c r="L26">
-        <v>0.02135348423023556</v>
+        <v>0.01957484450594661</v>
       </c>
       <c r="M26">
-        <v>50.328844</v>
+        <v>50.828844</v>
       </c>
       <c r="N26">
-        <v>141.5687591335634</v>
+        <v>117.3481973554214</v>
       </c>
       <c r="O26">
-        <v>49.67823836657794</v>
+        <v>48.92973042136821</v>
       </c>
       <c r="P26">
-        <v>65.17340790498862</v>
+        <v>63.29933696862528</v>
       </c>
       <c r="Q26">
-        <v>-2042.851958697625</v>
+        <v>-2020.634767301107</v>
       </c>
       <c r="R26">
-        <v>0.7127695351893818</v>
+        <v>0.4263631255787882</v>
       </c>
     </row>
     <row r="27" spans="1:18">
@@ -1898,49 +1898,49 @@
         <v>23.973616</v>
       </c>
       <c r="D27">
-        <v>5651.177573932118</v>
+        <v>5374.647291264197</v>
       </c>
       <c r="E27">
-        <v>-1802.200151020869</v>
+        <v>-1757.553400561376</v>
       </c>
       <c r="F27">
-        <v>8.519795366788271</v>
+        <v>9.496343899721124</v>
       </c>
       <c r="G27">
-        <v>100.2801388888889</v>
+        <v>99.59472222222227</v>
       </c>
       <c r="H27">
-        <v>50.79806753355153</v>
+        <v>50.21279382418135</v>
       </c>
       <c r="I27">
-        <v>66.15139989309198</v>
+        <v>64.49969967610194</v>
       </c>
       <c r="J27">
-        <v>1420.90255418595</v>
+        <v>1433.022055632722</v>
       </c>
       <c r="K27">
-        <v>-1914.826100390063</v>
+        <v>-1900.819258212674</v>
       </c>
       <c r="L27">
-        <v>0.02466806917883876</v>
+        <v>0.0226053837844949</v>
       </c>
       <c r="M27">
-        <v>16.473616</v>
+        <v>16.973616</v>
       </c>
       <c r="N27">
-        <v>1.386509105524513</v>
+        <v>3.299725684848065</v>
       </c>
       <c r="O27">
-        <v>51.44652185544338</v>
+        <v>50.68899345213989</v>
       </c>
       <c r="P27">
-        <v>66.93801445096734</v>
+        <v>65.05575466740198</v>
       </c>
       <c r="Q27">
-        <v>-1939.269495990676</v>
+        <v>-1918.845927406719</v>
       </c>
       <c r="R27">
-        <v>0.6488544796979492</v>
+        <v>0.3925655251366397</v>
       </c>
     </row>
     <row r="28" spans="1:18">
@@ -1954,49 +1954,49 @@
         <v>40.669435</v>
       </c>
       <c r="D28">
-        <v>628.9309410095537</v>
+        <v>538.9904101718889</v>
       </c>
       <c r="E28">
-        <v>-1019.928246256294</v>
+        <v>-944.1883947556449</v>
       </c>
       <c r="F28">
-        <v>48.09495791804826</v>
+        <v>40.294749377817</v>
       </c>
       <c r="G28">
-        <v>103.7069444444445</v>
+        <v>103.0361111111112</v>
       </c>
       <c r="H28">
-        <v>52.61503126171304</v>
+        <v>52.00795953877365</v>
       </c>
       <c r="I28">
-        <v>67.96670730927582</v>
+        <v>66.29394073657475</v>
       </c>
       <c r="J28">
-        <v>1174.299631558636</v>
+        <v>1184.315748456795</v>
       </c>
       <c r="K28">
-        <v>-1803.01481433367</v>
+        <v>-1789.796140905189</v>
       </c>
       <c r="L28">
-        <v>0.02788873375810076</v>
+        <v>0.02554856233057633</v>
       </c>
       <c r="M28">
-        <v>33.169435</v>
+        <v>33.669435</v>
       </c>
       <c r="N28">
-        <v>63.20255892206032</v>
+        <v>50.07407523277739</v>
       </c>
       <c r="O28">
-        <v>53.2138024811926</v>
+        <v>52.44729872810896</v>
       </c>
       <c r="P28">
-        <v>68.70362386006228</v>
+        <v>66.8131301209813</v>
       </c>
       <c r="Q28">
-        <v>-1823.533539747863</v>
+        <v>-1804.915510951509</v>
       </c>
       <c r="R28">
-        <v>0.5864043397403218</v>
+        <v>0.3590147140340142</v>
       </c>
     </row>
     <row r="29" spans="1:18">
@@ -2010,49 +2010,49 @@
         <v>16.560776</v>
       </c>
       <c r="D29">
-        <v>6738.30094852513</v>
+        <v>6436.022706730278</v>
       </c>
       <c r="E29">
-        <v>-1359.426979626482</v>
+        <v>-1328.585373024976</v>
       </c>
       <c r="F29">
-        <v>0.6894145758350496</v>
+        <v>0.5272818595790737</v>
       </c>
       <c r="G29">
-        <v>107.13375</v>
+        <v>106.4775000000001</v>
       </c>
       <c r="H29">
-        <v>54.43100074905288</v>
+        <v>53.80217263716703</v>
       </c>
       <c r="I29">
-        <v>69.78300896628133</v>
+        <v>68.08913441324646</v>
       </c>
       <c r="J29">
-        <v>951.182701562494</v>
+        <v>959.2957562500042</v>
       </c>
       <c r="K29">
-        <v>-1678.720101851722</v>
+        <v>-1666.38779200466</v>
       </c>
       <c r="L29">
-        <v>0.03095609646616805</v>
+        <v>0.02835009610583865</v>
       </c>
       <c r="M29">
-        <v>9.060776000000001</v>
+        <v>9.560776000000001</v>
       </c>
       <c r="N29">
-        <v>7.139143267823861</v>
+        <v>4.265418502147877</v>
       </c>
       <c r="O29">
-        <v>54.98007991923205</v>
+        <v>54.20464606331736</v>
       </c>
       <c r="P29">
-        <v>70.47023645686699</v>
+        <v>68.57146351532128</v>
       </c>
       <c r="Q29">
-        <v>-1695.65438980901</v>
+        <v>-1678.8534001961</v>
       </c>
       <c r="R29">
-        <v>0.5256577951078497</v>
+        <v>0.325867774703184</v>
       </c>
     </row>
     <row r="30" spans="1:18">
@@ -2066,49 +2066,49 @@
         <v>13.33273</v>
       </c>
       <c r="D30">
-        <v>6370.466245068867</v>
+        <v>6076.650253048384</v>
       </c>
       <c r="E30">
-        <v>-1064.154519349526</v>
+        <v>-1039.32459510056</v>
       </c>
       <c r="F30">
-        <v>27.69331925427065</v>
+        <v>26.40957148951076</v>
       </c>
       <c r="G30">
-        <v>110.5605555555556</v>
+        <v>109.918888888889</v>
       </c>
       <c r="H30">
-        <v>56.24597606009814</v>
+        <v>55.59543331546889</v>
       </c>
       <c r="I30">
-        <v>71.60030479958141</v>
+        <v>69.88528051000971</v>
       </c>
       <c r="J30">
-        <v>751.5517641975252</v>
+        <v>757.962079012349</v>
       </c>
       <c r="K30">
-        <v>-1541.952185923107</v>
+        <v>-1530.604051878546</v>
       </c>
       <c r="L30">
-        <v>0.03381682464072362</v>
+        <v>0.03096126669658746</v>
       </c>
       <c r="M30">
-        <v>5.83273</v>
+        <v>6.33273</v>
       </c>
       <c r="N30">
-        <v>50.00055776034725</v>
+        <v>41.65198814423763</v>
       </c>
       <c r="O30">
-        <v>56.74535423466948</v>
+        <v>55.96103565496856</v>
       </c>
       <c r="P30">
-        <v>72.23785217627371</v>
+        <v>70.33075465321845</v>
       </c>
       <c r="Q30">
-        <v>-1555.642361146661</v>
+        <v>-1540.669490509793</v>
       </c>
       <c r="R30">
-        <v>0.4668602009584451</v>
+        <v>0.2932877519227914</v>
       </c>
     </row>
     <row r="31" spans="1:18">
@@ -2122,49 +2122,49 @@
         <v>26.89</v>
       </c>
       <c r="D31">
-        <v>3990.187454901914</v>
+        <v>3758.376836582404</v>
       </c>
       <c r="E31">
-        <v>-1698.585653539315</v>
+        <v>-1648.50763778</v>
       </c>
       <c r="F31">
-        <v>0.2786579329193065</v>
+        <v>0.06937849741848641</v>
       </c>
       <c r="G31">
-        <v>113.9873611111112</v>
+        <v>113.3602777777779</v>
       </c>
       <c r="H31">
-        <v>58.05995764547634</v>
+        <v>57.38774215042637</v>
       </c>
       <c r="I31">
-        <v>73.41859435854857</v>
+        <v>71.68237845011731</v>
       </c>
       <c r="J31">
-        <v>575.4068194637294</v>
+        <v>580.3147167438299</v>
       </c>
       <c r="K31">
-        <v>-1392.721297903864</v>
+        <v>-1382.454767364288</v>
       </c>
       <c r="L31">
-        <v>0.03642366767334451</v>
+        <v>0.03333894995913642</v>
       </c>
       <c r="M31">
-        <v>19.39</v>
+        <v>19.89</v>
       </c>
       <c r="N31">
-        <v>4.389649785876047</v>
+        <v>1.959688360938462</v>
       </c>
       <c r="O31">
-        <v>58.50962588218749</v>
+        <v>57.71646808303345</v>
       </c>
       <c r="P31">
-        <v>74.00647056359988</v>
+        <v>72.09100295470196</v>
       </c>
       <c r="Q31">
-        <v>-1403.507777185894</v>
+        <v>-1390.373683768034</v>
       </c>
       <c r="R31">
-        <v>0.4102634275538884</v>
+        <v>0.2614435400877185</v>
       </c>
     </row>
     <row r="32" spans="1:18">
@@ -2178,49 +2178,49 @@
         <v>17.42932</v>
       </c>
       <c r="D32">
-        <v>6842.368537781424</v>
+        <v>6537.738338863523</v>
       </c>
       <c r="E32">
-        <v>-1441.729133911786</v>
+        <v>-1409.27001298824</v>
       </c>
       <c r="F32">
-        <v>0.1390488916445807</v>
+        <v>0.2225103642881569</v>
       </c>
       <c r="G32">
-        <v>117.4141666666667</v>
+        <v>116.8016666666667</v>
       </c>
       <c r="H32">
-        <v>59.87294634104097</v>
+        <v>59.17910009827472</v>
       </c>
       <c r="I32">
-        <v>75.23787680732929</v>
+        <v>73.48042727733406</v>
       </c>
       <c r="J32">
-        <v>422.7478673611065</v>
+        <v>426.3536694444465</v>
       </c>
       <c r="K32">
-        <v>-1231.037670893747</v>
+        <v>-1221.949785195879</v>
       </c>
       <c r="L32">
-        <v>0.03873547840421159</v>
+        <v>0.03544563347050846</v>
       </c>
       <c r="M32">
-        <v>9.929320000000001</v>
+        <v>10.42932</v>
       </c>
       <c r="N32">
-        <v>2.184104038934631</v>
+        <v>0.7642275744912972</v>
       </c>
       <c r="O32">
-        <v>60.27289570516118</v>
+        <v>59.470944309092</v>
       </c>
       <c r="P32">
-        <v>75.77609077547035</v>
+        <v>73.85220745819177</v>
       </c>
       <c r="Q32">
-        <v>-1239.260963111195</v>
+        <v>-1227.975881742238</v>
       </c>
       <c r="R32">
-        <v>0.3561256874373427</v>
+        <v>0.2305097588890266</v>
       </c>
     </row>
     <row r="33" spans="1:18">
@@ -2234,49 +2234,49 @@
         <v>24.270606</v>
       </c>
       <c r="D33">
-        <v>4661.793053037277</v>
+        <v>4410.951693680016</v>
       </c>
       <c r="E33">
-        <v>-1657.132043834729</v>
+        <v>-1611.932200407576</v>
       </c>
       <c r="F33">
-        <v>0.1930742946069086</v>
+        <v>0.04761764706150799</v>
       </c>
       <c r="G33">
-        <v>120.8409722222223</v>
+        <v>120.2430555555556</v>
       </c>
       <c r="H33">
-        <v>61.68494336625189</v>
+        <v>60.96950849283093</v>
       </c>
       <c r="I33">
-        <v>77.05815092646374</v>
+        <v>75.27942565784292</v>
       </c>
       <c r="J33">
-        <v>293.5749078896565</v>
+        <v>296.0789371141991</v>
       </c>
       <c r="K33">
-        <v>-1056.911533108002</v>
+        <v>-1049.098945441228</v>
       </c>
       <c r="L33">
-        <v>0.04071722266415587</v>
+        <v>0.03724942276711969</v>
       </c>
       <c r="M33">
-        <v>16.770606</v>
+        <v>17.270606</v>
       </c>
       <c r="N33">
-        <v>4.329560980436123</v>
+        <v>1.986508534300461</v>
       </c>
       <c r="O33">
-        <v>62.03516493402392</v>
+        <v>61.2244656744165</v>
       </c>
       <c r="P33">
-        <v>77.54671158145175</v>
+        <v>75.61436682241565</v>
       </c>
       <c r="Q33">
-        <v>-1062.912239178585</v>
+        <v>-1053.485979500483</v>
       </c>
       <c r="R33">
-        <v>0.3047113505470272</v>
+        <v>0.2006666177841511</v>
       </c>
     </row>
     <row r="34" spans="1:18">
@@ -2290,49 +2290,49 @@
         <v>20.22</v>
       </c>
       <c r="D34">
-        <v>5885.640873864929</v>
+        <v>5603.361150782404</v>
       </c>
       <c r="E34">
-        <v>-1551.236556510411</v>
+        <v>-1513.58027244</v>
       </c>
       <c r="F34">
-        <v>0.0002776495475180628</v>
+        <v>0.01768957183603532</v>
       </c>
       <c r="G34">
-        <v>124.2677777777778</v>
+        <v>123.6844444444445</v>
       </c>
       <c r="H34">
-        <v>63.49595032181759</v>
+        <v>62.75896904284201</v>
       </c>
       <c r="I34">
-        <v>78.87941511524338</v>
+        <v>77.07937188289694</v>
       </c>
       <c r="J34">
-        <v>187.8879410493794</v>
+        <v>189.4905197530875</v>
       </c>
       <c r="K34">
-        <v>-870.3531012723286</v>
+        <v>-863.9120749686354</v>
       </c>
       <c r="L34">
-        <v>0.04233997698433341</v>
+        <v>0.03872403640645273</v>
       </c>
       <c r="M34">
-        <v>12.72</v>
+        <v>13.22</v>
       </c>
       <c r="N34">
-        <v>3.169873062717155</v>
+        <v>1.31935476901507</v>
       </c>
       <c r="O34">
-        <v>63.7964351838886</v>
+        <v>62.97703389730484</v>
       </c>
       <c r="P34">
-        <v>79.31833136643124</v>
+        <v>77.3774793290757</v>
       </c>
       <c r="Q34">
-        <v>-874.4719140511497</v>
+        <v>-866.9138588374576</v>
       </c>
       <c r="R34">
-        <v>0.2562907478151345</v>
+        <v>0.1720997696884354</v>
       </c>
     </row>
     <row r="35" spans="1:18">
@@ -2346,49 +2346,49 @@
         <v>23.24</v>
       </c>
       <c r="D35">
-        <v>5185.14206771616</v>
+        <v>4920.405479942404</v>
       </c>
       <c r="E35">
-        <v>-1673.464306889315</v>
+        <v>-1630.18379048</v>
       </c>
       <c r="F35">
-        <v>0.2571861910731679</v>
+        <v>0.4854062642143876</v>
       </c>
       <c r="G35">
-        <v>127.6945833333334</v>
+        <v>127.1258333333334</v>
       </c>
       <c r="H35">
-        <v>65.30596918661048</v>
+        <v>64.54748382859982</v>
       </c>
       <c r="I35">
-        <v>80.70166739479585</v>
+        <v>78.88026387220422</v>
       </c>
       <c r="J35">
-        <v>105.6869668402752</v>
+        <v>106.5884173611118</v>
       </c>
       <c r="K35">
-        <v>-671.3725740588419</v>
+        <v>-666.3989809604381</v>
       </c>
       <c r="L35">
-        <v>0.04358091454733361</v>
+        <v>0.03984878993813478</v>
       </c>
       <c r="M35">
-        <v>15.74</v>
+        <v>16.24</v>
       </c>
       <c r="N35">
-        <v>1.41209981028068</v>
+        <v>0.2856590829780079</v>
       </c>
       <c r="O35">
-        <v>65.55670845143489</v>
+        <v>64.72865106967646</v>
       </c>
       <c r="P35">
-        <v>81.0909481337291</v>
+        <v>79.14154288625247</v>
       </c>
       <c r="Q35">
-        <v>-673.9502781759304</v>
+        <v>-668.2693817518534</v>
       </c>
       <c r="R35">
-        <v>0.2111399638507178</v>
+        <v>0.1450001543674762</v>
       </c>
     </row>
     <row r="36" spans="1:18">
@@ -2402,49 +2402,49 @@
         <v>52.269249</v>
       </c>
       <c r="D36">
-        <v>452.7821624957158</v>
+        <v>376.9946473224998</v>
       </c>
       <c r="E36">
-        <v>-1112.220549561558</v>
+        <v>-1014.87803282115</v>
       </c>
       <c r="F36">
-        <v>7.027468512631166</v>
+        <v>10.69534498492492</v>
       </c>
       <c r="G36">
-        <v>131.121388888889</v>
+        <v>130.5672222222223</v>
       </c>
       <c r="H36">
-        <v>67.11500231386837</v>
+        <v>66.33505529783811</v>
       </c>
       <c r="I36">
-        <v>82.5249054118833</v>
+        <v>80.68209917803101</v>
       </c>
       <c r="J36">
-        <v>46.97198526234387</v>
+        <v>47.37262993827216</v>
       </c>
       <c r="K36">
-        <v>-459.9801255805673</v>
+        <v>-456.5694444916228</v>
       </c>
       <c r="L36">
-        <v>0.04442327950560134</v>
+        <v>0.04060856892151829</v>
       </c>
       <c r="M36">
-        <v>44.769249</v>
+        <v>45.269249</v>
       </c>
       <c r="N36">
-        <v>2.859771352522934</v>
+        <v>6.669755448925468</v>
       </c>
       <c r="O36">
-        <v>67.31598711107674</v>
+        <v>66.4793196529465</v>
       </c>
       <c r="P36">
-        <v>82.86455950893142</v>
+        <v>80.90655503253079</v>
       </c>
       <c r="Q36">
-        <v>-461.357597219879</v>
+        <v>-457.5623839890883</v>
       </c>
       <c r="R36">
-        <v>0.1695406193526027</v>
+        <v>0.119563832054383</v>
       </c>
     </row>
     <row r="37" spans="1:18">
@@ -2458,49 +2458,49 @@
         <v>58.51</v>
       </c>
       <c r="D37">
-        <v>137.7790145131467</v>
+        <v>97.52751486240402</v>
       </c>
       <c r="E37">
-        <v>-686.7863187647947</v>
+        <v>-577.82147302</v>
       </c>
       <c r="F37">
-        <v>14.70945368514252</v>
+        <v>20.57141196608997</v>
       </c>
       <c r="G37">
-        <v>134.5481944444445</v>
+        <v>134.0086111111112</v>
       </c>
       <c r="H37">
-        <v>68.9230524266997</v>
+        <v>68.12168626093077</v>
       </c>
       <c r="I37">
-        <v>84.34912644339731</v>
+        <v>82.48487499000345</v>
       </c>
       <c r="J37">
-        <v>11.74299631558558</v>
+        <v>11.84315748456814</v>
       </c>
       <c r="K37">
-        <v>-236.1858989616529</v>
+        <v>-234.4332141907444</v>
       </c>
       <c r="L37">
-        <v>0.04485634984452243</v>
+        <v>0.04099379117632389</v>
       </c>
       <c r="M37">
-        <v>51.01</v>
+        <v>51.51</v>
       </c>
       <c r="N37">
-        <v>9.082901143982024</v>
+        <v>15.60236040908589</v>
       </c>
       <c r="O37">
-        <v>69.07427391042701</v>
+        <v>68.22904247319717</v>
       </c>
       <c r="P37">
-        <v>84.63916274442529</v>
+        <v>82.67251294182849</v>
       </c>
       <c r="Q37">
-        <v>-236.704105582209</v>
+        <v>-234.8026686667912</v>
       </c>
       <c r="R37">
-        <v>0.1317796439385638</v>
+        <v>0.09599180785773824</v>
       </c>
     </row>
     <row r="38" spans="1:18">
@@ -2514,49 +2514,49 @@
         <v>61</v>
       </c>
       <c r="D38">
-        <v>737.23487329753</v>
+        <v>841.835291302404</v>
       </c>
       <c r="E38">
-        <v>1656.276234068493</v>
+        <v>1769.878278</v>
       </c>
       <c r="F38">
-        <v>204.0783517135238</v>
+        <v>175.7156714243275</v>
       </c>
       <c r="G38">
-        <v>137.9750000000001</v>
+        <v>137.4500000000001</v>
       </c>
       <c r="H38">
-        <v>70.73012261291183</v>
+        <v>69.90737988541267</v>
       </c>
       <c r="I38">
-        <v>86.17432740153052</v>
+        <v>84.28858814058663</v>
       </c>
       <c r="J38">
-        <v>1.292469707114106E-26</v>
+        <v>8.077935669463161E-28</v>
       </c>
       <c r="K38">
-        <v>8.041083971524111E-12</v>
+        <v>-1.986887238144069E-12</v>
       </c>
       <c r="L38">
-        <v>0.04487538901670024</v>
+        <v>0.04100035850007877</v>
       </c>
       <c r="M38">
-        <v>53.5</v>
+        <v>54</v>
       </c>
       <c r="N38">
-        <v>211.5040425656361</v>
+        <v>180.2250256204241</v>
       </c>
       <c r="O38">
-        <v>70.83157196507941</v>
+        <v>69.97782271566803</v>
       </c>
       <c r="P38">
-        <v>86.41475472461704</v>
+        <v>84.43941342890602</v>
       </c>
       <c r="Q38">
-        <v>8.05261742756095E-12</v>
+        <v>-1.988889343797042E-12</v>
       </c>
       <c r="R38">
-        <v>0.0981490401159433</v>
+        <v>0.07448984756276589</v>
       </c>
     </row>
     <row r="39" spans="1:18">
@@ -2570,49 +2570,49 @@
         <v>89</v>
       </c>
       <c r="D39">
-        <v>1455.580400338626</v>
+        <v>1601.152047302404</v>
       </c>
       <c r="E39">
-        <v>3395.534177575342</v>
+        <v>3561.281422</v>
       </c>
       <c r="F39">
-        <v>62.16738474397535</v>
+        <v>81.13794251459477</v>
       </c>
       <c r="G39">
-        <v>141.4018055555556</v>
+        <v>140.891388888889</v>
       </c>
       <c r="H39">
-        <v>72.53621631918557</v>
+        <v>71.6921396898481</v>
       </c>
       <c r="I39">
-        <v>88.00050483960212</v>
+        <v>86.09323511121629</v>
       </c>
       <c r="J39">
-        <v>11.74299631558713</v>
+        <v>11.84315748456775</v>
       </c>
       <c r="K39">
-        <v>248.5675090615723</v>
+        <v>246.7205329493118</v>
       </c>
       <c r="L39">
-        <v>0.04448158662177031</v>
+        <v>0.04062959813196867</v>
       </c>
       <c r="M39">
-        <v>81.5</v>
+        <v>82</v>
       </c>
       <c r="N39">
-        <v>60.63046309827706</v>
+        <v>80.21846096535347</v>
       </c>
       <c r="O39">
-        <v>72.58788475273039</v>
+        <v>71.72566391859003</v>
       </c>
       <c r="P39">
-        <v>88.1913319718102</v>
+        <v>86.20725295553238</v>
       </c>
       <c r="Q39">
-        <v>248.7445667366905</v>
+        <v>246.8359028576128</v>
       </c>
       <c r="R39">
-        <v>0.0689456391504621</v>
+        <v>0.05526828546194416</v>
       </c>
     </row>
     <row r="40" spans="1:18">
@@ -2626,49 +2626,49 @@
         <v>82.7</v>
       </c>
       <c r="D40">
-        <v>6107.745953215338</v>
+        <v>6402.303887302404</v>
       </c>
       <c r="E40">
-        <v>6463.176140286301</v>
+        <v>6617.1907146</v>
       </c>
       <c r="F40">
-        <v>384.7300712468038</v>
+        <v>329.5154919450508</v>
       </c>
       <c r="G40">
-        <v>144.8286111111111</v>
+        <v>144.3327777777779</v>
       </c>
       <c r="H40">
-        <v>74.3413373446209</v>
+        <v>73.47596953707401</v>
       </c>
       <c r="I40">
-        <v>89.82765495851213</v>
+        <v>87.89881203905549</v>
       </c>
       <c r="J40">
-        <v>46.97198526234698</v>
+        <v>47.37262993827138</v>
       </c>
       <c r="K40">
-        <v>509.5066156399602</v>
+        <v>505.7187703304487</v>
       </c>
       <c r="L40">
-        <v>0.04368198845109393</v>
+        <v>0.03988819428520194</v>
       </c>
       <c r="M40">
-        <v>75.2</v>
+        <v>75.7</v>
       </c>
       <c r="N40">
-        <v>366.0559409963294</v>
+        <v>315.9605457724832</v>
       </c>
       <c r="O40">
-        <v>74.34321610666699</v>
+        <v>73.47256996639109</v>
       </c>
       <c r="P40">
-        <v>89.96889065271775</v>
+        <v>87.97602763727971</v>
       </c>
       <c r="Q40">
-        <v>509.5194919443945</v>
+        <v>505.6953718408984</v>
       </c>
       <c r="R40">
-        <v>0.04447084961861063</v>
+        <v>0.0385418248798863</v>
       </c>
     </row>
     <row r="41" spans="1:18">
@@ -2682,49 +2682,49 @@
         <v>47.28</v>
       </c>
       <c r="D41">
-        <v>904.0804499073934</v>
+        <v>795.5559841824039</v>
       </c>
       <c r="E41">
-        <v>-1421.611758249863</v>
+        <v>-1333.56086256</v>
       </c>
       <c r="F41">
-        <v>5.381512822540723</v>
+        <v>8.206898458902371</v>
       </c>
       <c r="G41">
-        <v>148.2554166666667</v>
+        <v>147.7741666666668</v>
       </c>
       <c r="H41">
-        <v>76.14548983368191</v>
+        <v>75.2588736268476</v>
       </c>
       <c r="I41">
-        <v>91.65577361379646</v>
+        <v>89.70531472434699</v>
       </c>
       <c r="J41">
-        <v>105.6869668402796</v>
+        <v>106.5884173611109</v>
       </c>
       <c r="K41">
-        <v>782.8073627776872</v>
+        <v>776.9851544691783</v>
       </c>
       <c r="L41">
-        <v>0.04248941625911343</v>
+        <v>0.03878811011056933</v>
       </c>
       <c r="M41">
-        <v>39.78</v>
+        <v>40.28</v>
       </c>
       <c r="N41">
-        <v>1.519076930741545</v>
+        <v>4.338197691412979</v>
       </c>
       <c r="O41">
-        <v>76.09757020864812</v>
+        <v>75.21854508230261</v>
       </c>
       <c r="P41">
-        <v>91.74742658558075</v>
+        <v>89.74573325091659</v>
       </c>
       <c r="Q41">
-        <v>782.3147290658295</v>
+        <v>776.5687958538717</v>
       </c>
       <c r="R41">
-        <v>0.02503039945074105</v>
+        <v>0.02452933208138387</v>
       </c>
     </row>
     <row r="42" spans="1:18">
@@ -2738,49 +2738,49 @@
         <v>146.5</v>
       </c>
       <c r="D42">
-        <v>24258.70712579617</v>
+        <v>24842.29845690241</v>
       </c>
       <c r="E42">
-        <v>22817.67816870548</v>
+        <v>23090.509307</v>
       </c>
       <c r="F42">
-        <v>9.357964218781817</v>
+        <v>26.81798225748312</v>
       </c>
       <c r="G42">
-        <v>151.6822222222222</v>
+        <v>151.2155555555557</v>
       </c>
       <c r="H42">
-        <v>77.94867826857077</v>
+        <v>77.04085648793065</v>
       </c>
       <c r="I42">
-        <v>93.48485632325293</v>
+        <v>91.51273863832901</v>
       </c>
       <c r="J42">
-        <v>187.8879410493848</v>
+        <v>189.4905197530863</v>
       </c>
       <c r="K42">
-        <v>1068.45985495581</v>
+        <v>1060.510190032192</v>
       </c>
       <c r="L42">
-        <v>0.04092237766278435</v>
+        <v>0.03734650049081102</v>
       </c>
       <c r="M42">
-        <v>139</v>
+        <v>139.5</v>
       </c>
       <c r="N42">
-        <v>21.77407768002555</v>
+        <v>40.79525415825609</v>
       </c>
       <c r="O42">
-        <v>77.85095158121003</v>
+        <v>76.96359382039944</v>
       </c>
       <c r="P42">
-        <v>93.52693524786299</v>
+        <v>91.51636524236812</v>
       </c>
       <c r="Q42">
-        <v>1067.120293535114</v>
+        <v>1059.44662648992</v>
       </c>
       <c r="R42">
-        <v>0.01093407229031343</v>
+        <v>0.01345362427126891</v>
       </c>
     </row>
     <row r="43" spans="1:18">
@@ -2794,49 +2794,49 @@
         <v>131.2</v>
       </c>
       <c r="D43">
-        <v>13306.09991739068</v>
+        <v>13739.2150985024</v>
       </c>
       <c r="E43">
-        <v>15134.19150671781</v>
+        <v>15378.5290176</v>
       </c>
       <c r="F43">
-        <v>84.09325664018766</v>
+        <v>119.8462706976806</v>
       </c>
       <c r="G43">
-        <v>155.1090277777778</v>
+        <v>154.6569444444446</v>
       </c>
       <c r="H43">
-        <v>79.75090746106285</v>
+        <v>78.82192296964406</v>
       </c>
       <c r="I43">
-        <v>95.31489827510619</v>
+        <v>93.3210789316807</v>
       </c>
       <c r="J43">
-        <v>293.5749078896628</v>
+        <v>296.0789371141976</v>
       </c>
       <c r="K43">
-        <v>1366.454263740841</v>
+        <v>1356.284449542945</v>
       </c>
       <c r="L43">
-        <v>0.03900496660658757</v>
+        <v>0.03558561609923037</v>
       </c>
       <c r="M43">
-        <v>123.7</v>
+        <v>124.2</v>
       </c>
       <c r="N43">
-        <v>103.8688466890079</v>
+        <v>137.4331556272097</v>
       </c>
       <c r="O43">
-        <v>79.60336507942783</v>
+        <v>78.70772105710734</v>
       </c>
       <c r="P43">
-        <v>95.30741178448933</v>
+        <v>93.28791873520862</v>
       </c>
       <c r="Q43">
-        <v>1363.926268475507</v>
+        <v>1354.319383578476</v>
       </c>
       <c r="R43">
-        <v>0.002495439006266882</v>
+        <v>0.005541252409383571</v>
       </c>
     </row>
     <row r="44" spans="1:18">
@@ -2850,49 +2850,49 @@
         <v>127</v>
       </c>
       <c r="D44">
-        <v>14197.21564491397</v>
+        <v>14644.4845233024</v>
       </c>
       <c r="E44">
-        <v>15132.31281519178</v>
+        <v>15368.828546</v>
       </c>
       <c r="F44">
-        <v>8.73980837448461</v>
+        <v>22.71200210221842</v>
       </c>
       <c r="G44">
-        <v>158.5358333333333</v>
+        <v>158.0983333333335</v>
       </c>
       <c r="H44">
-        <v>81.55218254383651</v>
+        <v>80.60207823292855</v>
       </c>
       <c r="I44">
-        <v>97.14589433667787</v>
+        <v>95.13033044346132</v>
       </c>
       <c r="J44">
-        <v>422.7478673611135</v>
+        <v>426.3536694444447</v>
       </c>
       <c r="K44">
-        <v>1676.780833253403</v>
+        <v>1664.29857871292</v>
       </c>
       <c r="L44">
-        <v>0.03676675486368033</v>
+        <v>0.03353269918664008</v>
       </c>
       <c r="M44">
-        <v>119.5</v>
+        <v>120</v>
       </c>
       <c r="N44">
-        <v>16.26337826108857</v>
+        <v>31.16064508294856</v>
       </c>
       <c r="O44">
-        <v>81.3548158821674</v>
+        <v>80.4509319822136</v>
       </c>
       <c r="P44">
-        <v>97.08885101659391</v>
+        <v>95.06038853965072</v>
       </c>
       <c r="Q44">
-        <v>1672.722810217268</v>
+        <v>1661.177660546075</v>
       </c>
       <c r="R44">
-        <v>3.158520301441498E-05</v>
+        <v>0.001022279574150402</v>
       </c>
     </row>
     <row r="45" spans="1:18">
@@ -2906,49 +2906,49 @@
         <v>98.86</v>
       </c>
       <c r="D45">
-        <v>9226.000038127668</v>
+        <v>9587.229335702405</v>
       </c>
       <c r="E45">
-        <v>9495.707581967397</v>
+        <v>9679.817386280001</v>
       </c>
       <c r="F45">
-        <v>167.4737367521918</v>
+        <v>128.3125016848963</v>
       </c>
       <c r="G45">
-        <v>161.9626388888889</v>
+        <v>161.5397222222224</v>
       </c>
       <c r="H45">
-        <v>83.35250896133319</v>
+        <v>82.38132774094845</v>
       </c>
       <c r="I45">
-        <v>98.97783906352653</v>
+        <v>96.94048771050652</v>
       </c>
       <c r="J45">
-        <v>575.406819463737</v>
+        <v>580.3147167438278</v>
       </c>
       <c r="K45">
-        <v>1999.42988544734</v>
+        <v>1984.543301577299</v>
       </c>
       <c r="L45">
-        <v>0.03424267507279459</v>
+        <v>0.0312198715871578</v>
       </c>
       <c r="M45">
-        <v>91.36</v>
+        <v>91.86</v>
       </c>
       <c r="N45">
-        <v>148.8316028719234</v>
+        <v>115.7450945913998</v>
       </c>
       <c r="O45">
-        <v>83.10530948286316</v>
+        <v>82.19323208941847</v>
       </c>
       <c r="P45">
-        <v>98.87124745074229</v>
+        <v>96.83376916199424</v>
       </c>
       <c r="Q45">
-        <v>1993.500153624279</v>
+        <v>1980.012129580734</v>
       </c>
       <c r="R45">
-        <v>0.003862835574149216</v>
+        <v>0.000130055613482142</v>
       </c>
     </row>
     <row r="46" spans="1:18">
@@ -2962,49 +2962,49 @@
         <v>110.1</v>
       </c>
       <c r="D46">
-        <v>4907.292428757804</v>
+        <v>5171.680639702405</v>
       </c>
       <c r="E46">
-        <v>7712.732842146575</v>
+        <v>7917.7752198</v>
       </c>
       <c r="F46">
-        <v>145.885187239876</v>
+        <v>181.4849046441677</v>
       </c>
       <c r="G46">
-        <v>165.3894444444444</v>
+        <v>164.9811111111113</v>
       </c>
       <c r="H46">
-        <v>85.15189246018396</v>
+        <v>84.159677249277</v>
       </c>
       <c r="I46">
-        <v>100.8107267090211</v>
+        <v>98.75154497724307</v>
       </c>
       <c r="J46">
-        <v>751.5517641975331</v>
+        <v>757.9620790123467</v>
       </c>
       <c r="K46">
-        <v>2334.391825189024</v>
+        <v>2317.009425425097</v>
       </c>
       <c r="L46">
-        <v>0.03147289583610845</v>
+        <v>0.02868401545673308</v>
       </c>
       <c r="M46">
-        <v>102.6</v>
+        <v>103.1</v>
       </c>
       <c r="N46">
-        <v>154.8229834370066</v>
+        <v>189.396808999235</v>
       </c>
       <c r="O46">
-        <v>84.85485167985846</v>
+        <v>83.93462716646539</v>
       </c>
       <c r="P46">
-        <v>100.6545952885911</v>
+        <v>98.60805481449569</v>
       </c>
       <c r="Q46">
-        <v>2326.248617219057</v>
+        <v>2310.813546589645</v>
       </c>
       <c r="R46">
-        <v>0.01431247594296764</v>
+        <v>0.003100988822564918</v>
       </c>
     </row>
     <row r="47" spans="1:18">
@@ -3018,49 +3018,49 @@
         <v>94.16</v>
       </c>
       <c r="D47">
-        <v>4713.106634407119</v>
+        <v>4972.280325302404</v>
       </c>
       <c r="E47">
-        <v>6464.27885573589</v>
+        <v>6639.63571568</v>
       </c>
       <c r="F47">
-        <v>9.732747127349256</v>
+        <v>3.021544019964498</v>
       </c>
       <c r="G47">
-        <v>168.81625</v>
+        <v>168.4225000000002</v>
       </c>
       <c r="H47">
-        <v>86.95033907924036</v>
+        <v>85.93713279570214</v>
       </c>
       <c r="I47">
-        <v>102.64455123431</v>
+        <v>100.563496205883</v>
       </c>
       <c r="J47">
-        <v>951.1827015625018</v>
+        <v>959.2957562500015</v>
       </c>
       <c r="K47">
-        <v>2681.657145127625</v>
+        <v>2661.687845514887</v>
       </c>
       <c r="L47">
-        <v>0.02850268942498137</v>
+        <v>0.02596664727728694</v>
       </c>
       <c r="M47">
-        <v>86.66</v>
+        <v>87.16</v>
       </c>
       <c r="N47">
-        <v>7.703630693403194</v>
+        <v>2.139600273802909</v>
       </c>
       <c r="O47">
-        <v>86.60344856634674</v>
+        <v>85.67512328489002</v>
       </c>
       <c r="P47">
-        <v>102.438888436947</v>
+        <v>100.3832394256195</v>
       </c>
       <c r="Q47">
-        <v>2670.958608096844</v>
+        <v>2653.572755941258</v>
       </c>
       <c r="R47">
-        <v>0.03170647382480175</v>
+        <v>0.01017431538422463</v>
       </c>
     </row>
     <row r="48" spans="1:18">
@@ -3074,49 +3074,49 @@
         <v>148.6</v>
       </c>
       <c r="D48">
-        <v>17490.60986348108</v>
+        <v>17986.6717509024</v>
       </c>
       <c r="E48">
-        <v>19652.65751446849</v>
+        <v>19929.3995428</v>
       </c>
       <c r="F48">
-        <v>310.2385362219957</v>
+        <v>381.5767044887225</v>
       </c>
       <c r="G48">
-        <v>172.2430555555555</v>
+        <v>171.8638888888891</v>
       </c>
       <c r="H48">
-        <v>88.74785513924773</v>
+        <v>87.71370068969291</v>
       </c>
       <c r="I48">
-        <v>104.479306318648</v>
+        <v>102.3763350869573</v>
       </c>
       <c r="J48">
-        <v>1174.299631558643</v>
+        <v>1184.315748456792</v>
       </c>
       <c r="K48">
-        <v>3041.21643034814</v>
+        <v>3018.569549568351</v>
       </c>
       <c r="L48">
-        <v>0.02538229265813277</v>
+        <v>0.02311378567480634</v>
       </c>
       <c r="M48">
-        <v>141.1</v>
+        <v>141.6</v>
       </c>
       <c r="N48">
-        <v>356.4550762283477</v>
+        <v>419.8717501737022</v>
       </c>
       <c r="O48">
-        <v>88.3511065199519</v>
+        <v>87.41472678942756</v>
       </c>
       <c r="P48">
-        <v>104.224120518186</v>
+        <v>102.1593166506303</v>
       </c>
       <c r="Q48">
-        <v>3027.62062662052</v>
+        <v>3008.280694983942</v>
       </c>
       <c r="R48">
-        <v>0.05637319833361964</v>
+        <v>0.02159186729954911</v>
       </c>
     </row>
     <row r="49" spans="1:18">
@@ -3130,49 +3130,49 @@
         <v>79.67</v>
       </c>
       <c r="D49">
-        <v>897.1264619989006</v>
+        <v>1012.155920102405</v>
       </c>
       <c r="E49">
-        <v>2386.281369971097</v>
+        <v>2534.653088660001</v>
       </c>
       <c r="F49">
-        <v>8.412661627687529</v>
+        <v>15.63416092416712</v>
       </c>
       <c r="G49">
-        <v>175.6698611111111</v>
+        <v>175.3052777777779</v>
       </c>
       <c r="H49">
-        <v>90.54444723219987</v>
+        <v>89.48938750156638</v>
       </c>
       <c r="I49">
-        <v>106.3149853700412</v>
+        <v>104.190055050149</v>
       </c>
       <c r="J49">
-        <v>1420.902554185958</v>
+        <v>1433.022055632719</v>
       </c>
       <c r="K49">
-        <v>3413.060362800104</v>
+        <v>3387.645622034994</v>
       </c>
       <c r="L49">
-        <v>0.02216676153098134</v>
+        <v>0.02017581361137463</v>
       </c>
       <c r="M49">
-        <v>72.17</v>
+        <v>72.67</v>
       </c>
       <c r="N49">
-        <v>7.201071838708973</v>
+        <v>14.55411585738259</v>
       </c>
       <c r="O49">
-        <v>90.09783219198721</v>
+        <v>89.15344428711929</v>
       </c>
       <c r="P49">
-        <v>106.0102848809948</v>
+        <v>103.9362798824869</v>
       </c>
       <c r="Q49">
-        <v>3396.225270889155</v>
+        <v>3374.928398334539</v>
       </c>
       <c r="R49">
-        <v>0.08864314023799579</v>
+        <v>0.03759783952414253</v>
       </c>
     </row>
     <row r="50" spans="1:18">
@@ -3186,49 +3186,49 @@
         <v>87.45</v>
       </c>
       <c r="D50">
-        <v>363.3624902282149</v>
+        <v>437.8304316624038</v>
       </c>
       <c r="E50">
-        <v>1666.977969988356</v>
+        <v>1829.8386051</v>
       </c>
       <c r="F50">
-        <v>270.6660682444503</v>
+        <v>303.2195713035505</v>
       </c>
       <c r="G50">
-        <v>179.0966666666666</v>
+        <v>178.7466666666668</v>
       </c>
       <c r="H50">
-        <v>92.34012221041425</v>
+        <v>91.26420005139568</v>
       </c>
       <c r="I50">
-        <v>108.1515815361722</v>
+        <v>106.0046492753848</v>
       </c>
       <c r="J50">
-        <v>1690.991469444445</v>
+        <v>1705.414677777781</v>
       </c>
       <c r="K50">
-        <v>3797.179725495918</v>
+        <v>3768.907248122474</v>
       </c>
       <c r="L50">
-        <v>0.01891582018464042</v>
+        <v>0.01720733551884646</v>
       </c>
       <c r="M50">
-        <v>79.95</v>
+        <v>80.45</v>
       </c>
       <c r="N50">
-        <v>258.4713284063972</v>
+        <v>294.3808696946356</v>
       </c>
       <c r="O50">
-        <v>91.84363249643216</v>
+        <v>90.89128263615851</v>
       </c>
       <c r="P50">
-        <v>107.797374611394</v>
+        <v>105.7141222629961</v>
       </c>
       <c r="Q50">
-        <v>3776.763240974118</v>
+        <v>3753.50700193123</v>
       </c>
       <c r="R50">
-        <v>0.1288486329507085</v>
+        <v>0.05843855700935006</v>
       </c>
     </row>
     <row r="51" spans="1:18">
@@ -3242,49 +3242,49 @@
         <v>75.53</v>
       </c>
       <c r="D51">
-        <v>477.0759961531464</v>
+        <v>561.8984845424039</v>
       </c>
       <c r="E51">
-        <v>1649.731502609726</v>
+        <v>1790.39318094</v>
       </c>
       <c r="F51">
-        <v>9.354972499758937</v>
+        <v>16.34921011511307</v>
       </c>
       <c r="G51">
-        <v>182.5234722222222</v>
+        <v>182.1880555555557</v>
       </c>
       <c r="H51">
-        <v>94.13488717536677</v>
+        <v>93.03814539769937</v>
       </c>
       <c r="I51">
-        <v>109.989087715565</v>
+        <v>107.8201107041461</v>
       </c>
       <c r="J51">
-        <v>1984.566377334104</v>
+        <v>2001.49361489198</v>
       </c>
       <c r="K51">
-        <v>4193.565406473849</v>
+        <v>4162.345717588134</v>
       </c>
       <c r="L51">
-        <v>0.01569370480962582</v>
+        <v>0.014267029945998</v>
       </c>
       <c r="M51">
-        <v>68.03</v>
+        <v>68.53</v>
       </c>
       <c r="N51">
-        <v>7.420246514846055</v>
+        <v>14.57348963622036</v>
       </c>
       <c r="O51">
-        <v>93.58851459866682</v>
+        <v>92.62824893451673</v>
       </c>
       <c r="P51">
-        <v>109.5853825440035</v>
+        <v>107.4928366941863</v>
       </c>
       <c r="Q51">
-        <v>4169.225342917747</v>
+        <v>4144.007746846244</v>
       </c>
       <c r="R51">
-        <v>0.1773235752106406</v>
+        <v>0.0843622423280844</v>
       </c>
     </row>
     <row r="52" spans="1:18">
@@ -3298,49 +3298,49 @@
         <v>59.43</v>
       </c>
       <c r="D52">
-        <v>73.7525518021877</v>
+        <v>45.23372226240393</v>
       </c>
       <c r="E52">
-        <v>-510.3807149067122</v>
+        <v>-399.7025268599997</v>
       </c>
       <c r="F52">
-        <v>9.522508288254597</v>
+        <v>14.53766787545371</v>
       </c>
       <c r="G52">
-        <v>185.9502777777777</v>
+        <v>185.6294444444446</v>
       </c>
       <c r="H52">
-        <v>95.92874946632517</v>
+        <v>94.81123082595202</v>
       </c>
       <c r="I52">
-        <v>111.8274965689519</v>
+        <v>109.6364320509586</v>
       </c>
       <c r="J52">
-        <v>2301.627277854937</v>
+        <v>2321.258866975314</v>
       </c>
       <c r="K52">
-        <v>4602.2084025218</v>
+        <v>4567.952428288359</v>
       </c>
       <c r="L52">
-        <v>0.01256900308166617</v>
+        <v>0.01141749829159993</v>
       </c>
       <c r="M52">
-        <v>51.93</v>
+        <v>52.43</v>
       </c>
       <c r="N52">
-        <v>5.336227121489804</v>
+        <v>10.63400115884414</v>
       </c>
       <c r="O52">
-        <v>95.33248590400291</v>
+        <v>94.36435050839006</v>
       </c>
       <c r="P52">
-        <v>111.3743012735115</v>
+        <v>109.2724158498613</v>
       </c>
       <c r="Q52">
-        <v>4573.602492490622</v>
+        <v>4546.421982855067</v>
       </c>
       <c r="R52">
-        <v>0.2344031561876098</v>
+        <v>0.1156187845416222</v>
       </c>
     </row>
     <row r="53" spans="1:18">
@@ -3354,49 +3354,49 @@
         <v>26.37</v>
       </c>
       <c r="D53">
-        <v>4573.536995756161</v>
+        <v>4325.114406422404</v>
       </c>
       <c r="E53">
-        <v>-1783.348529633014</v>
+        <v>-1734.23892474</v>
       </c>
       <c r="F53">
-        <v>1.731399388447165</v>
+        <v>2.379357915013926</v>
       </c>
       <c r="G53">
-        <v>189.3770833333332</v>
+        <v>189.0708333333335</v>
       </c>
       <c r="H53">
-        <v>97.72171664881964</v>
+        <v>96.5834638369552</v>
       </c>
       <c r="I53">
-        <v>113.6668005308028</v>
+        <v>111.4536058150205</v>
       </c>
       <c r="J53">
-        <v>2642.174171006942</v>
+        <v>2664.710434027784</v>
       </c>
       <c r="K53">
-        <v>5023.099822659012</v>
+        <v>4985.718889483498</v>
       </c>
       <c r="L53">
-        <v>0.009614489726277218</v>
+        <v>0.008725110192818677</v>
       </c>
       <c r="M53">
-        <v>18.87</v>
+        <v>19.37</v>
       </c>
       <c r="N53">
-        <v>0.09992833842617636</v>
+        <v>0.1283444848149766</v>
       </c>
       <c r="O53">
-        <v>97.07555404605063</v>
+        <v>96.09959490050504</v>
       </c>
       <c r="P53">
-        <v>113.164123166308</v>
+        <v>111.0528521872947</v>
       </c>
       <c r="Q53">
-        <v>4989.885718704596</v>
+        <v>4960.741171759826</v>
       </c>
       <c r="R53">
-        <v>0.3004235837084251</v>
+        <v>0.152459509938293</v>
       </c>
     </row>
     <row r="54" spans="1:18">
@@ -3410,49 +3410,49 @@
         <v>70.22</v>
       </c>
       <c r="D54">
-        <v>628.6086645479404</v>
+        <v>725.4617956224033</v>
       </c>
       <c r="E54">
-        <v>1760.560714037533</v>
+        <v>1891.333427559999</v>
       </c>
       <c r="F54">
-        <v>15.70729328455128</v>
+        <v>8.708679932506529</v>
       </c>
       <c r="G54">
-        <v>192.8038888888888</v>
+        <v>192.5122222222224</v>
       </c>
       <c r="H54">
-        <v>99.51379650298836</v>
+        <v>98.35485213510761</v>
       </c>
       <c r="I54">
-        <v>115.5069918209794</v>
+        <v>113.2716242919332</v>
       </c>
       <c r="J54">
-        <v>3006.20705679012</v>
+        <v>3031.84831604939</v>
       </c>
       <c r="K54">
-        <v>5456.230891373845</v>
+        <v>5415.636724897109</v>
       </c>
       <c r="L54">
-        <v>0.006906958804104087</v>
+        <v>0.006259846132464981</v>
       </c>
       <c r="M54">
-        <v>62.72</v>
+        <v>63.22</v>
       </c>
       <c r="N54">
-        <v>18.07085661033572</v>
+        <v>9.874301907915003</v>
       </c>
       <c r="O54">
-        <v>98.81772687495939</v>
+        <v>97.83398985832346</v>
       </c>
       <c r="P54">
-        <v>114.9548403722434</v>
+        <v>112.8341379590247</v>
       </c>
       <c r="Q54">
-        <v>5418.066167079714</v>
+        <v>5386.956890465648</v>
       </c>
       <c r="R54">
-        <v>0.3757218162685214</v>
+        <v>0.1951369552452435</v>
       </c>
     </row>
     <row r="55" spans="1:18">
@@ -3466,49 +3466,49 @@
         <v>41.98</v>
       </c>
       <c r="D55">
-        <v>839.7204612232836</v>
+        <v>735.2558718224037</v>
       </c>
       <c r="E55">
-        <v>-1216.493526127945</v>
+        <v>-1138.31297196</v>
       </c>
       <c r="F55">
-        <v>12.65842831872979</v>
+        <v>9.022048855405597</v>
       </c>
       <c r="G55">
-        <v>196.2306944444443</v>
+        <v>195.9536111111113</v>
       </c>
       <c r="H55">
-        <v>101.3049970118354</v>
+        <v>100.1254036166118</v>
       </c>
       <c r="I55">
-        <v>117.3480624564777</v>
+        <v>115.0904795854941</v>
       </c>
       <c r="J55">
-        <v>3393.72593520447</v>
+        <v>3422.672513040132</v>
       </c>
       <c r="K55">
-        <v>5901.592951616833</v>
+        <v>5857.697675529301</v>
       </c>
       <c r="L55">
-        <v>0.004527053301765544</v>
+        <v>0.004095137819228067</v>
       </c>
       <c r="M55">
-        <v>34.48</v>
+        <v>34.98</v>
       </c>
       <c r="N55">
-        <v>21.43100467452064</v>
+        <v>14.24255723523684</v>
       </c>
       <c r="O55">
-        <v>100.55901244557</v>
+        <v>99.56754332218297</v>
       </c>
       <c r="P55">
-        <v>116.7464448364769</v>
+        <v>114.6162652247135</v>
       </c>
       <c r="Q55">
-        <v>5858.135102664207</v>
+        <v>5825.060833809708</v>
       </c>
       <c r="R55">
-        <v>0.4606352994558383</v>
+        <v>0.2439046438846063</v>
       </c>
     </row>
     <row r="56" spans="1:18">
@@ -3522,49 +3522,49 @@
         <v>25.38</v>
       </c>
       <c r="D56">
-        <v>3046.811541312599</v>
+        <v>2844.686440702404</v>
       </c>
       <c r="E56">
-        <v>-1400.923478349863</v>
+        <v>-1353.65757876</v>
       </c>
       <c r="F56">
-        <v>39.21032219130352</v>
+        <v>35.16249454112818</v>
       </c>
       <c r="G56">
-        <v>199.6574999999999</v>
+        <v>199.3950000000002</v>
       </c>
       <c r="H56">
-        <v>103.0953263494366</v>
+        <v>101.895126357654</v>
       </c>
       <c r="I56">
-        <v>119.1900042632218</v>
+        <v>116.910163619517</v>
       </c>
       <c r="J56">
-        <v>3804.730806249994</v>
+        <v>3837.18302500001</v>
       </c>
       <c r="K56">
-        <v>6359.177467549121</v>
+        <v>6311.893602224884</v>
       </c>
       <c r="L56">
-        <v>0.002559092602069602</v>
+        <v>0.002307706883123237</v>
       </c>
       <c r="M56">
-        <v>17.88</v>
+        <v>18.38</v>
       </c>
       <c r="N56">
-        <v>59.49829441789209</v>
+        <v>48.73318648128324</v>
       </c>
       <c r="O56">
-        <v>102.2994190055146</v>
+        <v>101.3002634134109</v>
       </c>
       <c r="P56">
-        <v>118.5389283113764</v>
+        <v>116.399225863034</v>
       </c>
       <c r="Q56">
-        <v>6310.083912807651</v>
+        <v>6275.044817143747</v>
       </c>
       <c r="R56">
-        <v>0.5555017073753973</v>
+        <v>0.2990168658112813</v>
       </c>
     </row>
     <row r="57" spans="1:18">
@@ -3578,49 +3578,49 @@
         <v>63.92</v>
       </c>
       <c r="D57">
-        <v>191.3261441895851</v>
+        <v>246.3141285824042</v>
       </c>
       <c r="E57">
-        <v>884.1458767484935</v>
+        <v>1003.18592016</v>
       </c>
       <c r="F57">
-        <v>18.54402053734615</v>
+        <v>11.48752352321349</v>
       </c>
       <c r="G57">
-        <v>203.0843055555554</v>
+        <v>202.8363888888891</v>
       </c>
       <c r="H57">
-        <v>104.8847928691297</v>
+        <v>103.664028602592</v>
       </c>
       <c r="I57">
-        <v>121.032808887874</v>
+        <v>118.7306681496441</v>
       </c>
       <c r="J57">
-        <v>4239.221669926689</v>
+        <v>4275.379851929023</v>
       </c>
       <c r="K57">
-        <v>6828.976027047316</v>
+        <v>6778.216487997989</v>
       </c>
       <c r="L57">
-        <v>0.001090898394286475</v>
+        <v>0.0009774024137662752</v>
       </c>
       <c r="M57">
-        <v>56.42</v>
+        <v>56.92</v>
       </c>
       <c r="N57">
-        <v>22.62908008240437</v>
+        <v>13.69752716650641</v>
       </c>
       <c r="O57">
-        <v>104.0389549833001</v>
+        <v>103.0321584224462</v>
       </c>
       <c r="P57">
-        <v>120.3322823684351</v>
+        <v>118.1830115835471</v>
       </c>
       <c r="Q57">
-        <v>6773.904109688368</v>
+        <v>6736.900778671682</v>
       </c>
       <c r="R57">
-        <v>0.6606586896215181</v>
+        <v>0.3607284614354236</v>
       </c>
     </row>
     <row r="58" spans="1:18">
@@ -3634,49 +3634,49 @@
         <v>70.08</v>
       </c>
       <c r="D58">
-        <v>179.347523107941</v>
+        <v>232.6966583424039</v>
       </c>
       <c r="E58">
-        <v>938.5162243199994</v>
+        <v>1069.02821184</v>
       </c>
       <c r="F58">
-        <v>4.355209873552187</v>
+        <v>9.000825040046241</v>
       </c>
       <c r="G58">
-        <v>206.511111111111</v>
+        <v>206.277777777778</v>
       </c>
       <c r="H58">
-        <v>106.67340509172</v>
+        <v>105.4321187521848</v>
       </c>
       <c r="I58">
-        <v>122.8764678096291</v>
+        <v>120.5519847751164</v>
       </c>
       <c r="J58">
-        <v>4697.198526234558</v>
+        <v>4737.262993827173</v>
       </c>
       <c r="K58">
-        <v>7310.980343966678</v>
+        <v>7256.658440115664</v>
       </c>
       <c r="L58">
-        <v>0.000213619569067935</v>
+        <v>0.0001870378521160602</v>
       </c>
       <c r="M58">
-        <v>62.58</v>
+        <v>63.08</v>
       </c>
       <c r="N58">
-        <v>2.656271926977766</v>
+        <v>7.202418843200252</v>
       </c>
       <c r="O58">
-        <v>105.777628976408</v>
+        <v>104.7632367970031</v>
       </c>
       <c r="P58">
-        <v>122.1264984101713</v>
+        <v>119.9676139385386</v>
       </c>
       <c r="Q58">
-        <v>7249.587332596976</v>
+        <v>7210.620781544848</v>
       </c>
       <c r="R58">
-        <v>0.776443624303445</v>
+        <v>0.4292946100964903</v>
       </c>
     </row>
     <row r="59" spans="1:18">
@@ -3690,49 +3690,49 @@
         <v>128.96</v>
       </c>
       <c r="D59">
-        <v>20059.64308563067</v>
+        <v>20590.6422573824</v>
       </c>
       <c r="E59">
-        <v>18264.87167123726</v>
+        <v>18505.03756608</v>
       </c>
       <c r="F59">
-        <v>48.96661714603526</v>
+        <v>24.97734081407044</v>
       </c>
       <c r="G59">
-        <v>209.9379166666665</v>
+        <v>209.7191666666669</v>
       </c>
       <c r="H59">
-        <v>108.4611716937363</v>
+        <v>107.1994053518964</v>
       </c>
       <c r="I59">
-        <v>124.7209723519581</v>
+        <v>122.3741049504699</v>
       </c>
       <c r="J59">
-        <v>5178.661375173599</v>
+        <v>5222.832450694458</v>
       </c>
       <c r="K59">
-        <v>7805.182260165365</v>
+        <v>7747.211691943769</v>
       </c>
       <c r="L59">
-        <v>2.15566245370525E-05</v>
+        <v>2.222772726870638E-05</v>
       </c>
       <c r="M59">
-        <v>121.46</v>
+        <v>121.96</v>
       </c>
       <c r="N59">
-        <v>31.30594521140086</v>
+        <v>15.52733713113648</v>
       </c>
       <c r="O59">
-        <v>107.5154497394449</v>
+        <v>106.4935071303096</v>
       </c>
       <c r="P59">
-        <v>123.9215676819785</v>
+        <v>121.7530243347805</v>
       </c>
       <c r="Q59">
-        <v>7737.125349978855</v>
+        <v>7696.197015718207</v>
       </c>
       <c r="R59">
-        <v>0.9031933775862989</v>
+        <v>0.5049706235187873</v>
       </c>
     </row>
     <row r="60" spans="1:18">
@@ -3746,49 +3746,49 @@
         <v>54.86</v>
       </c>
       <c r="D60">
-        <v>448.9284026460236</v>
+        <v>373.4788926624041</v>
       </c>
       <c r="E60">
-        <v>-1162.369872114795</v>
+        <v>-1060.20252572</v>
       </c>
       <c r="F60">
-        <v>26.97341593121452</v>
+        <v>33.80026165364934</v>
       </c>
       <c r="G60">
-        <v>213.3647222222221</v>
+        <v>213.1605555555558</v>
       </c>
       <c r="H60">
-        <v>110.2481014957671</v>
+        <v>108.9658970803031</v>
       </c>
       <c r="I60">
-        <v>126.5663136942727</v>
+        <v>124.1970199971283</v>
       </c>
       <c r="J60">
-        <v>5683.610216743814</v>
+        <v>5732.08822253088</v>
       </c>
       <c r="K60">
-        <v>8311.573747293232</v>
+        <v>8249.868604559246</v>
       </c>
       <c r="L60">
-        <v>0.0006119860896338537</v>
+        <v>0.0005712247089502928</v>
       </c>
       <c r="M60">
-        <v>47.36</v>
+        <v>47.86</v>
       </c>
       <c r="N60">
-        <v>17.9357179220887</v>
+        <v>26.28596950727089</v>
       </c>
       <c r="O60">
-        <v>109.2524261723731</v>
+        <v>108.2229781494501</v>
       </c>
       <c r="P60">
-        <v>125.7174812838945</v>
+        <v>123.5392340451883</v>
       </c>
       <c r="Q60">
-        <v>8236.51006123904</v>
+        <v>8193.621799571631</v>
       </c>
       <c r="R60">
-        <v>1.041244070166768</v>
+        <v>0.5880117446404332</v>
       </c>
     </row>
     <row r="61" spans="1:18">
@@ -3802,49 +3802,49 @@
         <v>46.12</v>
       </c>
       <c r="D61">
-        <v>433.386234010133</v>
+        <v>359.314847182404</v>
       </c>
       <c r="E61">
-        <v>-960.1229587665754</v>
+        <v>-874.2323642399999</v>
       </c>
       <c r="F61">
-        <v>14.00629542856391</v>
+        <v>9.729145426464875</v>
       </c>
       <c r="G61">
-        <v>216.7915277777776</v>
+        <v>216.6019444444447</v>
       </c>
       <c r="H61">
-        <v>112.0342034509046</v>
+        <v>110.7316027376345</v>
       </c>
       <c r="I61">
-        <v>128.4124828834805</v>
+        <v>126.020721114862</v>
       </c>
       <c r="J61">
-        <v>6212.0450509452</v>
+        <v>6265.030309336437</v>
       </c>
       <c r="K61">
-        <v>8830.146908349418</v>
+        <v>8764.62166813355</v>
       </c>
       <c r="L61">
-        <v>0.002084985448831207</v>
+        <v>0.001924757423883817</v>
       </c>
       <c r="M61">
-        <v>38.62</v>
+        <v>39.12</v>
       </c>
       <c r="N61">
-        <v>22.04930637691362</v>
+        <v>14.45527462485848</v>
       </c>
       <c r="O61">
-        <v>110.9885673088512</v>
+        <v>109.9516587038426</v>
       </c>
       <c r="P61">
-        <v>127.5142301822606</v>
+        <v>125.3262342203442</v>
       </c>
       <c r="Q61">
-        <v>8747.733498313815</v>
+        <v>8702.887581301076</v>
       </c>
       <c r="R61">
-        <v>1.190930851058731</v>
+        <v>0.6786729521701084</v>
       </c>
     </row>
     <row r="62" spans="1:18">
@@ -3858,49 +3858,49 @@
         <v>106.61</v>
       </c>
       <c r="D62">
-        <v>20375.298379723</v>
+        <v>20910.43192094241</v>
       </c>
       <c r="E62">
-        <v>15217.73201990233</v>
+        <v>15416.27487078</v>
       </c>
       <c r="F62">
-        <v>896.1576289666037</v>
+        <v>779.8952513276754</v>
       </c>
       <c r="G62">
-        <v>220.2183333333332</v>
+        <v>220.0433333333336</v>
       </c>
       <c r="H62">
-        <v>113.8194866333265</v>
+        <v>112.4965312344737</v>
       </c>
       <c r="I62">
-        <v>130.259470845404</v>
+        <v>127.8451993930878</v>
       </c>
       <c r="J62">
-        <v>6763.96587777776</v>
+        <v>6821.65871111113</v>
       </c>
       <c r="K62">
-        <v>9360.893979013534</v>
+        <v>9291.463503092647</v>
       </c>
       <c r="L62">
-        <v>0.004543259028679176</v>
+        <v>0.004175869460340174</v>
       </c>
       <c r="M62">
-        <v>99.11</v>
+        <v>99.61</v>
       </c>
       <c r="N62">
-        <v>813.2394148413639</v>
+        <v>721.3229120431415</v>
       </c>
       <c r="O62">
-        <v>112.7238823047127</v>
+        <v>111.6795577538748</v>
       </c>
       <c r="P62">
-        <v>129.3118052212432</v>
+        <v>127.1140158998604</v>
       </c>
       <c r="Q62">
-        <v>9270.78782701391</v>
+        <v>9223.986940085044</v>
       </c>
       <c r="R62">
-        <v>1.352587679019741</v>
+        <v>0.7772087711877002</v>
       </c>
     </row>
     <row r="63" spans="1:18">
@@ -3914,49 +3914,49 @@
         <v>139.19</v>
       </c>
       <c r="D63">
-        <v>24489.76778852438</v>
+        <v>25076.11536594239</v>
       </c>
       <c r="E63">
-        <v>21782.13114131137</v>
+        <v>22041.34865762</v>
       </c>
       <c r="F63">
-        <v>21.55842966324419</v>
+        <v>6.336829317251824</v>
       </c>
       <c r="G63">
-        <v>223.6451388888887</v>
+        <v>223.4847222222225</v>
       </c>
       <c r="H63">
-        <v>115.6039602270389</v>
+        <v>114.260691580642</v>
       </c>
       <c r="I63">
-        <v>132.1072683960369</v>
+        <v>129.6704458219847</v>
       </c>
       <c r="J63">
-        <v>7339.372697241492</v>
+        <v>7401.973427854959</v>
       </c>
       <c r="K63">
-        <v>9903.807328756</v>
+        <v>9830.386861059555</v>
       </c>
       <c r="L63">
-        <v>0.008091965281790981</v>
+        <v>0.007419759960310863</v>
       </c>
       <c r="M63">
-        <v>131.69</v>
+        <v>132.19</v>
       </c>
       <c r="N63">
-        <v>9.151738064705578</v>
+        <v>1.692265889806671</v>
       </c>
       <c r="O63">
-        <v>114.4583804266081</v>
+        <v>113.4066843597276</v>
       </c>
       <c r="P63">
-        <v>131.1101971341919</v>
+        <v>128.902570023556</v>
       </c>
       <c r="Q63">
-        <v>9805.665348144788</v>
+        <v>9756.91258703241</v>
       </c>
       <c r="R63">
-        <v>1.526547111908036</v>
+        <v>0.8838730900668454</v>
       </c>
     </row>
     <row r="64" spans="1:18">
@@ -3970,49 +3970,49 @@
         <v>77.29000000000001</v>
       </c>
       <c r="D64">
-        <v>194.660240848215</v>
+        <v>250.0951841024039</v>
       </c>
       <c r="E64">
-        <v>1078.355444773013</v>
+        <v>1222.29482142</v>
       </c>
       <c r="F64">
-        <v>81.00226122592399</v>
+        <v>98.36859649574232</v>
       </c>
       <c r="G64">
-        <v>227.0719444444443</v>
+        <v>226.9261111111114</v>
       </c>
       <c r="H64">
-        <v>117.3876335148061</v>
+        <v>116.024092874291</v>
       </c>
       <c r="I64">
-        <v>133.9558662526151</v>
+        <v>131.4964513034008</v>
       </c>
       <c r="J64">
-        <v>7938.265509336397</v>
+        <v>8005.974459567924</v>
       </c>
       <c r="K64">
-        <v>10458.87946173347</v>
+        <v>10381.38462558595</v>
       </c>
       <c r="L64">
-        <v>0.0128385458778908</v>
+        <v>0.01175362617295372</v>
       </c>
       <c r="M64">
-        <v>69.79000000000001</v>
+        <v>70.29000000000001</v>
       </c>
       <c r="N64">
-        <v>73.12198329262063</v>
+        <v>92.30766275162644</v>
       </c>
       <c r="O64">
-        <v>116.1920710408345</v>
+        <v>115.1330476704059</v>
       </c>
       <c r="P64">
-        <v>132.9093965548096</v>
+        <v>130.691887442426</v>
       </c>
       <c r="Q64">
-        <v>10352.35849841016</v>
+        <v>10301.65736591811</v>
       </c>
       <c r="R64">
-        <v>1.713140104213984</v>
+        <v>0.9989189839604071</v>
       </c>
     </row>
     <row r="65" spans="1:18">
@@ -4026,49 +4026,49 @@
         <v>12.62</v>
       </c>
       <c r="D65">
-        <v>7626.167460964381</v>
+        <v>7304.369125222404</v>
       </c>
       <c r="E65">
-        <v>-1102.078484033699</v>
+        <v>-1078.57589724</v>
       </c>
       <c r="F65">
-        <v>3.974376369907381</v>
+        <v>3.739675338103519</v>
       </c>
       <c r="G65">
-        <v>230.4987499999998</v>
+        <v>230.3675000000003</v>
       </c>
       <c r="H65">
-        <v>119.1705158672869</v>
+        <v>117.7867442912234</v>
       </c>
       <c r="I65">
-        <v>135.8052550444796</v>
+        <v>133.3232066615334</v>
       </c>
       <c r="J65">
-        <v>8560.644314062474</v>
+        <v>8633.661806250024</v>
       </c>
       <c r="K65">
-        <v>11026.10301747587</v>
+        <v>10944.44981267977</v>
       </c>
       <c r="L65">
-        <v>0.01889255698499265</v>
+        <v>0.01727650831659461</v>
       </c>
       <c r="M65">
-        <v>5.119999999999999</v>
+        <v>5.619999999999999</v>
       </c>
       <c r="N65">
-        <v>15.29737215370083</v>
+        <v>11.08296463040097</v>
       </c>
       <c r="O65">
-        <v>117.9249636023747</v>
+        <v>116.858656913</v>
       </c>
       <c r="P65">
-        <v>134.7093940281136</v>
+        <v>132.4819589293804</v>
       </c>
       <c r="Q65">
-        <v>10910.8598511052</v>
+        <v>10858.21425371369</v>
       </c>
       <c r="R65">
-        <v>1.912695812972148</v>
+        <v>1.122598545052705</v>
       </c>
     </row>
     <row r="66" spans="1:18">
@@ -4082,49 +4082,49 @@
         <v>61.58</v>
       </c>
       <c r="D66">
-        <v>374.5025904865713</v>
+        <v>450.0506825024041</v>
       </c>
       <c r="E66">
-        <v>1191.700434326849</v>
+        <v>1306.38262884</v>
       </c>
       <c r="F66">
-        <v>91.61862602266228</v>
+        <v>74.09827592278457</v>
       </c>
       <c r="G66">
-        <v>233.9255555555553</v>
+        <v>233.8088888888892</v>
       </c>
       <c r="H66">
-        <v>120.9526167324001</v>
+        <v>119.5486550744617</v>
       </c>
       <c r="I66">
-        <v>137.6554253237117</v>
+        <v>135.1507026533602</v>
       </c>
       <c r="J66">
-        <v>9206.509111419726</v>
+        <v>9285.035467901262</v>
       </c>
       <c r="K66">
-        <v>11605.47077137196</v>
+        <v>11519.57557113618</v>
       </c>
       <c r="L66">
-        <v>0.02636550309636471</v>
+        <v>0.02408913706999165</v>
       </c>
       <c r="M66">
-        <v>54.08</v>
+        <v>54.58</v>
       </c>
       <c r="N66">
-        <v>98.85221813457385</v>
+        <v>78.51021876812278</v>
       </c>
       <c r="O66">
-        <v>119.6570676441665</v>
+        <v>118.583521382195</v>
       </c>
       <c r="P66">
-        <v>136.510180021166</v>
+        <v>134.2727751897337</v>
       </c>
       <c r="Q66">
-        <v>11481.16211660645</v>
+        <v>11426.57636092012</v>
       </c>
       <c r="R66">
-        <v>2.125541412215482</v>
+        <v>1.255162719747894</v>
       </c>
     </row>
     <row r="67" spans="1:18">
@@ -4138,49 +4138,49 @@
         <v>20.29</v>
       </c>
       <c r="D67">
-        <v>5529.101841484655</v>
+        <v>5255.612309342405</v>
       </c>
       <c r="E67">
-        <v>-1508.722411651644</v>
+        <v>-1470.93576458</v>
       </c>
       <c r="F67">
-        <v>1.433799487726851</v>
+        <v>1.056271986650776</v>
       </c>
       <c r="G67">
-        <v>237.3523611111109</v>
+        <v>237.2502777777781</v>
       </c>
       <c r="H67">
-        <v>122.7339456249357</v>
+        <v>121.3098345240806</v>
       </c>
       <c r="I67">
-        <v>139.5063675755214</v>
+        <v>136.9789299788065</v>
       </c>
       <c r="J67">
-        <v>9875.859901408148</v>
+        <v>9960.095444521634</v>
       </c>
       <c r="K67">
-        <v>12196.97563496069</v>
+        <v>12106.75518267951</v>
       </c>
       <c r="L67">
-        <v>0.03537067373149987</v>
+        <v>0.03229378398647876</v>
       </c>
       <c r="M67">
-        <v>12.79</v>
+        <v>13.29</v>
       </c>
       <c r="N67">
-        <v>8.566997020613439</v>
+        <v>5.217136740284063</v>
       </c>
       <c r="O67">
-        <v>121.3883927666208</v>
+        <v>120.3076504300477</v>
       </c>
       <c r="P67">
-        <v>138.3117449335558</v>
+        <v>136.0643268714294</v>
       </c>
       <c r="Q67">
-        <v>12063.25814266584</v>
+        <v>12006.73693171056</v>
       </c>
       <c r="R67">
-        <v>2.352001916097539</v>
+        <v>1.396861152926691</v>
       </c>
     </row>
     <row r="68" spans="1:18">
@@ -4194,49 +4194,49 @@
         <v>24.7</v>
       </c>
       <c r="D68">
-        <v>4589.78209909753</v>
+        <v>4340.912550902405</v>
       </c>
       <c r="E68">
-        <v>-1673.373885549315</v>
+        <v>-1627.3743694</v>
       </c>
       <c r="F68">
-        <v>0.08443440909446139</v>
+        <v>0.004212345869516114</v>
       </c>
       <c r="G68">
-        <v>240.7791666666664</v>
+        <v>240.6916666666669</v>
       </c>
       <c r="H68">
-        <v>124.5145121164284</v>
+        <v>123.0702919873202</v>
       </c>
       <c r="I68">
-        <v>141.3580722283741</v>
+        <v>138.8078792906319</v>
       </c>
       <c r="J68">
-        <v>10568.69668402774</v>
+        <v>10658.84173611114</v>
       </c>
       <c r="K68">
-        <v>12800.61065603597</v>
+        <v>12705.98206192427</v>
       </c>
       <c r="L68">
-        <v>0.04602298331158477</v>
+        <v>0.04199411509794655</v>
       </c>
       <c r="M68">
-        <v>17.2</v>
+        <v>17.7</v>
       </c>
       <c r="N68">
-        <v>3.7027650165217</v>
+        <v>1.563632079879703</v>
       </c>
       <c r="O68">
-        <v>123.1189486274038</v>
+        <v>122.0310534560439</v>
       </c>
       <c r="P68">
-        <v>140.1140791076169</v>
+        <v>137.8566045749816</v>
       </c>
       <c r="Q68">
-        <v>12657.14091451637</v>
+        <v>12598.68934389108</v>
       </c>
       <c r="R68">
-        <v>2.592400010768319</v>
+        <v>1.547942039373849</v>
       </c>
     </row>
     <row r="69" spans="1:18">
@@ -4250,49 +4250,49 @@
         <v>60.69</v>
       </c>
       <c r="D69">
-        <v>311.8025126873934</v>
+        <v>249.5010425424041</v>
       </c>
       <c r="E69">
-        <v>-1071.659807448904</v>
+        <v>-958.6350853800001</v>
       </c>
       <c r="F69">
-        <v>83.77314853571174</v>
+        <v>96.09654787374522</v>
       </c>
       <c r="G69">
-        <v>244.205972222222</v>
+        <v>244.1330555555558</v>
       </c>
       <c r="H69">
-        <v>126.2943258253089</v>
+        <v>124.8300368489928</v>
       </c>
       <c r="I69">
-        <v>143.2105296638389</v>
+        <v>140.6375412040244</v>
       </c>
       <c r="J69">
-        <v>11285.01945927851</v>
+        <v>11381.27434266979</v>
       </c>
       <c r="K69">
-        <v>13416.36901857266</v>
+        <v>13317.24975616317</v>
       </c>
       <c r="L69">
-        <v>0.05843881448232428</v>
+        <v>0.05329504794891016</v>
       </c>
       <c r="M69">
-        <v>53.19</v>
+        <v>53.69</v>
       </c>
       <c r="N69">
-        <v>67.9869286813701</v>
+        <v>83.79355691894094</v>
       </c>
       <c r="O69">
-        <v>124.8487449314997</v>
+        <v>123.7537398974512</v>
       </c>
       <c r="P69">
-        <v>141.9171728383652</v>
+        <v>139.6495988631226</v>
       </c>
       <c r="Q69">
-        <v>13262.80355479743</v>
+        <v>13202.42710868758</v>
       </c>
       <c r="R69">
-        <v>2.847055895055858</v>
+        <v>1.70865198244392</v>
       </c>
     </row>
     <row r="70" spans="1:18">
@@ -4306,49 +4306,49 @@
         <v>49.9</v>
       </c>
       <c r="D70">
-        <v>17.20532817150281</v>
+        <v>5.223976502403987</v>
       </c>
       <c r="E70">
-        <v>-206.9817363931507</v>
+        <v>-114.0515397999999</v>
       </c>
       <c r="F70">
-        <v>77.39163144694125</v>
+        <v>64.52355020228318</v>
       </c>
       <c r="G70">
-        <v>247.6327777777775</v>
+        <v>247.5744444444447</v>
       </c>
       <c r="H70">
-        <v>128.0733964073445</v>
+        <v>126.5890785221932</v>
       </c>
       <c r="I70">
-        <v>145.0637302261487</v>
+        <v>142.4679063058892</v>
       </c>
       <c r="J70">
-        <v>12024.82822716045</v>
+        <v>12127.39326419757</v>
       </c>
       <c r="K70">
-        <v>14044.2440424818</v>
+        <v>13940.5519449907</v>
       </c>
       <c r="L70">
-        <v>0.07273586512957372</v>
+        <v>0.0663026122747362</v>
       </c>
       <c r="M70">
-        <v>42.4</v>
+        <v>42.9</v>
       </c>
       <c r="N70">
-        <v>90.41532969900841</v>
+        <v>72.8793988322512</v>
       </c>
       <c r="O70">
-        <v>126.5777914215653</v>
+        <v>125.4757192199782</v>
       </c>
       <c r="P70">
-        <v>143.7210163831438</v>
+        <v>141.443300270144</v>
       </c>
       <c r="Q70">
-        <v>13880.23932330789</v>
+        <v>13817.94387036722</v>
       </c>
       <c r="R70">
-        <v>3.116287129968308</v>
+        <v>1.879235860002964</v>
       </c>
     </row>
     <row r="71" spans="1:18">
@@ -4362,49 +4362,49 @@
         <v>17.56</v>
       </c>
       <c r="D71">
-        <v>6254.900764856982</v>
+        <v>5963.793604262403</v>
       </c>
       <c r="E71">
-        <v>-1388.784061143562</v>
+        <v>-1356.08157112</v>
       </c>
       <c r="F71">
-        <v>2.018138968297384</v>
+        <v>1.666757709440546</v>
       </c>
       <c r="G71">
-        <v>251.0595833333331</v>
+        <v>251.0158333333336</v>
       </c>
       <c r="H71">
-        <v>129.8517335463809</v>
+        <v>128.3474264393248</v>
       </c>
       <c r="I71">
-        <v>146.9176642314576</v>
+        <v>144.2989651638226</v>
       </c>
       <c r="J71">
-        <v>12788.12298767357</v>
+        <v>12897.19850069448</v>
       </c>
       <c r="K71">
-        <v>14684.22918320348</v>
+        <v>14575.88243977065</v>
       </c>
       <c r="L71">
-        <v>0.08903299930658022</v>
+        <v>0.08112381451229411</v>
       </c>
       <c r="M71">
-        <v>10.06</v>
+        <v>10.56</v>
       </c>
       <c r="N71">
-        <v>10.36021889435651</v>
+        <v>6.749864900395438</v>
       </c>
       <c r="O71">
-        <v>128.3060978685884</v>
+        <v>127.19700090875</v>
       </c>
       <c r="P71">
-        <v>145.5255999709648</v>
+        <v>143.2376993109206</v>
       </c>
       <c r="Q71">
-        <v>14509.44161659518</v>
+        <v>14445.23340570297</v>
       </c>
       <c r="R71">
-        <v>3.400408497002338</v>
+        <v>2.059936697657413</v>
       </c>
     </row>
     <row r="72" spans="1:18">
@@ -4418,49 +4418,49 @@
         <v>48.02</v>
       </c>
       <c r="D72">
-        <v>446.3894509753386</v>
+        <v>371.163420422404</v>
       </c>
       <c r="E72">
-        <v>-1014.563226885754</v>
+        <v>-925.1342080400001</v>
       </c>
       <c r="F72">
-        <v>2.816372058336018</v>
+        <v>1.118287401912193</v>
       </c>
       <c r="G72">
-        <v>254.4863888888886</v>
+        <v>254.4572222222225</v>
       </c>
       <c r="H72">
-        <v>131.6293469453946</v>
+        <v>130.1050900434481</v>
       </c>
       <c r="I72">
-        <v>148.7723219767892</v>
+        <v>146.1307083347644</v>
       </c>
       <c r="J72">
-        <v>13574.90374081785</v>
+        <v>13690.69005216053</v>
       </c>
       <c r="K72">
-        <v>15336.31803114533</v>
+        <v>15223.23518295599</v>
       </c>
       <c r="L72">
-        <v>0.1074501022647955</v>
+        <v>0.09786650630660242</v>
       </c>
       <c r="M72">
-        <v>40.52</v>
+        <v>41.02</v>
       </c>
       <c r="N72">
-        <v>6.947813407133877</v>
+        <v>3.040361308651526</v>
       </c>
       <c r="O72">
-        <v>130.0336740628599</v>
+        <v>128.9175944596079</v>
       </c>
       <c r="P72">
-        <v>147.3309138115375</v>
+        <v>145.0327864896111</v>
       </c>
       <c r="Q72">
-        <v>15150.40396738886</v>
+        <v>15084.28962328969</v>
       </c>
       <c r="R72">
-        <v>3.699731865211875</v>
+        <v>2.250995549251936</v>
       </c>
     </row>
     <row r="73" spans="1:18">
@@ -4474,49 +4474,49 @@
         <v>18.74</v>
       </c>
       <c r="D73">
-        <v>5853.46344301753</v>
+        <v>5571.965897942404</v>
       </c>
       <c r="E73">
-        <v>-1433.75861923863</v>
+        <v>-1398.85858148</v>
       </c>
       <c r="F73">
-        <v>2.5855303624884</v>
+        <v>2.121433074947147</v>
       </c>
       <c r="G73">
-        <v>257.9131944444442</v>
+        <v>257.8986111111114</v>
       </c>
       <c r="H73">
-        <v>133.4062463178628</v>
+        <v>131.8620787799574</v>
       </c>
       <c r="I73">
-        <v>150.6276937486664</v>
+        <v>147.9631263733202</v>
       </c>
       <c r="J73">
-        <v>14385.17048659331</v>
+        <v>14507.86791859572</v>
       </c>
       <c r="K73">
-        <v>16000.50431097525</v>
+        <v>15882.6042472698</v>
       </c>
       <c r="L73">
-        <v>0.1281079397551228</v>
+        <v>0.1166392571522363</v>
       </c>
       <c r="M73">
-        <v>11.24</v>
+        <v>11.74</v>
       </c>
       <c r="N73">
-        <v>11.34789879501029</v>
+        <v>7.485140098459544</v>
       </c>
       <c r="O73">
-        <v>131.7605298052656</v>
+        <v>130.6375093707405</v>
       </c>
       <c r="P73">
-        <v>149.1369481039758</v>
+        <v>146.8285523080268</v>
       </c>
       <c r="Q73">
-        <v>15803.12004388694</v>
+        <v>15735.10656272048</v>
       </c>
       <c r="R73">
-        <v>4.014566066962534</v>
+        <v>2.452651384592165</v>
       </c>
     </row>
     <row r="74" spans="1:18">
@@ -4530,49 +4530,49 @@
         <v>62.81</v>
       </c>
       <c r="D74">
-        <v>147.672790968763</v>
+        <v>196.403351302404</v>
       </c>
       <c r="E74">
-        <v>763.2714797023286</v>
+        <v>880.24433838</v>
       </c>
       <c r="F74">
-        <v>20.48387822754294</v>
+        <v>13.12754650706101</v>
       </c>
       <c r="G74">
-        <v>261.3399999999997</v>
+        <v>261.3400000000003</v>
       </c>
       <c r="H74">
-        <v>135.1824413794576</v>
+        <v>133.6184020885921</v>
       </c>
       <c r="I74">
-        <v>152.483769831417</v>
+        <v>149.7962098397506</v>
       </c>
       <c r="J74">
-        <v>15218.92322499995</v>
+        <v>15348.73210000003</v>
       </c>
       <c r="K74">
-        <v>16676.78188077676</v>
+        <v>16553.98383475569</v>
       </c>
       <c r="L74">
-        <v>0.1511280217409577</v>
+        <v>0.1375512312857222</v>
       </c>
       <c r="M74">
-        <v>55.31</v>
+        <v>55.81</v>
       </c>
       <c r="N74">
-        <v>25.00999276115364</v>
+        <v>15.62528666367672</v>
       </c>
       <c r="O74">
-        <v>133.4866748989063</v>
+        <v>132.3567551346499</v>
       </c>
       <c r="P74">
-        <v>150.9436930451793</v>
+        <v>148.6249872736658</v>
       </c>
       <c r="Q74">
-        <v>16467.58364890355</v>
+        <v>16397.67839363179</v>
       </c>
       <c r="R74">
-        <v>4.345216782270708</v>
+        <v>2.665140984329368</v>
       </c>
     </row>
   </sheetData>

</xml_diff>